<commit_message>
Daily injury update: Judge, Vientos, Gelof, Tchouameni, Jarvis, Mustafizur, Henry, Diggins
</commit_message>
<xml_diff>
--- a/injury_report.xlsx
+++ b/injury_report.xlsx
@@ -145,8 +145,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Injuries" displayName="Injuries" ref="A1:J45" headerRowCount="1">
-  <autoFilter ref="A1:J45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Injuries" displayName="Injuries" ref="A1:J53" headerRowCount="1">
+  <autoFilter ref="A1:J53"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Athlete"/>
     <tableColumn id="2" name="Organization"/>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -782,27 +782,27 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Connor Bedard</t>
+          <t>Aaron Judge</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Chicago Blackhawks (NHL)</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Hockey</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Surgery on left shoulder after an injury sustained during a practice session in Vancouver on July 2</t>
+          <t>Stress fracture in right rib; has not played since May 31 and went on the injured list June 5</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Expected to need approximately four months to recover; will miss training camp and at least the start of the 2026-27 season</t>
+          <t>Will have the rib reimaged during the All-Star break; no firm return date, GM Brian Cashman says he must be fully asymptomatic and show healing on imaging before resuming activity</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -812,49 +812,49 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Blackhawks will open the 2026-27 season, played under the NHL's expanded 84-game schedule, without their No. 1 center for at least the opening month</t>
+          <t>Yankees continue without their three-time AL MVP and captain in the middle of the lineup</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>NHL.com - Bedard to miss start of 2026-27 season for Blackhawks after shoulder surgery</t>
+          <t>ESPN - Yankees' Aaron Judge to have rib reimaged during All-Star break</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>https://www.nhl.com/news/connor-bedard-injury-status-update-july-8-2026</t>
+          <t>https://www.espn.com/mlb/story/_/id/49317023/yankees-aaron-judge-rib-reimaged-all-star-break</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Aliyah Boston</t>
+          <t>Mark Vientos</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Indiana Fever (WNBA)</t>
+          <t>New York Mets (MLB)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Lower right leg injury</t>
+          <t>Fractured bone in right hand after being hit by a pitch from Michael Wacha</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Listed out for the Fever's game vs. the LA Sparks; expected to be available for the following game vs. Phoenix</t>
+          <t>Headed to the injured list; broken bones of this type typically take around six weeks to heal, though the Mets have not given an official timeline and have not yet said whether surgery is needed</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -864,49 +864,49 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Fever forced to manage the availability of both Boston and Caitlin Clark during a back-to-back stretch; Boston, a voted-in 2026 All-Star starter, is having a career-best scoring season (17.1 ppg on 50.4% shooting) and was in danger of missing her first game since May 17</t>
+          <t>Mets lose a regular infielder/DH (.211, 11 HR, 35 RBI in 72 games) just ahead of the trade deadline</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Athlon Sports - Indiana Fever Announce Aliyah Boston Injury Update Before LA Sparks Game</t>
+          <t>amNewYork - Mark Vientos injury: Mets IF/DH headed to IL with hand fracture</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>https://athlonsports.com/wnba/indiana-fever/indiana-fever-announce-aliyah-boston-injury-update-la-sparks-game</t>
+          <t>https://www.amny.com/sports/mark-vientos-injury-mets-7-9-26/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Reece James</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Chelsea FC (Premier League) / England National Team (2026 FIFA World Cup)</t>
+          <t>Athletics (MLB)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury sustained in England's final group-stage match vs. Ghana on June 23; described by reporting as worse than first thought</t>
+          <t>Deep cut underneath the right kneecap after colliding with the left field fence on a sliding catch; came just missed the tendon per the team</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Touch-and-go for England's July 11 World Cup quarterfinal vs. Norway; has missed England's last three matches and was the sole absentee from the team's final group training session, requiring final medical clearance just to be considered for the bench</t>
+          <t>Left the July 9 game early; scheduled for an MRI on July 10 to confirm the extent of the injury</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -916,49 +916,49 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Compounds an England right-back crisis that worsened after Jarell Quansah's red card vs. Mexico, leaving manager Thomas Tuchel with very limited options at the position for the quarterfinal</t>
+          <t>Athletics risk losing an everyday infielder/outfielder who had an on-base streak of 27 straight games and a 13-game scoring streak snapped by the injury</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Sky Sports - England World Cup latest: Reece James in race to be fit for quarter-final clash with Norway to ease right-back crisis</t>
+          <t>ESPN - Athletics' Gelof to have MRI on knee after sliding into fence</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>https://www.skysports.com/football/news/11095/13561150/england-world-cup-latest-reece-james-in-race-to-be-fit-for-quarter-final-clash-with-norway-to-ease-right-back-crisis</t>
+          <t>https://www.espn.com/mlb/story/_/id/49319837/athletics-gelof-mri-knee-sliding-fence</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Marco Raya</t>
+          <t>Chinelle Henry</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Twins (MLB)</t>
+          <t>West Indies Women's National Cricket Team</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Right shoulder impingement</t>
+          <t>Exacerbation of a previous injury originally suffered fielding (stretchered off) in a T20 World Cup warm-up match in June</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Placed on 15-day IL July 8, retroactive to July 5</t>
+          <t>Ruled out of the Women's ODI tour of Ireland beginning July 10; no return timeline disclosed</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -968,49 +968,49 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Twins lose a pitching option for at least 15 days</t>
+          <t>West Indies lose their vice-captain and a key all-rounder; Realeanna Grimmond called up as her replacement for the Ireland series</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>MLB.com - Latest Twins injuries &amp; transactions</t>
+          <t>ESPNcricinfo - Realeanna Grimmond replaces injured Chinelle Henry in West Indies squad for Ireland Women's ODIs</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://www.mlb.com/news/twins-injuries-and-roster-moves</t>
+          <t>https://www.espncricinfo.com/story/slug-1545066</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Endy Rodriguez</t>
+          <t>Connor Bedard</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates (MLB)</t>
+          <t>Chicago Blackhawks (NHL)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Hockey</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Left glute strain</t>
+          <t>Surgery on left shoulder after an injury sustained during a practice session in Vancouver on July 2</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Placed on 10-day IL July 8, retroactive to July 6</t>
+          <t>Expected to need approximately four months to recover; will miss training camp and at least the start of the 2026-27 season</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pirates lose their starting catcher for at least 10 days</t>
+          <t>Blackhawks will open the 2026-27 season, played under the NHL's expanded 84-game schedule, without their No. 1 center for at least the opening month</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1030,24 +1030,24 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>MLB Trade Rumors - Pirates Place Endy Rodriguez On Injured List</t>
+          <t>NHL.com - Bedard to miss start of 2026-27 season for Blackhawks after shoulder surgery</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>https://www.mlbtraderumors.com/2026/07/pirates-to-place-endy-rodriguez-on-injured-list.html</t>
+          <t>https://www.nhl.com/news/connor-bedard-injury-status-update-july-8-2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Jalen Brunson</t>
+          <t>Aliyah Boston</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>New York Knicks (NBA)</t>
+          <t>Indiana Fever (WNBA)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Surgery to repair a left wrist injury that he played through during the Knicks' championship playoff run</t>
+          <t>Lower right leg injury</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>At least two months of rehab expected; targeting readiness for the start of the 2026-27 NBA season</t>
+          <t>Listed out for the Fever's game vs. the LA Sparks; expected to be available for the following game vs. Phoenix</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1072,34 +1072,34 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Reigning Finals MVP and starting point guard sidelined for part of the offseason program, though expected back for training camp</t>
+          <t>Fever forced to manage the availability of both Boston and Caitlin Clark during a back-to-back stretch; Boston, a voted-in 2026 All-Star starter, is having a career-best scoring season (17.1 ppg on 50.4% shooting) and was in danger of missing her first game since May 17</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports - Knicks superstar Jalen Brunson undergoes left wrist surgery, expected to be ready for 2026-27 NBA season</t>
+          <t>Athlon Sports - Indiana Fever Announce Aliyah Boston Injury Update Before LA Sparks Game</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/nba/breaking-news/article/knicks-superstar-jalen-brunson-undergoes-left-wrist-surgery-expected-to-be-ready-for-2026-27-nba-season-155927234.html</t>
+          <t>https://athlonsports.com/wnba/indiana-fever/indiana-fever-announce-aliyah-boston-injury-update-la-sparks-game</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Amadou Onana</t>
+          <t>Reece James</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Aston Villa (Premier League) / Belgium National Team (2026 FIFA World Cup)</t>
+          <t>Chelsea FC (Premier League) / England National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1109,12 +1109,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Torn anterior cruciate ligament (ACL), sustained in the 21st minute of Belgium's Round of 16 win over the United States after a challenge with Christian Pulisic</t>
+          <t>Hamstring injury sustained in England's final group-stage match vs. Ghana on June 23; described by reporting as worse than first thought</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of the World Cup; reported to be facing up to eight months out</t>
+          <t>Touch-and-go for England's July 11 World Cup quarterfinal vs. Norway; has missed England's last three matches and was the sole absentee from the team's final group training session, requiring final medical clearance just to be considered for the bench</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1124,49 +1124,49 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Belgium loses a key defensive midfielder ahead of their World Cup quarterfinal vs. Spain, and Aston Villa will be without him for a significant part of the 2026-27 season</t>
+          <t>Compounds an England right-back crisis that worsened after Jarell Quansah's red card vs. Mexico, leaving manager Thomas Tuchel with very limited options at the position for the quarterfinal</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Belgium's Amadou Onana out of World Cup after suffering ACL injury</t>
+          <t>Sky Sports - England World Cup latest: Reece James in race to be fit for quarter-final clash with Norway to ease right-back crisis</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49298508/belgium-amadou-onana-world-cup-suffering-acl-injury</t>
+          <t>https://www.skysports.com/football/news/11095/13561150/england-world-cup-latest-reece-james-in-race-to-be-fit-for-quarter-final-clash-with-norway-to-ease-right-back-crisis</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Giancarlo Stanton</t>
+          <t>Aurelien Tchouameni</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>New York Yankees (MLB)</t>
+          <t>Real Madrid (La Liga) / France National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Right calf strain (originally suffered running the bases on April 24 vs. the Astros); recent rehab setback after re-aggravating the calf during a running progression</t>
+          <t>Muscle tear involving the left adductor and upper thigh, a recurrence of the groin/thigh issue that previously sidelined him for France's group-stage match vs. Iraq</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>No firm timeline; has not resumed running since the setback, no target return date given</t>
+          <t>Missed France's Round of 16 win over Paraguay; returned to partial team training on July 8, with a decision on his availability for the July 11 quarterfinal vs. Morocco pending</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1176,153 +1176,153 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Yankees continue without their veteran slugger amid an offense that has struggled with injuries; manager Aaron Boone still expects him back at some point in 2026</t>
+          <t>France's vice-captain and starting defensive midfielder is a doubt for the quarterfinal, with Manu Kone deputizing in his absence</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Last Word on Sports - Stanton Injury Update: Slugger Yet To Resume Rehab On Calf</t>
+          <t>Sportskeeda - France handed huge injury boost as star man returns to training ahead of FIFA World Cup Q/F against Morocco</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://lastwordonsports.com/baseball/2026/07/07/nyy-stanton-injury-update/</t>
+          <t>https://www.sportskeeda.com/football/rumor-france-handed-huge-injury-boost-star-man-returns-training-ahead-fifa-world-cup-q-f-morocco-reports</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Matteo Berrettini</t>
+          <t>Mustafizur Rahman</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>ATP Tour</t>
+          <t>Bangladesh National Cricket Team</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Diagnosed with chronic hip pain, a recurrence of the left hip issue that forced his retirement from his Roland Garros quarterfinal in early June</t>
+          <t>Grade 1 muscle tear in the right hamstring and meniscal degeneration in the right knee, felt while bowling in the first ODI vs. Zimbabwe</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Withdrawing from the ATP tournaments in Gstaad and Kitzbuhel to rest on medical advice, with the goal of being ready for the US hard-court swing culminating in the US Open; no firm return date given</t>
+          <t>Ruled out for four weeks, covering the remainder of Bangladesh's tour of Zimbabwe (concluding July 19), including the T20I series; has returned home for rehab</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Forfeits ranking points and prize money from both the Gstaad and Kitzbuhel events</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Removes him from the draw at both tournaments immediately following his third-round Wimbledon loss to Grigor Dimitrov</t>
+          <t>Bangladesh lose a frontline pace bowler for the rest of the Zimbabwe tour</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Puntodebreak - Berrettini withdraws from competing in upcoming tournaments due to "chronic hip pain"</t>
+          <t>ESPNcricinfo - Zim vs Ban: Mustafizur Rahman ruled out for four weeks with hamstring and knee injuries</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>https://www.puntodebreak.com/en/2026/07/07/berrettini-withdraws-from-competing-in-upcoming-tournaments-due-to-chronic-hip-pain</t>
+          <t>https://www.espncricinfo.com/story/zim-vs-ban-mustafizur-rahman-ruled-out-for-four-weeks-with-hamstring-and-knee-injuries-1545065</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Emma Raducanu</t>
+          <t>Marco Raya</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>Minnesota Twins (MLB)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Stress fracture in lower right leg (ankle area); withdrew hours before her scheduled first-round match</t>
+          <t>Right shoulder impingement</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of Wimbledon 2026; still on crutches and wearing a protective boot several days after withdrawal, no return timeline given</t>
+          <t>Placed on 15-day IL July 8, retroactive to July 5</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Loses out on Wimbledon prize money and ranking points for the event</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Removes a top British draw from the tournament</t>
+          <t>Twins lose a pitching option for at least 15 days</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - Emma Raducanu setback deepens as British star remains on crutches after Wimbledon withdrawal</t>
+          <t>MLB.com - Latest Twins injuries &amp; transactions</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/tennis/articles/emma_raducanu_setback_deepens_as_british_star_remains_on_crutches_after_wimbledon_withdrawal/s1_17460_44037038</t>
+          <t>https://www.mlb.com/news/twins-injuries-and-roster-moves</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Jordan Henderson</t>
+          <t>Endy Rodriguez</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>England National Team (2026 FIFA World Cup)</t>
+          <t>Pittsburgh Pirates (MLB)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Wrist fracture sustained in a freak fall while celebrating England's Round of 16 win over Mexico; reportedly requires surgery</t>
+          <t>Left glute strain</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of the 2026 World Cup; exact surgery date and recovery length not yet specified</t>
+          <t>Placed on 10-day IL July 8, retroactive to July 6</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1332,49 +1332,49 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>England advance to the quarterfinals without an experienced veteran midfielder, compounding a growing injury list</t>
+          <t>Pirates lose their starting catcher for at least 10 days</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>ESPN - England's Henderson hospitalized with wrist injury during celebration</t>
+          <t>MLB Trade Rumors - Pirates Place Endy Rodriguez On Injured List</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49283507/jordan-henderson-taken-hospital-wrist-injury-falling-mexico-victory-celebrations-england-world-cup</t>
+          <t>https://www.mlbtraderumors.com/2026/07/pirates-to-place-endy-rodriguez-on-injured-list.html</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Santiago Gimenez</t>
+          <t>Jalen Brunson</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>AC Milan (Serie A) / Mexico National Team</t>
+          <t>New York Knicks (NBA)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Grade II right ankle sprain suffered in stoppage time of Mexico's Round of 16 loss to England; hospitalized, but avoided fracture and ligament damage</t>
+          <t>Surgery to repair a left wrist injury that he played through during the Knicks' championship playoff run</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Not yet specified by club or national team</t>
+          <t>At least two months of rehab expected; targeting readiness for the start of the 2026-27 NBA season</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1384,34 +1384,34 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Injury compounds Mexico's World Cup elimination and raises concern over his fitness for AC Milan's preseason</t>
+          <t>Reigning Finals MVP and starting point guard sidelined for part of the offseason program, though expected back for training camp</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>beIN Sports - Adding insult to injury! Santiago Gimenez suffers injury during Mexico's loss to England</t>
+          <t>Yahoo Sports - Knicks superstar Jalen Brunson undergoes left wrist surgery, expected to be ready for 2026-27 NBA season</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.beinsports.com/en-us/soccer/fifa-world-cup-2026/articles/adding-insult-to-injury-santiago-gimenez-suffers-injury-during-mexico-s-loss-to-england-2026-07-06</t>
+          <t>https://sports.yahoo.com/nba/breaking-news/article/knicks-superstar-jalen-brunson-undergoes-left-wrist-surgery-expected-to-be-ready-for-2026-27-nba-season-155927234.html</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Ismael Saibari</t>
+          <t>Amadou Onana</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Bayern Munich (Bundesliga, incoming) / Morocco National Team (2026 FIFA World Cup)</t>
+          <t>Aston Villa (Premier League) / Belgium National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1421,12 +1421,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury (minor muscle issue per medical tests; serious strain ruled out) suffered in the 22nd minute of Morocco's Round of 16 win over Canada</t>
+          <t>Torn anterior cruciate ligament (ACL), sustained in the 21st minute of Belgium's Round of 16 win over the United States after a challenge with Christian Pulisic</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Day-to-day pending fitness test; final decision on availability for the World Cup quarterfinal vs. France expected only hours before kickoff</t>
+          <t>Ruled out for the remainder of the World Cup; reported to be facing up to eight months out</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1436,49 +1436,49 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Morocco risks losing their top attacking threat (three group-stage goals) for the biggest match of their World Cup run</t>
+          <t>Belgium loses a key defensive midfielder ahead of their World Cup quarterfinal vs. Spain, and Aston Villa will be without him for a significant part of the 2026-27 season</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>The National - Ismael Saibari fitness concern for Morocco ahead of France World Cup quarter-final clash</t>
+          <t>ESPN - Belgium's Amadou Onana out of World Cup after suffering ACL injury</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>https://www.thenationalnews.com/sport/world-cup-2026/2026/07/06/ismael-saibari-fitness-concern-for-morocco-ahead-of-france-world-cup-quarter-final-clash/</t>
+          <t>https://www.espn.com/soccer/story/_/id/49298508/belgium-amadou-onana-world-cup-suffering-acl-injury</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>A'ja Wilson</t>
+          <t>Giancarlo Stanton</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Las Vegas Aces (WNBA)</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Foot injury sustained in a game against the Chicago Sky</t>
+          <t>Right calf strain (originally suffered running the bases on April 24 vs. the Astros); recent rehab setback after re-aggravating the calf during a running progression</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Missed 3 games; coach Becky Hammon said she could have played if it were a playoff game, suggesting an imminent return</t>
+          <t>No firm timeline; has not resumed running since the setback, no target return date given</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1488,86 +1488,86 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Aces without their All-Star forward/center for a short stretch, including a loss to Indiana</t>
+          <t>Yankees continue without their veteran slugger amid an offense that has struggled with injuries; manager Aaron Boone still expects him back at some point in 2026</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>Last Word on Sports - Stanton Injury Update: Slugger Yet To Resume Rehab On Calf</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://lastwordonsports.com/baseball/2026/07/07/nyy-stanton-injury-update/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Caitlin Clark</t>
+          <t>Matteo Berrettini</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Indiana Fever (WNBA)</t>
+          <t>ATP Tour</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Tennis</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Aggravated back injury</t>
+          <t>Diagnosed with chronic hip pain, a recurrence of the left hip issue that forced his retirement from his Roland Garros quarterfinal in early June</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Has resumed practicing; no confirmed timeline yet for a game return</t>
+          <t>Withdrawing from the ATP tournaments in Gstaad and Kitzbuhel to rest on medical advice, with the goal of being ready for the US hard-court swing culminating in the US Open; no firm return date given</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Forfeits ranking points and prize money from both the Gstaad and Kitzbuhel events</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Fever have played without their All-Star starting guard for an extended stretch</t>
+          <t>Removes him from the draw at both tournaments immediately following his third-round Wimbledon loss to Grigor Dimitrov</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>Puntodebreak - Berrettini withdraws from competing in upcoming tournaments due to "chronic hip pain"</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://www.puntodebreak.com/en/2026/07/07/berrettini-withdraws-from-competing-in-upcoming-tournaments-due-to-chronic-hip-pain</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Napheesa Collier</t>
+          <t>Skylar Diggins</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Lynx (WNBA)</t>
+          <t>Chicago Sky (WNBA)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1577,12 +1577,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Offseason surgery on both ankles</t>
+          <t>Right knee injury; Diggins has said a knee surgery from last October has contributed to ongoing strain</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Has yet to play in the 2026 season; recently resumed practicing</t>
+          <t>Ruled out for the July 7 game vs. Phoenix Mercury; no return timeline given</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1592,101 +1592,101 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Lynx have been without their All-Star forward for the entire season to date</t>
+          <t>Comes as Diggins was moved to the bench for the first time in a decade, ending a streak of 341 consecutive starts; Sky beat Phoenix 77-66 in her absence</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>Yahoo Sports - Sky's Skylar Diggins ruled out (knee) after being benched, Vandersloot starting</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://sports.yahoo.com/articles/skys-skylar-diggins-ruled-vs-010259203.html</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Byron Buxton</t>
+          <t>Emma Raducanu</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Twins (MLB)</t>
+          <t>WTA Tour</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Tennis</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Aggravated hip injury while being caught stealing in the 1st inning vs. Yankees</t>
+          <t>Stress fracture in lower right leg (ankle area); withdrew hours before her scheduled first-round match</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Day-to-day; had already missed 4 games earlier in the week with the same hip issue</t>
+          <t>Ruled out of Wimbledon 2026; still on crutches and wearing a protective boot several days after withdrawal, no return timeline given</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Loses out on Wimbledon prize money and ranking points for the event</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Twins lose their 2026 All-Star outfielder from the lineup for an undetermined stretch</t>
+          <t>Removes a top British draw from the tournament</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>Yardbarker - Emma Raducanu setback deepens as British star remains on crutches after Wimbledon withdrawal</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.yardbarker.com/tennis/articles/emma_raducanu_setback_deepens_as_british_star_remains_on_crutches_after_wimbledon_withdrawal/s1_17460_44037038</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Jazz Chisholm Jr.</t>
+          <t>Jordan Henderson</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>New York Yankees (MLB)</t>
+          <t>England National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Right toe discomfort, noticed jogging gingerly to first base after a fly out</t>
+          <t>Wrist fracture sustained in a freak fall while celebrating England's Round of 16 win over Mexico; reportedly requires surgery</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Being monitored day-to-day; no IL move confirmed yet</t>
+          <t>Ruled out for the remainder of the 2026 World Cup; exact surgery date and recovery length not yet specified</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1696,49 +1696,49 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Risk of losing Yankees' starting second baseman if it worsens</t>
+          <t>England advance to the quarterfinals without an experienced veteran midfielder, compounding a growing injury list</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>ESPN - England's Henderson hospitalized with wrist injury during celebration</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.espn.com/soccer/story/_/id/49283507/jordan-henderson-taken-hospital-wrist-injury-falling-mexico-victory-celebrations-england-world-cup</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Ranger Suarez</t>
+          <t>Santiago Gimenez</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies (MLB)</t>
+          <t>AC Milan (Serie A) / Mexico National Team</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Left adductor tightness, pulled early from start vs. Angels</t>
+          <t>Grade II right ankle sprain suffered in stoppage time of Mexico's Round of 16 loss to England; hospitalized, but avoided fracture and ligament damage</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Undetermined, pending further evaluation</t>
+          <t>Not yet specified by club or national team</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1748,49 +1748,49 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Phillies could lose their 2026 AL All-Star-caliber starter from the rotation</t>
+          <t>Injury compounds Mexico's World Cup elimination and raises concern over his fitness for AC Milan's preseason</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>beIN Sports - Adding insult to injury! Santiago Gimenez suffers injury during Mexico's loss to England</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.beinsports.com/en-us/soccer/fifa-world-cup-2026/articles/adding-insult-to-injury-santiago-gimenez-suffers-injury-during-mexico-s-loss-to-england-2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Brandon Woodruff</t>
+          <t>Ismael Saibari</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers (MLB)</t>
+          <t>Bayern Munich (Bundesliga, incoming) / Morocco National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Right shoulder inflammation</t>
+          <t>Hamstring injury (minor muscle issue per medical tests; serious strain ruled out) suffered in the 22nd minute of Morocco's Round of 16 win over Canada</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Placed on 15-day Injured List (minimum)</t>
+          <t>Day-to-day pending fitness test; final decision on availability for the World Cup quarterfinal vs. France expected only hours before kickoff</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1800,49 +1800,49 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Brewers rotation loses a top starter for at least two full turns</t>
+          <t>Morocco risks losing their top attacking threat (three group-stage goals) for the biggest match of their World Cup run</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Covers - MLB Injuries 2026</t>
+          <t>The National - Ismael Saibari fitness concern for Morocco ahead of France World Cup quarter-final clash</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.covers.com/sport/baseball/mlb/injuries</t>
+          <t>https://www.thenationalnews.com/sport/world-cup-2026/2026/07/06/ismael-saibari-fitness-concern-for-morocco-ahead-of-france-world-cup-quarter-final-clash/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Triston Casas</t>
+          <t>A'ja Wilson</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Boston Red Sox (MLB)</t>
+          <t>Las Vegas Aces (WNBA)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Torn right patellar tendon (out since May); recently shut down from hitting progression</t>
+          <t>Foot injury sustained in a game against the Chicago Sky</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Likely season-ending; setback in rehab timeline</t>
+          <t>Missed 3 games; coach Becky Hammon said she could have played if it were a playoff game, suggesting an imminent return</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1852,49 +1852,49 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Red Sox lose starting first baseman for the remainder of the 2026 season</t>
+          <t>Aces without their All-Star forward/center for a short stretch, including a loss to Indiana</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>James Maddison</t>
+          <t>Caitlin Clark</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Tottenham Hotspur (Premier League)</t>
+          <t>Indiana Fever (WNBA)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>ACL reconstruction rehab (returning from tear)</t>
+          <t>Aggravated back injury</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Ongoing; currently restricted to 20-25 minutes per match</t>
+          <t>Has resumed practicing; no confirmed timeline yet for a game return</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1904,101 +1904,101 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Spurs managing his minutes carefully, limiting his impact as a starter</t>
+          <t>Fever have played without their All-Star starting guard for an extended stretch</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Seamus Power</t>
+          <t>Napheesa Collier</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>PGA Tour</t>
+          <t>Minnesota Lynx (WNBA)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Golf</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Recurrence of long-standing back and hip issues he has dealt with since 2023</t>
+          <t>Offseason surgery on both ankles</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Withdrew after an opening-round 6-over 77 at the John Deere Classic on July 2; no return timeline given</t>
+          <t>Has yet to play in the 2026 season; recently resumed practicing</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Forfeits prize money and FedEx Cup points from the John Deere Classic</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Removes a two-time PGA Tour winner from the field partway through the event</t>
+          <t>Lynx have been without their All-Star forward for the entire season to date</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Golfmagic - Two-time PGA Tour winner forced out of John Deere Classic as injury problems strike again</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>https://www.golfmagic.com/tour/pga-tour/two-time-pga-tour-winner-forced-out-john-deere-classic-injury-problems-strike-again</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Nahikari Garcia</t>
+          <t>Byron Buxton</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Denver Summit FC (NWSL)</t>
+          <t>Minnesota Twins (MLB)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Season-ending knee (ACL) injury</t>
+          <t>Aggravated hip injury while being caught stealing in the 1st inning vs. Yankees</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Out for the remainder of the 2026 NWSL season</t>
+          <t>Day-to-day; had already missed 4 games earlier in the week with the same hip issue</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2008,49 +2008,49 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Denver Summit FC lose a starter for the rest of the season</t>
+          <t>Twins lose their 2026 All-Star outfielder from the lineup for an undetermined stretch</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Spotrac - 2026 NWSL Injured Tracker</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Brandon Ingram</t>
+          <t>Jazz Chisholm Jr.</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Toronto Raptors (NBA)</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Recovering from offseason surgery (lower body)</t>
+          <t>Right toe discomfort, noticed jogging gingerly to first base after a fly out</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Expected back for training camp, fall 2026</t>
+          <t>Being monitored day-to-day; no IL move confirmed yet</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2060,49 +2060,49 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Raptors plan around his absence through the offseason program</t>
+          <t>Risk of losing Yankees' starting second baseman if it worsens</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Brandon Ingram Injury Update Provided by Raptors After Surgery</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25426220-brandon-ingram-injury-update-provided-raptors-after-surgery-latest-timeline-2026-nba-season</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Josh Giddey</t>
+          <t>Ranger Suarez</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Chicago Bulls (NBA)</t>
+          <t>Philadelphia Phillies (MLB)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Arthroscopic surgery on right ankle</t>
+          <t>Left adductor tightness, pulled early from start vs. Angels</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>~3 months to resume basketball activities; targeting training camp</t>
+          <t>Undetermined, pending further evaluation</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2112,34 +2112,34 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Bulls lose a starting guard for the entire offseason program</t>
+          <t>Phillies could lose their 2026 AL All-Star-caliber starter from the rotation</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Josh Giddey Injury Update Provided by Bulls After Ankle Surgery</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25427505-josh-giddey-injury-update-provided-bulls-after-ankle-surgery-latest-timeline-2026-nba-season</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Corey Seager</t>
+          <t>Brandon Woodruff</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Texas Rangers (MLB)</t>
+          <t>Milwaukee Brewers (MLB)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2149,12 +2149,12 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Recurrence of lower back inflammation; his third injured list stint of the 2026 season (previously missed time with the same back issue and with a concussion)</t>
+          <t>Right shoulder inflammation</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Placed on the 10-day injured list</t>
+          <t>Placed on 15-day Injured List (minimum)</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2164,34 +2164,34 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Rangers lose their star shortstop again, continuing a season of infield instability; Josh Smith recalled from Triple-A as replacement</t>
+          <t>Brewers rotation loses a top starter for at least two full turns</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Rangers' Corey Seager back on IL with lower back inflammation</t>
+          <t>Covers - MLB Injuries 2026</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49238350/rangers-corey-seager-back-il-lower-back-inflammation</t>
+          <t>https://www.covers.com/sport/baseball/mlb/injuries</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Brent Rooker</t>
+          <t>Triston Casas</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Athletics (MLB)</t>
+          <t>Boston Red Sox (MLB)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2201,12 +2201,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Cartilage tear in left knee, discovered during an examination at Stanford; requires season-ending surgery</t>
+          <t>Torn right patellar tendon (out since May); recently shut down from hitting progression</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Season-ending; hadn't played since June 8 and had been on the injured list since June 9</t>
+          <t>Likely season-ending; setback in rehab timeline</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2216,49 +2216,49 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Athletics lose their two-time All-Star middle-of-the-order bat for the remainder of the 2026 season</t>
+          <t>Red Sox lose starting first baseman for the remainder of the 2026 season</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>ESPN - A's slugger Brent Rooker to have season-ending left knee surgery</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49244022/a-slugger-brent-rooker-season-ending-left-knee-surgery</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>JuJu Watkins</t>
+          <t>James Maddison</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>USC Trojans (NCAA Division I Women's Basketball)</t>
+          <t>Tottenham Hotspur (Premier League)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Recovering from a torn ACL that cost her the entire 2025-26 season</t>
+          <t>ACL reconstruction rehab (returning from tear)</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Returned to the court roughly 14 months after the injury</t>
+          <t>Ongoing; currently restricted to 20-25 minutes per match</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2268,86 +2268,86 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>USC gets back its star guard after a full season lost to the injury</t>
+          <t>Spurs managing his minutes carefully, limiting his impact as a starter</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Fox Sports - 2026-2027 College Basketball Offseason Buzz</t>
+          <t>Premier League club injury coverage</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>https://www.foxsports.com/stories/college-basketball/college-basketball-2026-2027-buzz-news-injuries-transfers</t>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Jaren Jackson Jr.</t>
+          <t>Seamus Power</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Memphis Grizzlies (NBA)</t>
+          <t>PGA Tour</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Golf</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Turf toe surgery (right foot)</t>
+          <t>Recurrence of long-standing back and hip issues he has dealt with since 2023</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Re-evaluation in approximately 12 weeks</t>
+          <t>Withdrew after an opening-round 6-over 77 at the John Deere Classic on July 2; no return timeline given</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Forfeits prize money and FedEx Cup points from the John Deere Classic</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Grizzlies lose their All-Star big man through the offseason and possibly into training camp</t>
+          <t>Removes a two-time PGA Tour winner from the field partway through the event</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>NBA.com - Grizzlies' Jaren Jackson Jr. has surgery to repair turf toe injury</t>
+          <t>Golfmagic - Two-time PGA Tour winner forced out of John Deere Classic as injury problems strike again</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.nba.com/news/memphis-grizzlies-jaren-jackson-jr-turf-toe-surgery</t>
+          <t>https://www.golfmagic.com/tour/pga-tour/two-time-pga-tour-winner-forced-out-john-deere-classic-injury-problems-strike-again</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Manuel Ugarte</t>
+          <t>Nahikari Garcia</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Manchester United (Premier League) / Uruguay National Team</t>
+          <t>Denver Summit FC (NWSL)</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2357,12 +2357,12 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Knee ligament injury suffered vs. Spain at the World Cup; possible cruciate ligament (ACL) damage</t>
+          <t>Season-ending knee (ACL) injury</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Potentially several months if ACL is confirmed</t>
+          <t>Out for the remainder of the 2026 NWSL season</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2372,49 +2372,49 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Would be a significant blow to Manchester United's midfield depth heading into 2026-27</t>
+          <t>Denver Summit FC lose a starter for the rest of the season</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>Spotrac - 2026 NWSL Injured Tracker</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Rodri</t>
+          <t>Brandon Ingram</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Manchester City (Premier League)</t>
+          <t>Toronto Raptors (NBA)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Undisclosed injury expected to require surgery after the World Cup</t>
+          <t>Recovering from offseason surgery (lower body)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Out for the opening weeks of the 2026-27 season</t>
+          <t>Expected back for training camp, fall 2026</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2424,34 +2424,34 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Manchester City to start the new season without their midfield anchor</t>
+          <t>Raptors plan around his absence through the offseason program</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>Bleacher Report - Brandon Ingram Injury Update Provided by Raptors After Surgery</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://bleacherreport.com/articles/25426220-brandon-ingram-injury-update-provided-raptors-after-surgery-latest-timeline-2026-nba-season</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Kelsey Plum</t>
+          <t>Josh Giddey</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks (WNBA)</t>
+          <t>Chicago Bulls (NBA)</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2461,12 +2461,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Lower leg injury</t>
+          <t>Arthroscopic surgery on right ankle</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for at least 4 weeks as of late June; All-Star Game (July 25) status still to be decided</t>
+          <t>~3 months to resume basketball activities; targeting training camp</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2476,49 +2476,49 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Sparks lose a starting guard through their All-Star break stretch</t>
+          <t>Bulls lose a starting guard for the entire offseason program</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Angel Reese, Kelsey Plum Headline 2026 WNBA All-Star Game Reserves</t>
+          <t>Bleacher Report - Josh Giddey Injury Update Provided by Bulls After Ankle Surgery</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25452286-angel-reese-kelsey-plum-headline-2026-wnba-all-star-game-reserves-full-roster-announced</t>
+          <t>https://bleacherreport.com/articles/25427505-josh-giddey-injury-update-provided-bulls-after-ankle-surgery-latest-timeline-2026-nba-season</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Bradley Beal</t>
+          <t>Corey Seager</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>LA Clippers (NBA)</t>
+          <t>Texas Rangers (MLB)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Hip fracture requiring season-ending surgery</t>
+          <t>Recurrence of lower back inflammation; his third injured list stint of the 2026 season (previously missed time with the same back issue and with a concussion)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Season-ending; recovery expected to extend into 2026-27 preseason</t>
+          <t>Placed on the 10-day injured list</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2528,101 +2528,101 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Clippers lose a veteran guard for the balance of the season and into next year's planning</t>
+          <t>Rangers lose their star shortstop again, continuing a season of infield instability; Josh Smith recalled from Triple-A as replacement</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>NBA.com - Clippers' Bradley Beal (hip) to undergo season-ending surgery</t>
+          <t>ESPN - Rangers' Corey Seager back on IL with lower back inflammation</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.nba.com/news/clippers-bradley-beal-out-season-hip-fracture</t>
+          <t>https://www.espn.com/mlb/story/_/id/49238350/rangers-corey-seager-back-il-lower-back-inflammation</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Bejlek</t>
+          <t>Brent Rooker</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>Athletics (MLB)</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Elbow injury</t>
+          <t>Cartilage tear in left knee, discovered during an examination at Stanford; requires season-ending surgery</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Withdrew mid-tournament from Eastbourne</t>
+          <t>Season-ending; hadn't played since June 8 and had been on the injured list since June 9</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Forfeits Eastbourne prize money/points from the round of withdrawal</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Opponent Zeynep Sonmez advances by walkover</t>
+          <t>Athletics lose their two-time All-Star middle-of-the-order bat for the remainder of the 2026 season</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>RotoWire - Fantasy Tennis Injury News</t>
+          <t>ESPN - A's slugger Brent Rooker to have season-ending left knee surgery</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+          <t>https://www.espn.com/mlb/story/_/id/49244022/a-slugger-brent-rooker-season-ending-left-knee-surgery</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Matthijs de Ligt</t>
+          <t>JuJu Watkins</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Manchester United (Premier League)</t>
+          <t>USC Trojans (NCAA Division I Women's Basketball)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Surgery on a long-standing back injury</t>
+          <t>Recovering from a torn ACL that cost her the entire 2025-26 season</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Will miss the 2026 World Cup; club return timeline unconfirmed</t>
+          <t>Returned to the court roughly 14 months after the injury</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2632,86 +2632,86 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>United lose a starting center-back for an extended stretch</t>
+          <t>USC gets back its star guard after a full season lost to the injury</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>Fox Sports - 2026-2027 College Basketball Offseason Buzz</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.foxsports.com/stories/college-basketball/college-basketball-2026-2027-buzz-news-injuries-transfers</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Elina Svitolina</t>
+          <t>Jaren Jackson Jr.</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>Memphis Grizzlies (NBA)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Hip injury</t>
+          <t>Turf toe surgery (right foot)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Withdrew before her Bad Homburg quarterfinal</t>
+          <t>Re-evaluation in approximately 12 weeks</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Forfeits Bad Homburg quarterfinal prize money/points</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Opponent Xinyu Wang advances by walkover</t>
+          <t>Grizzlies lose their All-Star big man through the offseason and possibly into training camp</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>RotoWire - Fantasy Tennis Injury News</t>
+          <t>NBA.com - Grizzlies' Jaren Jackson Jr. has surgery to repair turf toe injury</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+          <t>https://www.nba.com/news/memphis-grizzlies-jaren-jackson-jr-turf-toe-surgery</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Chris Richards</t>
+          <t>Manuel Ugarte</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Crystal Palace (Premier League) / USMNT</t>
+          <t>Manchester United (Premier League) / Uruguay National Team</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2721,12 +2721,12 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Torn ankle ligaments (two ligaments) suffered vs. Brentford</t>
+          <t>Knee ligament injury suffered vs. Spain at the World Cup; possible cruciate ligament (ACL) damage</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Expected to recover in time for the 2026 World Cup</t>
+          <t>Potentially several months if ACL is confirmed</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2736,12 +2736,12 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Crystal Palace lose a starting center-back for a multi-week stretch</t>
+          <t>Would be a significant blow to Manchester United's midfield depth heading into 2026-27</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -2758,50 +2758,466 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
+          <t>Rodri</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Manchester City (Premier League)</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Soccer</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Undisclosed injury expected to require surgery after the World Cup</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Out for the opening weeks of the 2026-27 season</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Manchester City to start the new season without their midfield anchor</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Premier League club injury coverage</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Kelsey Plum</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks (WNBA)</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Basketball</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Lower leg injury</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Ruled out for at least 4 weeks as of late June; All-Star Game (July 25) status still to be decided</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Sparks lose a starting guard through their All-Star break stretch</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Bleacher Report - Angel Reese, Kelsey Plum Headline 2026 WNBA All-Star Game Reserves</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>https://bleacherreport.com/articles/25452286-angel-reese-kelsey-plum-headline-2026-wnba-all-star-game-reserves-full-roster-announced</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Seth Jarvis</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Carolina Hurricanes (NHL)</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Hockey</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Shoulder surgery, the same shoulder that had a torn labrum and rotator cuff during the 2023-24 season</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Expected recovery of approximately 4-6 months, meaning the earliest return would be late October</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Hurricanes will be without a top-six forward for the start of the 2026-27 season</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>NHL.com - Jarvis expected to miss start of next season for Hurricanes after shoulder surgery</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nhl.com/news/seth-jarvis-to-miss-beginning-of-2026-2027-season-for-hurricanes-after-shoulder-surgery</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Bradley Beal</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>LA Clippers (NBA)</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Basketball</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Hip fracture requiring season-ending surgery</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Season-ending; recovery expected to extend into 2026-27 preseason</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Clippers lose a veteran guard for the balance of the season and into next year's planning</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>NBA.com - Clippers' Bradley Beal (hip) to undergo season-ending surgery</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nba.com/news/clippers-bradley-beal-out-season-hip-fracture</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Bejlek</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>WTA Tour</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Elbow injury</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Withdrew mid-tournament from Eastbourne</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Forfeits Eastbourne prize money/points from the round of withdrawal</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Opponent Zeynep Sonmez advances by walkover</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>RotoWire - Fantasy Tennis Injury News</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Matthijs de Ligt</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Manchester United (Premier League)</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Soccer</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Surgery on a long-standing back injury</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Will miss the 2026 World Cup; club return timeline unconfirmed</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>United lose a starting center-back for an extended stretch</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Premier League club injury coverage</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Elina Svitolina</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>WTA Tour</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Hip injury</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Withdrew before her Bad Homburg quarterfinal</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Forfeits Bad Homburg quarterfinal prize money/points</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Opponent Xinyu Wang advances by walkover</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>RotoWire - Fantasy Tennis Injury News</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Chris Richards</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Crystal Palace (Premier League) / USMNT</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Soccer</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Torn ankle ligaments (two ligaments) suffered vs. Brentford</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Expected to recover in time for the 2026 World Cup</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Crystal Palace lose a starting center-back for a multi-week stretch</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Premier League club injury coverage</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
           <t>Chloe Ricketts</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>Boston Legacy FC (NWSL)</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Soccer</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Ankle injury</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>Placed on the 45-day short-term injury list</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>Not disclosed in available reporting</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>Boston Legacy FC without a rostered defender for at least 45 days</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr">
         <is>
           <t>Washington Spirit / NWSL transactions coverage</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="J53" s="2" t="inlineStr">
         <is>
           <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
         </is>
@@ -2853,10 +3269,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId45"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId53"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Daily injury update: Tour de France crashes (Træen, Molenaar, de Kleijn) and Murray-Boyles thumb sprain
</commit_message>
<xml_diff>
--- a/injury_report.xlsx
+++ b/injury_report.xlsx
@@ -145,8 +145,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Injuries" displayName="Injuries" ref="A1:J53" headerRowCount="1">
-  <autoFilter ref="A1:J53"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Injuries" displayName="Injuries" ref="A1:J57" headerRowCount="1">
+  <autoFilter ref="A1:J57"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Athlete"/>
     <tableColumn id="2" name="Organization"/>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -522,27 +522,27 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gout Gout</t>
+          <t>Collin Murray-Boyles</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Athletics Australia (Track &amp; Field)</t>
+          <t>Toronto Raptors (NBA) — Las Vegas Summer League</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Athletics (Track &amp; Field)</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Grade-three left hamstring tear suffered in training in Brisbane</t>
+          <t>Sprained thumb/finger, diagnosed after exiting a Summer League game against the Lakers</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of the 2026 season, including the World Athletics U20 Championships (Aug. 5-9, Eugene, Oregon); targeting a return in 2027</t>
+          <t>Ruled out of the Raptors' Summer League opener vs. Boston; next possible return targeted for the Houston game; full recovery timeline not specified in available reporting</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -552,49 +552,49 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Removes the U20 200m world record holder from an anticipated showdown with American Tate Taylor at the World U20 Championships</t>
+          <t>Raptors lose their 2025 first-round pick (9th overall) for early Summer League reps as a point-forward, part of his developmental push</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Olympics.com - Gout Gout to miss World U20 Championships and rest of the season with hamstring injury</t>
+          <t>Raptors Republic - Collin Murray-Boyles, Alijah Martin to miss Raptors' Summer League opener</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>https://www.olympics.com/en/news/gout-gout-injury-hamstring-world-athletics-under-20-championships</t>
+          <t>https://raptorsrepublic.com/2026/07/10/collin-murray-boyles-alijah-martin-to-miss-raptors-summer-league-opener/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Harshit Rana</t>
+          <t>Gout Gout</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>India National Cricket Team</t>
+          <t>Athletics Australia (Track &amp; Field)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Athletics (Track &amp; Field)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury sustained during the third T20I vs. England at Trent Bridge</t>
+          <t>Grade-three left hamstring tear suffered in training in Brisbane</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
+          <t>Ruled out for the remainder of the 2026 season, including the World Athletics U20 Championships (Aug. 5-9, Eugene, Oregon); targeting a return in 2027</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Deepens India's bowling injury crisis on the England tour, with Rana joining Varun Chakaravarthy, Hardik Pandya, and Nitish Kumar Reddy on the unavailable list</t>
+          <t>Removes the U20 200m world record holder from an anticipated showdown with American Tate Taylor at the World U20 Championships</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -614,19 +614,19 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
+          <t>Olympics.com - Gout Gout to miss World U20 Championships and rest of the season with hamstring injury</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
+          <t>https://www.olympics.com/en/news/gout-gout-injury-hamstring-world-athletics-under-20-championships</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Varun Chakaravarthy</t>
+          <t>Harshit Rana</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>India's frontline wrist-spinner is unavailable as the team's injury list grows on the England tour</t>
+          <t>Deepens India's bowling injury crisis on the England tour, with Rana joining Varun Chakaravarthy, Hardik Pandya, and Nitish Kumar Reddy on the unavailable list</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -678,12 +678,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Litton Das</t>
+          <t>Varun Chakaravarthy</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh national cricket team</t>
+          <t>India National Cricket Team</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -693,12 +693,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Left calf injury; failed a fitness test ahead of the second ODI</t>
+          <t>Hamstring injury sustained during the third T20I vs. England at Trent Bridge</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the remainder of the ODI series vs. Zimbabwe; continuing rehab in Dhaka</t>
+          <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh loses their starting wicketkeeper-batter for the series; Parvez Hossain Emon named as replacement for the 2nd and 3rd ODIs</t>
+          <t>India's frontline wrist-spinner is unavailable as the team's injury list grows on the England tour</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -718,24 +718,24 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>The Nation - Injured Litton Das to miss rest of Zimbabwe ODI series</t>
+          <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>https://www.nation.com.pk/09-Jul-2026/injured-litton-das-miss-rest-zimbabwe-odi-series</t>
+          <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Ravichandran Ashwin</t>
+          <t>Litton Das</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>San Francisco Unicorns (Major League Cricket)</t>
+          <t>Bangladesh national cricket team</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -745,12 +745,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Right knee injury</t>
+          <t>Left calf injury; failed a fitness test ahead of the second ODI</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of MLC 2026; replaced by Peter Siddle</t>
+          <t>Ruled out of the remainder of the ODI series vs. Zimbabwe; continuing rehab in Dhaka</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Unicorns lose the veteran spinner after just one appearance this MLC season</t>
+          <t>Bangladesh loses their starting wicketkeeper-batter for the series; Parvez Hossain Emon named as replacement for the 2nd and 3rd ODIs</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -770,39 +770,39 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>India TV News - Why is Ravichandran Ashwin ruled out of ongoing MLC 2026? San Francisco Unicorns announce replacement</t>
+          <t>The Nation - Injured Litton Das to miss rest of Zimbabwe ODI series</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>https://www.indiatvnews.com/sports/cricket/why-is-ravichandran-ashwin-ruled-out-of-ongoing-mlc-2026-san-francisco-unicorns-announce-replacement-2026-07-09-1047737</t>
+          <t>https://www.nation.com.pk/09-Jul-2026/injured-litton-das-miss-rest-zimbabwe-odi-series</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Aaron Judge</t>
+          <t>Ravichandran Ashwin</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>New York Yankees (MLB)</t>
+          <t>San Francisco Unicorns (Major League Cricket)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Stress fracture in right rib; has not played since May 31 and went on the injured list June 5</t>
+          <t>Right knee injury</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Will have the rib reimaged during the All-Star break; no firm return date, GM Brian Cashman says he must be fully asymptomatic and show healing on imaging before resuming activity</t>
+          <t>Ruled out for the remainder of MLC 2026; replaced by Peter Siddle</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Yankees continue without their three-time AL MVP and captain in the middle of the lineup</t>
+          <t>Unicorns lose the veteran spinner after just one appearance this MLC season</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -822,24 +822,24 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Yankees' Aaron Judge to have rib reimaged during All-Star break</t>
+          <t>India TV News - Why is Ravichandran Ashwin ruled out of ongoing MLC 2026? San Francisco Unicorns announce replacement</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49317023/yankees-aaron-judge-rib-reimaged-all-star-break</t>
+          <t>https://www.indiatvnews.com/sports/cricket/why-is-ravichandran-ashwin-ruled-out-of-ongoing-mlc-2026-san-francisco-unicorns-announce-replacement-2026-07-09-1047737</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Mark Vientos</t>
+          <t>Aaron Judge</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>New York Mets (MLB)</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Fractured bone in right hand after being hit by a pitch from Michael Wacha</t>
+          <t>Stress fracture in right rib; has not played since May 31 and went on the injured list June 5</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Headed to the injured list; broken bones of this type typically take around six weeks to heal, though the Mets have not given an official timeline and have not yet said whether surgery is needed</t>
+          <t>Will have the rib reimaged during the All-Star break; no firm return date, GM Brian Cashman says he must be fully asymptomatic and show healing on imaging before resuming activity</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Mets lose a regular infielder/DH (.211, 11 HR, 35 RBI in 72 games) just ahead of the trade deadline</t>
+          <t>Yankees continue without their three-time AL MVP and captain in the middle of the lineup</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -874,24 +874,24 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>amNewYork - Mark Vientos injury: Mets IF/DH headed to IL with hand fracture</t>
+          <t>ESPN - Yankees' Aaron Judge to have rib reimaged during All-Star break</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>https://www.amny.com/sports/mark-vientos-injury-mets-7-9-26/</t>
+          <t>https://www.espn.com/mlb/story/_/id/49317023/yankees-aaron-judge-rib-reimaged-all-star-break</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Mark Vientos</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Athletics (MLB)</t>
+          <t>New York Mets (MLB)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -901,12 +901,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Deep cut underneath the right kneecap after colliding with the left field fence on a sliding catch; came just missed the tendon per the team</t>
+          <t>Fractured bone in right hand after being hit by a pitch from Michael Wacha</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Left the July 9 game early; scheduled for an MRI on July 10 to confirm the extent of the injury</t>
+          <t>Headed to the injured list; broken bones of this type typically take around six weeks to heal, though the Mets have not given an official timeline and have not yet said whether surgery is needed</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Athletics risk losing an everyday infielder/outfielder who had an on-base streak of 27 straight games and a 13-game scoring streak snapped by the injury</t>
+          <t>Mets lose a regular infielder/DH (.211, 11 HR, 35 RBI in 72 games) just ahead of the trade deadline</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -926,39 +926,39 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Athletics' Gelof to have MRI on knee after sliding into fence</t>
+          <t>amNewYork - Mark Vientos injury: Mets IF/DH headed to IL with hand fracture</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49319837/athletics-gelof-mri-knee-sliding-fence</t>
+          <t>https://www.amny.com/sports/mark-vientos-injury-mets-7-9-26/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Chinelle Henry</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>West Indies Women's National Cricket Team</t>
+          <t>Athletics (MLB)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Exacerbation of a previous injury originally suffered fielding (stretchered off) in a T20 World Cup warm-up match in June</t>
+          <t>Deep cut underneath the right kneecap after colliding with the left field fence on a sliding catch; came just missed the tendon per the team</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the Women's ODI tour of Ireland beginning July 10; no return timeline disclosed</t>
+          <t>Left the July 9 game early; scheduled for an MRI on July 10 to confirm the extent of the injury</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>West Indies lose their vice-captain and a key all-rounder; Realeanna Grimmond called up as her replacement for the Ireland series</t>
+          <t>Athletics risk losing an everyday infielder/outfielder who had an on-base streak of 27 straight games and a 13-game scoring streak snapped by the injury</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -978,39 +978,39 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>ESPNcricinfo - Realeanna Grimmond replaces injured Chinelle Henry in West Indies squad for Ireland Women's ODIs</t>
+          <t>ESPN - Athletics' Gelof to have MRI on knee after sliding into fence</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://www.espncricinfo.com/story/slug-1545066</t>
+          <t>https://www.espn.com/mlb/story/_/id/49319837/athletics-gelof-mri-knee-sliding-fence</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Connor Bedard</t>
+          <t>Chinelle Henry</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Chicago Blackhawks (NHL)</t>
+          <t>West Indies Women's National Cricket Team</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hockey</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Surgery on left shoulder after an injury sustained during a practice session in Vancouver on July 2</t>
+          <t>Exacerbation of a previous injury originally suffered fielding (stretchered off) in a T20 World Cup warm-up match in June</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Expected to need approximately four months to recover; will miss training camp and at least the start of the 2026-27 season</t>
+          <t>Ruled out of the Women's ODI tour of Ireland beginning July 10; no return timeline disclosed</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1020,49 +1020,49 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Blackhawks will open the 2026-27 season, played under the NHL's expanded 84-game schedule, without their No. 1 center for at least the opening month</t>
+          <t>West Indies lose their vice-captain and a key all-rounder; Realeanna Grimmond called up as her replacement for the Ireland series</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>NHL.com - Bedard to miss start of 2026-27 season for Blackhawks after shoulder surgery</t>
+          <t>ESPNcricinfo - Realeanna Grimmond replaces injured Chinelle Henry in West Indies squad for Ireland Women's ODIs</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>https://www.nhl.com/news/connor-bedard-injury-status-update-july-8-2026</t>
+          <t>https://www.espncricinfo.com/story/slug-1545066</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Aliyah Boston</t>
+          <t>Torstein Træen</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Indiana Fever (WNBA)</t>
+          <t>Uno-X Mobility (Tour de France) — Norway</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Cycling</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Lower right leg injury</t>
+          <t>Concussion and multiple fractured ribs sustained in a crash on the descent of the Col du Tourmalet during stage 6</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Listed out for the Fever's game vs. the LA Sparks; expected to be available for the following game vs. Phoenix</t>
+          <t>Withdrew from the Tour de France (did not start stage 7); no return timeline specified in available reporting</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1072,49 +1072,49 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Fever forced to manage the availability of both Boston and Caitlin Clark during a back-to-back stretch; Boston, a voted-in 2026 All-Star starter, is having a career-best scoring season (17.1 ppg on 50.4% shooting) and was in danger of missing her first game since May 17</t>
+          <t>Uno-X Mobility loses the rider who had been wearing the race's yellow jersey after stage 5; Tadej Pogačar reclaimed the overall race lead the same day</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Athlon Sports - Indiana Fever Announce Aliyah Boston Injury Update Before LA Sparks Game</t>
+          <t>Cyclingnews - 'Not the ending we wanted for this yellow adventure' - Torstein Træen out of Tour de France due to injuries from Tourmalet crash</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://athlonsports.com/wnba/indiana-fever/indiana-fever-announce-aliyah-boston-injury-update-la-sparks-game</t>
+          <t>https://www.cyclingnews.com/pro-cycling/teams-riders/not-the-ending-we-wanted-for-this-yellow-adventure-torstein-traeen-out-of-tour-de-france-due-to-injuries-from-tourmalet-crash/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Reece James</t>
+          <t>Alex Molenaar</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Chelsea FC (Premier League) / England National Team (2026 FIFA World Cup)</t>
+          <t>Caja Rural-Seguros RGA (Tour de France) — Netherlands</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Cycling</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury sustained in England's final group-stage match vs. Ghana on June 23; described by reporting as worse than first thought</t>
+          <t>Fracture of the first metacarpal in his right hand plus multiple contusions, sustained in a high-speed crash roughly 5km from the finish of stage 5; evaluated under concussion protocol after losing memory of the incident</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Touch-and-go for England's July 11 World Cup quarterfinal vs. Norway; has missed England's last three matches and was the sole absentee from the team's final group training session, requiring final medical clearance just to be considered for the bench</t>
+          <t>Abandoned the Tour de France; did not start stage 6; recovery timeline not specified in available reporting</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1124,49 +1124,49 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Compounds an England right-back crisis that worsened after Jarell Quansah's red card vs. Mexico, leaving manager Thomas Tuchel with very limited options at the position for the quarterfinal</t>
+          <t>Caja Rural-Seguros RGA loses a rider mid-Tour</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Sky Sports - England World Cup latest: Reece James in race to be fit for quarter-final clash with Norway to ease right-back crisis</t>
+          <t>Cycling Weekly - 'I don't remember the crash' – Caja Rural rider abandons Tour de France with fractured hand</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>https://www.skysports.com/football/news/11095/13561150/england-world-cup-latest-reece-james-in-race-to-be-fit-for-quarter-final-clash-with-norway-to-ease-right-back-crisis</t>
+          <t>https://www.cyclingweekly.com/racing/tour-de-france/i-dont-remember-the-crash-caja-rural-rider-abandons-tour-de-france-with-fractured-hand</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Aurelien Tchouameni</t>
+          <t>Arvid de Kleijn</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Real Madrid (La Liga) / France National Team (2026 FIFA World Cup)</t>
+          <t>Tudor Pro Cycling Team (Tour de France) — Netherlands</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Cycling</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Muscle tear involving the left adductor and upper thigh, a recurrence of the groin/thigh issue that previously sidelined him for France's group-stage match vs. Iraq</t>
+          <t>Muscle tears sustained during the stage 1 team time trial, which hampered him for the rest of the race</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Missed France's Round of 16 win over Paraguay; returned to partial team training on July 8, with a decision on his availability for the July 11 quarterfinal vs. Morocco pending</t>
+          <t>Abandoned the Tour de France on stage 6 after struggling since the opening days; recovery timeline not specified in available reporting</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1176,49 +1176,49 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>France's vice-captain and starting defensive midfielder is a doubt for the quarterfinal, with Manu Kone deputizing in his absence</t>
+          <t>Tudor Pro Cycling Team loses a rider mid-Tour after he battled to beat the time cut on multiple stages</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Sportskeeda - France handed huge injury boost as star man returns to training ahead of FIFA World Cup Q/F against Morocco</t>
+          <t>idlprocycling - Suffering ends: Arvid de Kleijn and Cian Uijtdebroeks abandon Tour de France</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.sportskeeda.com/football/rumor-france-handed-huge-injury-boost-star-man-returns-training-ahead-fifa-world-cup-q-f-morocco-reports</t>
+          <t>https://www.idlprocycling.com/cycling/suffering-ends-arvid-de-kleijn-and-cian-uijtdebroeks-abandon-tour-de-france</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Mustafizur Rahman</t>
+          <t>Connor Bedard</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh National Cricket Team</t>
+          <t>Chicago Blackhawks (NHL)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Hockey</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Grade 1 muscle tear in the right hamstring and meniscal degeneration in the right knee, felt while bowling in the first ODI vs. Zimbabwe</t>
+          <t>Surgery on left shoulder after an injury sustained during a practice session in Vancouver on July 2</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for four weeks, covering the remainder of Bangladesh's tour of Zimbabwe (concluding July 19), including the T20I series; has returned home for rehab</t>
+          <t>Expected to need approximately four months to recover; will miss training camp and at least the start of the 2026-27 season</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh lose a frontline pace bowler for the rest of the Zimbabwe tour</t>
+          <t>Blackhawks will open the 2026-27 season, played under the NHL's expanded 84-game schedule, without their No. 1 center for at least the opening month</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1238,39 +1238,39 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>ESPNcricinfo - Zim vs Ban: Mustafizur Rahman ruled out for four weeks with hamstring and knee injuries</t>
+          <t>NHL.com - Bedard to miss start of 2026-27 season for Blackhawks after shoulder surgery</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>https://www.espncricinfo.com/story/zim-vs-ban-mustafizur-rahman-ruled-out-for-four-weeks-with-hamstring-and-knee-injuries-1545065</t>
+          <t>https://www.nhl.com/news/connor-bedard-injury-status-update-july-8-2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Marco Raya</t>
+          <t>Aliyah Boston</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Twins (MLB)</t>
+          <t>Indiana Fever (WNBA)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Right shoulder impingement</t>
+          <t>Lower right leg injury</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Placed on 15-day IL July 8, retroactive to July 5</t>
+          <t>Listed out for the Fever's game vs. the LA Sparks; expected to be available for the following game vs. Phoenix</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Twins lose a pitching option for at least 15 days</t>
+          <t>Fever forced to manage the availability of both Boston and Caitlin Clark during a back-to-back stretch; Boston, a voted-in 2026 All-Star starter, is having a career-best scoring season (17.1 ppg on 50.4% shooting) and was in danger of missing her first game since May 17</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1290,39 +1290,39 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>MLB.com - Latest Twins injuries &amp; transactions</t>
+          <t>Athlon Sports - Indiana Fever Announce Aliyah Boston Injury Update Before LA Sparks Game</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.mlb.com/news/twins-injuries-and-roster-moves</t>
+          <t>https://athlonsports.com/wnba/indiana-fever/indiana-fever-announce-aliyah-boston-injury-update-la-sparks-game</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Endy Rodriguez</t>
+          <t>Reece James</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates (MLB)</t>
+          <t>Chelsea FC (Premier League) / England National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Left glute strain</t>
+          <t>Hamstring injury sustained in England's final group-stage match vs. Ghana on June 23; described by reporting as worse than first thought</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Placed on 10-day IL July 8, retroactive to July 6</t>
+          <t>Touch-and-go for England's July 11 World Cup quarterfinal vs. Norway; has missed England's last three matches and was the sole absentee from the team's final group training session, requiring final medical clearance just to be considered for the bench</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pirates lose their starting catcher for at least 10 days</t>
+          <t>Compounds an England right-back crisis that worsened after Jarell Quansah's red card vs. Mexico, leaving manager Thomas Tuchel with very limited options at the position for the quarterfinal</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1342,39 +1342,39 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>MLB Trade Rumors - Pirates Place Endy Rodriguez On Injured List</t>
+          <t>Sky Sports - England World Cup latest: Reece James in race to be fit for quarter-final clash with Norway to ease right-back crisis</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>https://www.mlbtraderumors.com/2026/07/pirates-to-place-endy-rodriguez-on-injured-list.html</t>
+          <t>https://www.skysports.com/football/news/11095/13561150/england-world-cup-latest-reece-james-in-race-to-be-fit-for-quarter-final-clash-with-norway-to-ease-right-back-crisis</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Jalen Brunson</t>
+          <t>Aurelien Tchouameni</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>New York Knicks (NBA)</t>
+          <t>Real Madrid (La Liga) / France National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Surgery to repair a left wrist injury that he played through during the Knicks' championship playoff run</t>
+          <t>Muscle tear involving the left adductor and upper thigh, a recurrence of the groin/thigh issue that previously sidelined him for France's group-stage match vs. Iraq</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>At least two months of rehab expected; targeting readiness for the start of the 2026-27 NBA season</t>
+          <t>Missed France's Round of 16 win over Paraguay; returned to partial team training on July 8, with a decision on his availability for the July 11 quarterfinal vs. Morocco pending</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1384,49 +1384,49 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Reigning Finals MVP and starting point guard sidelined for part of the offseason program, though expected back for training camp</t>
+          <t>France's vice-captain and starting defensive midfielder is a doubt for the quarterfinal, with Manu Kone deputizing in his absence</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports - Knicks superstar Jalen Brunson undergoes left wrist surgery, expected to be ready for 2026-27 NBA season</t>
+          <t>Sportskeeda - France handed huge injury boost as star man returns to training ahead of FIFA World Cup Q/F against Morocco</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/nba/breaking-news/article/knicks-superstar-jalen-brunson-undergoes-left-wrist-surgery-expected-to-be-ready-for-2026-27-nba-season-155927234.html</t>
+          <t>https://www.sportskeeda.com/football/rumor-france-handed-huge-injury-boost-star-man-returns-training-ahead-fifa-world-cup-q-f-morocco-reports</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Amadou Onana</t>
+          <t>Mustafizur Rahman</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Aston Villa (Premier League) / Belgium National Team (2026 FIFA World Cup)</t>
+          <t>Bangladesh National Cricket Team</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Torn anterior cruciate ligament (ACL), sustained in the 21st minute of Belgium's Round of 16 win over the United States after a challenge with Christian Pulisic</t>
+          <t>Grade 1 muscle tear in the right hamstring and meniscal degeneration in the right knee, felt while bowling in the first ODI vs. Zimbabwe</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of the World Cup; reported to be facing up to eight months out</t>
+          <t>Ruled out for four weeks, covering the remainder of Bangladesh's tour of Zimbabwe (concluding July 19), including the T20I series; has returned home for rehab</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1436,34 +1436,34 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Belgium loses a key defensive midfielder ahead of their World Cup quarterfinal vs. Spain, and Aston Villa will be without him for a significant part of the 2026-27 season</t>
+          <t>Bangladesh lose a frontline pace bowler for the rest of the Zimbabwe tour</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Belgium's Amadou Onana out of World Cup after suffering ACL injury</t>
+          <t>ESPNcricinfo - Zim vs Ban: Mustafizur Rahman ruled out for four weeks with hamstring and knee injuries</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49298508/belgium-amadou-onana-world-cup-suffering-acl-injury</t>
+          <t>https://www.espncricinfo.com/story/zim-vs-ban-mustafizur-rahman-ruled-out-for-four-weeks-with-hamstring-and-knee-injuries-1545065</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Giancarlo Stanton</t>
+          <t>Marco Raya</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>New York Yankees (MLB)</t>
+          <t>Minnesota Twins (MLB)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1473,12 +1473,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Right calf strain (originally suffered running the bases on April 24 vs. the Astros); recent rehab setback after re-aggravating the calf during a running progression</t>
+          <t>Right shoulder impingement</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>No firm timeline; has not resumed running since the setback, no target return date given</t>
+          <t>Placed on 15-day IL July 8, retroactive to July 5</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1488,86 +1488,86 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Yankees continue without their veteran slugger amid an offense that has struggled with injuries; manager Aaron Boone still expects him back at some point in 2026</t>
+          <t>Twins lose a pitching option for at least 15 days</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Last Word on Sports - Stanton Injury Update: Slugger Yet To Resume Rehab On Calf</t>
+          <t>MLB.com - Latest Twins injuries &amp; transactions</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://lastwordonsports.com/baseball/2026/07/07/nyy-stanton-injury-update/</t>
+          <t>https://www.mlb.com/news/twins-injuries-and-roster-moves</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Matteo Berrettini</t>
+          <t>Endy Rodriguez</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>ATP Tour</t>
+          <t>Pittsburgh Pirates (MLB)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Diagnosed with chronic hip pain, a recurrence of the left hip issue that forced his retirement from his Roland Garros quarterfinal in early June</t>
+          <t>Left glute strain</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Withdrawing from the ATP tournaments in Gstaad and Kitzbuhel to rest on medical advice, with the goal of being ready for the US hard-court swing culminating in the US Open; no firm return date given</t>
+          <t>Placed on 10-day IL July 8, retroactive to July 6</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Forfeits ranking points and prize money from both the Gstaad and Kitzbuhel events</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Removes him from the draw at both tournaments immediately following his third-round Wimbledon loss to Grigor Dimitrov</t>
+          <t>Pirates lose their starting catcher for at least 10 days</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Puntodebreak - Berrettini withdraws from competing in upcoming tournaments due to "chronic hip pain"</t>
+          <t>MLB Trade Rumors - Pirates Place Endy Rodriguez On Injured List</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://www.puntodebreak.com/en/2026/07/07/berrettini-withdraws-from-competing-in-upcoming-tournaments-due-to-chronic-hip-pain</t>
+          <t>https://www.mlbtraderumors.com/2026/07/pirates-to-place-endy-rodriguez-on-injured-list.html</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Skylar Diggins</t>
+          <t>Jalen Brunson</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Chicago Sky (WNBA)</t>
+          <t>New York Knicks (NBA)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1577,12 +1577,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Right knee injury; Diggins has said a knee surgery from last October has contributed to ongoing strain</t>
+          <t>Surgery to repair a left wrist injury that he played through during the Knicks' championship playoff run</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the July 7 game vs. Phoenix Mercury; no return timeline given</t>
+          <t>At least two months of rehab expected; targeting readiness for the start of the 2026-27 NBA season</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Comes as Diggins was moved to the bench for the first time in a decade, ending a streak of 341 consecutive starts; Sky beat Phoenix 77-66 in her absence</t>
+          <t>Reigning Finals MVP and starting point guard sidelined for part of the offseason program, though expected back for training camp</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1602,91 +1602,91 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports - Sky's Skylar Diggins ruled out (knee) after being benched, Vandersloot starting</t>
+          <t>Yahoo Sports - Knicks superstar Jalen Brunson undergoes left wrist surgery, expected to be ready for 2026-27 NBA season</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/articles/skys-skylar-diggins-ruled-vs-010259203.html</t>
+          <t>https://sports.yahoo.com/nba/breaking-news/article/knicks-superstar-jalen-brunson-undergoes-left-wrist-surgery-expected-to-be-ready-for-2026-27-nba-season-155927234.html</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Emma Raducanu</t>
+          <t>Amadou Onana</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>Aston Villa (Premier League) / Belgium National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Stress fracture in lower right leg (ankle area); withdrew hours before her scheduled first-round match</t>
+          <t>Torn anterior cruciate ligament (ACL), sustained in the 21st minute of Belgium's Round of 16 win over the United States after a challenge with Christian Pulisic</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of Wimbledon 2026; still on crutches and wearing a protective boot several days after withdrawal, no return timeline given</t>
+          <t>Ruled out for the remainder of the World Cup; reported to be facing up to eight months out</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Loses out on Wimbledon prize money and ranking points for the event</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Removes a top British draw from the tournament</t>
+          <t>Belgium loses a key defensive midfielder ahead of their World Cup quarterfinal vs. Spain, and Aston Villa will be without him for a significant part of the 2026-27 season</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - Emma Raducanu setback deepens as British star remains on crutches after Wimbledon withdrawal</t>
+          <t>ESPN - Belgium's Amadou Onana out of World Cup after suffering ACL injury</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/tennis/articles/emma_raducanu_setback_deepens_as_british_star_remains_on_crutches_after_wimbledon_withdrawal/s1_17460_44037038</t>
+          <t>https://www.espn.com/soccer/story/_/id/49298508/belgium-amadou-onana-world-cup-suffering-acl-injury</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Jordan Henderson</t>
+          <t>Giancarlo Stanton</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>England National Team (2026 FIFA World Cup)</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Wrist fracture sustained in a freak fall while celebrating England's Round of 16 win over Mexico; reportedly requires surgery</t>
+          <t>Right calf strain (originally suffered running the bases on April 24 vs. the Astros); recent rehab setback after re-aggravating the calf during a running progression</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of the 2026 World Cup; exact surgery date and recovery length not yet specified</t>
+          <t>No firm timeline; has not resumed running since the setback, no target return date given</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1696,101 +1696,101 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>England advance to the quarterfinals without an experienced veteran midfielder, compounding a growing injury list</t>
+          <t>Yankees continue without their veteran slugger amid an offense that has struggled with injuries; manager Aaron Boone still expects him back at some point in 2026</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>ESPN - England's Henderson hospitalized with wrist injury during celebration</t>
+          <t>Last Word on Sports - Stanton Injury Update: Slugger Yet To Resume Rehab On Calf</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49283507/jordan-henderson-taken-hospital-wrist-injury-falling-mexico-victory-celebrations-england-world-cup</t>
+          <t>https://lastwordonsports.com/baseball/2026/07/07/nyy-stanton-injury-update/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Santiago Gimenez</t>
+          <t>Matteo Berrettini</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>AC Milan (Serie A) / Mexico National Team</t>
+          <t>ATP Tour</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Tennis</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Grade II right ankle sprain suffered in stoppage time of Mexico's Round of 16 loss to England; hospitalized, but avoided fracture and ligament damage</t>
+          <t>Diagnosed with chronic hip pain, a recurrence of the left hip issue that forced his retirement from his Roland Garros quarterfinal in early June</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Not yet specified by club or national team</t>
+          <t>Withdrawing from the ATP tournaments in Gstaad and Kitzbuhel to rest on medical advice, with the goal of being ready for the US hard-court swing culminating in the US Open; no firm return date given</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Forfeits ranking points and prize money from both the Gstaad and Kitzbuhel events</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Injury compounds Mexico's World Cup elimination and raises concern over his fitness for AC Milan's preseason</t>
+          <t>Removes him from the draw at both tournaments immediately following his third-round Wimbledon loss to Grigor Dimitrov</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>beIN Sports - Adding insult to injury! Santiago Gimenez suffers injury during Mexico's loss to England</t>
+          <t>Puntodebreak - Berrettini withdraws from competing in upcoming tournaments due to "chronic hip pain"</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://www.beinsports.com/en-us/soccer/fifa-world-cup-2026/articles/adding-insult-to-injury-santiago-gimenez-suffers-injury-during-mexico-s-loss-to-england-2026-07-06</t>
+          <t>https://www.puntodebreak.com/en/2026/07/07/berrettini-withdraws-from-competing-in-upcoming-tournaments-due-to-chronic-hip-pain</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Ismael Saibari</t>
+          <t>Skylar Diggins</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Bayern Munich (Bundesliga, incoming) / Morocco National Team (2026 FIFA World Cup)</t>
+          <t>Chicago Sky (WNBA)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury (minor muscle issue per medical tests; serious strain ruled out) suffered in the 22nd minute of Morocco's Round of 16 win over Canada</t>
+          <t>Right knee injury; Diggins has said a knee surgery from last October has contributed to ongoing strain</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Day-to-day pending fitness test; final decision on availability for the World Cup quarterfinal vs. France expected only hours before kickoff</t>
+          <t>Ruled out for the July 7 game vs. Phoenix Mercury; no return timeline given</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1800,59 +1800,59 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Morocco risks losing their top attacking threat (three group-stage goals) for the biggest match of their World Cup run</t>
+          <t>Comes as Diggins was moved to the bench for the first time in a decade, ending a streak of 341 consecutive starts; Sky beat Phoenix 77-66 in her absence</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>The National - Ismael Saibari fitness concern for Morocco ahead of France World Cup quarter-final clash</t>
+          <t>Yahoo Sports - Sky's Skylar Diggins ruled out (knee) after being benched, Vandersloot starting</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.thenationalnews.com/sport/world-cup-2026/2026/07/06/ismael-saibari-fitness-concern-for-morocco-ahead-of-france-world-cup-quarter-final-clash/</t>
+          <t>https://sports.yahoo.com/articles/skys-skylar-diggins-ruled-vs-010259203.html</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>A'ja Wilson</t>
+          <t>Emma Raducanu</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Las Vegas Aces (WNBA)</t>
+          <t>WTA Tour</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Tennis</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Foot injury sustained in a game against the Chicago Sky</t>
+          <t>Stress fracture in lower right leg (ankle area); withdrew hours before her scheduled first-round match</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Missed 3 games; coach Becky Hammon said she could have played if it were a playoff game, suggesting an imminent return</t>
+          <t>Ruled out of Wimbledon 2026; still on crutches and wearing a protective boot several days after withdrawal, no return timeline given</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Loses out on Wimbledon prize money and ranking points for the event</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Aces without their All-Star forward/center for a short stretch, including a loss to Indiana</t>
+          <t>Removes a top British draw from the tournament</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1862,39 +1862,39 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>Yardbarker - Emma Raducanu setback deepens as British star remains on crutches after Wimbledon withdrawal</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://www.yardbarker.com/tennis/articles/emma_raducanu_setback_deepens_as_british_star_remains_on_crutches_after_wimbledon_withdrawal/s1_17460_44037038</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Caitlin Clark</t>
+          <t>Jordan Henderson</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Indiana Fever (WNBA)</t>
+          <t>England National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Aggravated back injury</t>
+          <t>Wrist fracture sustained in a freak fall while celebrating England's Round of 16 win over Mexico; reportedly requires surgery</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Has resumed practicing; no confirmed timeline yet for a game return</t>
+          <t>Ruled out for the remainder of the 2026 World Cup; exact surgery date and recovery length not yet specified</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Fever have played without their All-Star starting guard for an extended stretch</t>
+          <t>England advance to the quarterfinals without an experienced veteran midfielder, compounding a growing injury list</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1914,39 +1914,39 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>ESPN - England's Henderson hospitalized with wrist injury during celebration</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://www.espn.com/soccer/story/_/id/49283507/jordan-henderson-taken-hospital-wrist-injury-falling-mexico-victory-celebrations-england-world-cup</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Napheesa Collier</t>
+          <t>Santiago Gimenez</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Lynx (WNBA)</t>
+          <t>AC Milan (Serie A) / Mexico National Team</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Offseason surgery on both ankles</t>
+          <t>Grade II right ankle sprain suffered in stoppage time of Mexico's Round of 16 loss to England; hospitalized, but avoided fracture and ligament damage</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Has yet to play in the 2026 season; recently resumed practicing</t>
+          <t>Not yet specified by club or national team</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Lynx have been without their All-Star forward for the entire season to date</t>
+          <t>Injury compounds Mexico's World Cup elimination and raises concern over his fitness for AC Milan's preseason</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1966,39 +1966,39 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>beIN Sports - Adding insult to injury! Santiago Gimenez suffers injury during Mexico's loss to England</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://www.beinsports.com/en-us/soccer/fifa-world-cup-2026/articles/adding-insult-to-injury-santiago-gimenez-suffers-injury-during-mexico-s-loss-to-england-2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Byron Buxton</t>
+          <t>Ismael Saibari</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Twins (MLB)</t>
+          <t>Bayern Munich (Bundesliga, incoming) / Morocco National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Aggravated hip injury while being caught stealing in the 1st inning vs. Yankees</t>
+          <t>Hamstring injury (minor muscle issue per medical tests; serious strain ruled out) suffered in the 22nd minute of Morocco's Round of 16 win over Canada</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Day-to-day; had already missed 4 games earlier in the week with the same hip issue</t>
+          <t>Day-to-day pending fitness test; final decision on availability for the World Cup quarterfinal vs. France expected only hours before kickoff</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2008,49 +2008,49 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Twins lose their 2026 All-Star outfielder from the lineup for an undetermined stretch</t>
+          <t>Morocco risks losing their top attacking threat (three group-stage goals) for the biggest match of their World Cup run</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>The National - Ismael Saibari fitness concern for Morocco ahead of France World Cup quarter-final clash</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.thenationalnews.com/sport/world-cup-2026/2026/07/06/ismael-saibari-fitness-concern-for-morocco-ahead-of-france-world-cup-quarter-final-clash/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Jazz Chisholm Jr.</t>
+          <t>A'ja Wilson</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>New York Yankees (MLB)</t>
+          <t>Las Vegas Aces (WNBA)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Right toe discomfort, noticed jogging gingerly to first base after a fly out</t>
+          <t>Foot injury sustained in a game against the Chicago Sky</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Being monitored day-to-day; no IL move confirmed yet</t>
+          <t>Missed 3 games; coach Becky Hammon said she could have played if it were a playoff game, suggesting an imminent return</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2060,49 +2060,49 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Risk of losing Yankees' starting second baseman if it worsens</t>
+          <t>Aces without their All-Star forward/center for a short stretch, including a loss to Indiana</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Ranger Suarez</t>
+          <t>Caitlin Clark</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies (MLB)</t>
+          <t>Indiana Fever (WNBA)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Left adductor tightness, pulled early from start vs. Angels</t>
+          <t>Aggravated back injury</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Undetermined, pending further evaluation</t>
+          <t>Has resumed practicing; no confirmed timeline yet for a game return</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2112,49 +2112,49 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Phillies could lose their 2026 AL All-Star-caliber starter from the rotation</t>
+          <t>Fever have played without their All-Star starting guard for an extended stretch</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Brandon Woodruff</t>
+          <t>Napheesa Collier</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers (MLB)</t>
+          <t>Minnesota Lynx (WNBA)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Right shoulder inflammation</t>
+          <t>Offseason surgery on both ankles</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Placed on 15-day Injured List (minimum)</t>
+          <t>Has yet to play in the 2026 season; recently resumed practicing</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2164,34 +2164,34 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Brewers rotation loses a top starter for at least two full turns</t>
+          <t>Lynx have been without their All-Star forward for the entire season to date</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Covers - MLB Injuries 2026</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>https://www.covers.com/sport/baseball/mlb/injuries</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Triston Casas</t>
+          <t>Byron Buxton</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Boston Red Sox (MLB)</t>
+          <t>Minnesota Twins (MLB)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2201,12 +2201,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Torn right patellar tendon (out since May); recently shut down from hitting progression</t>
+          <t>Aggravated hip injury while being caught stealing in the 1st inning vs. Yankees</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Likely season-ending; setback in rehab timeline</t>
+          <t>Day-to-day; had already missed 4 games earlier in the week with the same hip issue</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Red Sox lose starting first baseman for the remainder of the 2026 season</t>
+          <t>Twins lose their 2026 All-Star outfielder from the lineup for an undetermined stretch</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2238,27 +2238,27 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>James Maddison</t>
+          <t>Jazz Chisholm Jr.</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Tottenham Hotspur (Premier League)</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>ACL reconstruction rehab (returning from tear)</t>
+          <t>Right toe discomfort, noticed jogging gingerly to first base after a fly out</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Ongoing; currently restricted to 20-25 minutes per match</t>
+          <t>Being monitored day-to-day; no IL move confirmed yet</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2268,101 +2268,101 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Spurs managing his minutes carefully, limiting his impact as a starter</t>
+          <t>Risk of losing Yankees' starting second baseman if it worsens</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Seamus Power</t>
+          <t>Ranger Suarez</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>PGA Tour</t>
+          <t>Philadelphia Phillies (MLB)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Golf</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Recurrence of long-standing back and hip issues he has dealt with since 2023</t>
+          <t>Left adductor tightness, pulled early from start vs. Angels</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Withdrew after an opening-round 6-over 77 at the John Deere Classic on July 2; no return timeline given</t>
+          <t>Undetermined, pending further evaluation</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Forfeits prize money and FedEx Cup points from the John Deere Classic</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Removes a two-time PGA Tour winner from the field partway through the event</t>
+          <t>Phillies could lose their 2026 AL All-Star-caliber starter from the rotation</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Golfmagic - Two-time PGA Tour winner forced out of John Deere Classic as injury problems strike again</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.golfmagic.com/tour/pga-tour/two-time-pga-tour-winner-forced-out-john-deere-classic-injury-problems-strike-again</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Nahikari Garcia</t>
+          <t>Brandon Woodruff</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Denver Summit FC (NWSL)</t>
+          <t>Milwaukee Brewers (MLB)</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Season-ending knee (ACL) injury</t>
+          <t>Right shoulder inflammation</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Out for the remainder of the 2026 NWSL season</t>
+          <t>Placed on 15-day Injured List (minimum)</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2372,49 +2372,49 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Denver Summit FC lose a starter for the rest of the season</t>
+          <t>Brewers rotation loses a top starter for at least two full turns</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Spotrac - 2026 NWSL Injured Tracker</t>
+          <t>Covers - MLB Injuries 2026</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
+          <t>https://www.covers.com/sport/baseball/mlb/injuries</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Brandon Ingram</t>
+          <t>Triston Casas</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Toronto Raptors (NBA)</t>
+          <t>Boston Red Sox (MLB)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Recovering from offseason surgery (lower body)</t>
+          <t>Torn right patellar tendon (out since May); recently shut down from hitting progression</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Expected back for training camp, fall 2026</t>
+          <t>Likely season-ending; setback in rehab timeline</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2424,49 +2424,49 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Raptors plan around his absence through the offseason program</t>
+          <t>Red Sox lose starting first baseman for the remainder of the 2026 season</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Brandon Ingram Injury Update Provided by Raptors After Surgery</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25426220-brandon-ingram-injury-update-provided-raptors-after-surgery-latest-timeline-2026-nba-season</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Josh Giddey</t>
+          <t>James Maddison</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Chicago Bulls (NBA)</t>
+          <t>Tottenham Hotspur (Premier League)</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Arthroscopic surgery on right ankle</t>
+          <t>ACL reconstruction rehab (returning from tear)</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>~3 months to resume basketball activities; targeting training camp</t>
+          <t>Ongoing; currently restricted to 20-25 minutes per match</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2476,101 +2476,101 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Bulls lose a starting guard for the entire offseason program</t>
+          <t>Spurs managing his minutes carefully, limiting his impact as a starter</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Josh Giddey Injury Update Provided by Bulls After Ankle Surgery</t>
+          <t>Premier League club injury coverage</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25427505-josh-giddey-injury-update-provided-bulls-after-ankle-surgery-latest-timeline-2026-nba-season</t>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Corey Seager</t>
+          <t>Seamus Power</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Texas Rangers (MLB)</t>
+          <t>PGA Tour</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Golf</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Recurrence of lower back inflammation; his third injured list stint of the 2026 season (previously missed time with the same back issue and with a concussion)</t>
+          <t>Recurrence of long-standing back and hip issues he has dealt with since 2023</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Placed on the 10-day injured list</t>
+          <t>Withdrew after an opening-round 6-over 77 at the John Deere Classic on July 2; no return timeline given</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Forfeits prize money and FedEx Cup points from the John Deere Classic</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Rangers lose their star shortstop again, continuing a season of infield instability; Josh Smith recalled from Triple-A as replacement</t>
+          <t>Removes a two-time PGA Tour winner from the field partway through the event</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Rangers' Corey Seager back on IL with lower back inflammation</t>
+          <t>Golfmagic - Two-time PGA Tour winner forced out of John Deere Classic as injury problems strike again</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49238350/rangers-corey-seager-back-il-lower-back-inflammation</t>
+          <t>https://www.golfmagic.com/tour/pga-tour/two-time-pga-tour-winner-forced-out-john-deere-classic-injury-problems-strike-again</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Brent Rooker</t>
+          <t>Nahikari Garcia</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Athletics (MLB)</t>
+          <t>Denver Summit FC (NWSL)</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Cartilage tear in left knee, discovered during an examination at Stanford; requires season-ending surgery</t>
+          <t>Season-ending knee (ACL) injury</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Season-ending; hadn't played since June 8 and had been on the injured list since June 9</t>
+          <t>Out for the remainder of the 2026 NWSL season</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2580,34 +2580,34 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Athletics lose their two-time All-Star middle-of-the-order bat for the remainder of the 2026 season</t>
+          <t>Denver Summit FC lose a starter for the rest of the season</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>ESPN - A's slugger Brent Rooker to have season-ending left knee surgery</t>
+          <t>Spotrac - 2026 NWSL Injured Tracker</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49244022/a-slugger-brent-rooker-season-ending-left-knee-surgery</t>
+          <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>JuJu Watkins</t>
+          <t>Brandon Ingram</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>USC Trojans (NCAA Division I Women's Basketball)</t>
+          <t>Toronto Raptors (NBA)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2617,12 +2617,12 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Recovering from a torn ACL that cost her the entire 2025-26 season</t>
+          <t>Recovering from offseason surgery (lower body)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Returned to the court roughly 14 months after the injury</t>
+          <t>Expected back for training camp, fall 2026</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>USC gets back its star guard after a full season lost to the injury</t>
+          <t>Raptors plan around his absence through the offseason program</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2642,24 +2642,24 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Fox Sports - 2026-2027 College Basketball Offseason Buzz</t>
+          <t>Bleacher Report - Brandon Ingram Injury Update Provided by Raptors After Surgery</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.foxsports.com/stories/college-basketball/college-basketball-2026-2027-buzz-news-injuries-transfers</t>
+          <t>https://bleacherreport.com/articles/25426220-brandon-ingram-injury-update-provided-raptors-after-surgery-latest-timeline-2026-nba-season</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Jaren Jackson Jr.</t>
+          <t>Josh Giddey</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Memphis Grizzlies (NBA)</t>
+          <t>Chicago Bulls (NBA)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2669,12 +2669,12 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Turf toe surgery (right foot)</t>
+          <t>Arthroscopic surgery on right ankle</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Re-evaluation in approximately 12 weeks</t>
+          <t>~3 months to resume basketball activities; targeting training camp</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2684,49 +2684,49 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Grizzlies lose their All-Star big man through the offseason and possibly into training camp</t>
+          <t>Bulls lose a starting guard for the entire offseason program</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>NBA.com - Grizzlies' Jaren Jackson Jr. has surgery to repair turf toe injury</t>
+          <t>Bleacher Report - Josh Giddey Injury Update Provided by Bulls After Ankle Surgery</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>https://www.nba.com/news/memphis-grizzlies-jaren-jackson-jr-turf-toe-surgery</t>
+          <t>https://bleacherreport.com/articles/25427505-josh-giddey-injury-update-provided-bulls-after-ankle-surgery-latest-timeline-2026-nba-season</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Manuel Ugarte</t>
+          <t>Corey Seager</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Manchester United (Premier League) / Uruguay National Team</t>
+          <t>Texas Rangers (MLB)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Knee ligament injury suffered vs. Spain at the World Cup; possible cruciate ligament (ACL) damage</t>
+          <t>Recurrence of lower back inflammation; his third injured list stint of the 2026 season (previously missed time with the same back issue and with a concussion)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Potentially several months if ACL is confirmed</t>
+          <t>Placed on the 10-day injured list</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2736,49 +2736,49 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Would be a significant blow to Manchester United's midfield depth heading into 2026-27</t>
+          <t>Rangers lose their star shortstop again, continuing a season of infield instability; Josh Smith recalled from Triple-A as replacement</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>ESPN - Rangers' Corey Seager back on IL with lower back inflammation</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.espn.com/mlb/story/_/id/49238350/rangers-corey-seager-back-il-lower-back-inflammation</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Rodri</t>
+          <t>Brent Rooker</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Manchester City (Premier League)</t>
+          <t>Athletics (MLB)</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Undisclosed injury expected to require surgery after the World Cup</t>
+          <t>Cartilage tear in left knee, discovered during an examination at Stanford; requires season-ending surgery</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Out for the opening weeks of the 2026-27 season</t>
+          <t>Season-ending; hadn't played since June 8 and had been on the injured list since June 9</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2788,34 +2788,34 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Manchester City to start the new season without their midfield anchor</t>
+          <t>Athletics lose their two-time All-Star middle-of-the-order bat for the remainder of the 2026 season</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>ESPN - A's slugger Brent Rooker to have season-ending left knee surgery</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.espn.com/mlb/story/_/id/49244022/a-slugger-brent-rooker-season-ending-left-knee-surgery</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Kelsey Plum</t>
+          <t>JuJu Watkins</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks (WNBA)</t>
+          <t>USC Trojans (NCAA Division I Women's Basketball)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2825,12 +2825,12 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Lower leg injury</t>
+          <t>Recovering from a torn ACL that cost her the entire 2025-26 season</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for at least 4 weeks as of late June; All-Star Game (July 25) status still to be decided</t>
+          <t>Returned to the court roughly 14 months after the injury</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2840,49 +2840,49 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Sparks lose a starting guard through their All-Star break stretch</t>
+          <t>USC gets back its star guard after a full season lost to the injury</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Angel Reese, Kelsey Plum Headline 2026 WNBA All-Star Game Reserves</t>
+          <t>Fox Sports - 2026-2027 College Basketball Offseason Buzz</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25452286-angel-reese-kelsey-plum-headline-2026-wnba-all-star-game-reserves-full-roster-announced</t>
+          <t>https://www.foxsports.com/stories/college-basketball/college-basketball-2026-2027-buzz-news-injuries-transfers</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Seth Jarvis</t>
+          <t>Jaren Jackson Jr.</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Carolina Hurricanes (NHL)</t>
+          <t>Memphis Grizzlies (NBA)</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Hockey</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Shoulder surgery, the same shoulder that had a torn labrum and rotator cuff during the 2023-24 season</t>
+          <t>Turf toe surgery (right foot)</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Expected recovery of approximately 4-6 months, meaning the earliest return would be late October</t>
+          <t>Re-evaluation in approximately 12 weeks</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2892,49 +2892,49 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Hurricanes will be without a top-six forward for the start of the 2026-27 season</t>
+          <t>Grizzlies lose their All-Star big man through the offseason and possibly into training camp</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>NHL.com - Jarvis expected to miss start of next season for Hurricanes after shoulder surgery</t>
+          <t>NBA.com - Grizzlies' Jaren Jackson Jr. has surgery to repair turf toe injury</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>https://www.nhl.com/news/seth-jarvis-to-miss-beginning-of-2026-2027-season-for-hurricanes-after-shoulder-surgery</t>
+          <t>https://www.nba.com/news/memphis-grizzlies-jaren-jackson-jr-turf-toe-surgery</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Bradley Beal</t>
+          <t>Manuel Ugarte</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>LA Clippers (NBA)</t>
+          <t>Manchester United (Premier League) / Uruguay National Team</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Hip fracture requiring season-ending surgery</t>
+          <t>Knee ligament injury suffered vs. Spain at the World Cup; possible cruciate ligament (ACL) damage</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Season-ending; recovery expected to extend into 2026-27 preseason</t>
+          <t>Potentially several months if ACL is confirmed</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2944,101 +2944,101 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Clippers lose a veteran guard for the balance of the season and into next year's planning</t>
+          <t>Would be a significant blow to Manchester United's midfield depth heading into 2026-27</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>NBA.com - Clippers' Bradley Beal (hip) to undergo season-ending surgery</t>
+          <t>Premier League club injury coverage</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.nba.com/news/clippers-bradley-beal-out-season-hip-fracture</t>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Bejlek</t>
+          <t>Rodri</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>Manchester City (Premier League)</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Elbow injury</t>
+          <t>Undisclosed injury expected to require surgery after the World Cup</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Withdrew mid-tournament from Eastbourne</t>
+          <t>Out for the opening weeks of the 2026-27 season</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Forfeits Eastbourne prize money/points from the round of withdrawal</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Opponent Zeynep Sonmez advances by walkover</t>
+          <t>Manchester City to start the new season without their midfield anchor</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>RotoWire - Fantasy Tennis Injury News</t>
+          <t>Premier League club injury coverage</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Matthijs de Ligt</t>
+          <t>Kelsey Plum</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Manchester United (Premier League)</t>
+          <t>Los Angeles Sparks (WNBA)</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Surgery on a long-standing back injury</t>
+          <t>Lower leg injury</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Will miss the 2026 World Cup; club return timeline unconfirmed</t>
+          <t>Ruled out for at least 4 weeks as of late June; All-Star Game (July 25) status still to be decided</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3048,101 +3048,101 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>United lose a starting center-back for an extended stretch</t>
+          <t>Sparks lose a starting guard through their All-Star break stretch</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>Bleacher Report - Angel Reese, Kelsey Plum Headline 2026 WNBA All-Star Game Reserves</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://bleacherreport.com/articles/25452286-angel-reese-kelsey-plum-headline-2026-wnba-all-star-game-reserves-full-roster-announced</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Elina Svitolina</t>
+          <t>Seth Jarvis</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>Carolina Hurricanes (NHL)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Hockey</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Hip injury</t>
+          <t>Shoulder surgery, the same shoulder that had a torn labrum and rotator cuff during the 2023-24 season</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Withdrew before her Bad Homburg quarterfinal</t>
+          <t>Expected recovery of approximately 4-6 months, meaning the earliest return would be late October</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Forfeits Bad Homburg quarterfinal prize money/points</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Opponent Xinyu Wang advances by walkover</t>
+          <t>Hurricanes will be without a top-six forward for the start of the 2026-27 season</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>RotoWire - Fantasy Tennis Injury News</t>
+          <t>NHL.com - Jarvis expected to miss start of next season for Hurricanes after shoulder surgery</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+          <t>https://www.nhl.com/news/seth-jarvis-to-miss-beginning-of-2026-2027-season-for-hurricanes-after-shoulder-surgery</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Chris Richards</t>
+          <t>Bradley Beal</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Crystal Palace (Premier League) / USMNT</t>
+          <t>LA Clippers (NBA)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Torn ankle ligaments (two ligaments) suffered vs. Brentford</t>
+          <t>Hip fracture requiring season-ending surgery</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Expected to recover in time for the 2026 World Cup</t>
+          <t>Season-ending; recovery expected to extend into 2026-27 preseason</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3152,72 +3152,280 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Crystal Palace lose a starting center-back for a multi-week stretch</t>
+          <t>Clippers lose a veteran guard for the balance of the season and into next year's planning</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>NBA.com - Clippers' Bradley Beal (hip) to undergo season-ending surgery</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.nba.com/news/clippers-bradley-beal-out-season-hip-fracture</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
+          <t>Bejlek</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>WTA Tour</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Elbow injury</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Withdrew mid-tournament from Eastbourne</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Forfeits Eastbourne prize money/points from the round of withdrawal</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Opponent Zeynep Sonmez advances by walkover</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>RotoWire - Fantasy Tennis Injury News</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Matthijs de Ligt</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Manchester United (Premier League)</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Soccer</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Surgery on a long-standing back injury</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Will miss the 2026 World Cup; club return timeline unconfirmed</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>United lose a starting center-back for an extended stretch</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Premier League club injury coverage</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Elina Svitolina</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>WTA Tour</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Hip injury</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Withdrew before her Bad Homburg quarterfinal</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Forfeits Bad Homburg quarterfinal prize money/points</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Opponent Xinyu Wang advances by walkover</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>RotoWire - Fantasy Tennis Injury News</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Chris Richards</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Crystal Palace (Premier League) / USMNT</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Soccer</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Torn ankle ligaments (two ligaments) suffered vs. Brentford</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Expected to recover in time for the 2026 World Cup</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Crystal Palace lose a starting center-back for a multi-week stretch</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Premier League club injury coverage</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
           <t>Chloe Ricketts</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>Boston Legacy FC (NWSL)</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>Soccer</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>Ankle injury</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>Placed on the 45-day short-term injury list</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>Not disclosed in available reporting</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>Boston Legacy FC without a rostered defender for at least 45 days</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr">
         <is>
           <t>Washington Spirit / NWSL transactions coverage</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr">
+      <c r="J57" s="2" t="inlineStr">
         <is>
           <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
         </is>
@@ -3277,10 +3485,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId53"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId57"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Daily injury update: Sabally, Reese, Ohtani, Kurtz, Manzambi, Guehi, Serena Williams and 9 more
</commit_message>
<xml_diff>
--- a/injury_report.xlsx
+++ b/injury_report.xlsx
@@ -145,8 +145,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Injuries" displayName="Injuries" ref="A1:J57" headerRowCount="1">
-  <autoFilter ref="A1:J57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Injuries" displayName="Injuries" ref="A1:J73" headerRowCount="1">
+  <autoFilter ref="A1:J73"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Athlete"/>
     <tableColumn id="2" name="Organization"/>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -522,12 +522,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Collin Murray-Boyles</t>
+          <t>Satou Sabally</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Toronto Raptors (NBA) — Las Vegas Summer League</t>
+          <t>New York Liberty (WNBA)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -537,12 +537,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Sprained thumb/finger, diagnosed after exiting a Summer League game against the Lakers</t>
+          <t>Concussion protocol after being elbowed in the face by Aces forward NaLyssa Smith while contesting a rebound; symptoms had delayed onset</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the Raptors' Summer League opener vs. Boston; next possible return targeted for the Houston game; full recovery timeline not specified in available reporting</t>
+          <t>Downgraded from questionable to out; remains in concussion protocol with no return timeline given</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -552,49 +552,49 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Raptors lose their 2025 first-round pick (9th overall) for early Summer League reps as a point-forward, part of his developmental push</t>
+          <t>Liberty without their All-Star forward for multiple games as she works through the NBA/WNBA-mandated concussion protocol; notable given she also missed time with a concussion in the 2025 WNBA Finals</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Raptors Republic - Collin Murray-Boyles, Alijah Martin to miss Raptors' Summer League opener</t>
+          <t>Yahoo Sports - Liberty injury report: Star forward Satou Sabally in concussion protocol</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>https://raptorsrepublic.com/2026/07/10/collin-murray-boyles-alijah-martin-to-miss-raptors-summer-league-opener/</t>
+          <t>https://sports.yahoo.com/articles/liberty-injury-report-star-forward-satou-sabally-in-concussion-protocol-224647068.html</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Gout Gout</t>
+          <t>Angel Reese</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Athletics Australia (Track &amp; Field)</t>
+          <t>Atlanta Dream (WNBA)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Athletics (Track &amp; Field)</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Grade-three left hamstring tear suffered in training in Brisbane</t>
+          <t>Lower leg/ankle injury sustained falling under the basket late in a win over the Seattle Storm</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of the 2026 season, including the World Athletics U20 Championships (Aug. 5-9, Eugene, Oregon); targeting a return in 2027</t>
+          <t>Listed questionable for the Dream's game vs. the Portland Fire; no firm return timeline given</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -604,49 +604,49 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Removes the U20 200m world record holder from an anticipated showdown with American Tate Taylor at the World U20 Championships</t>
+          <t>Puts a third-straight All-Star selection and Dream's first year with Reese (acquired in an offseason trade from Chicago) at risk of interruption during a stretch where the team is trying to build momentum after a five-game losing streak</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Olympics.com - Gout Gout to miss World U20 Championships and rest of the season with hamstring injury</t>
+          <t>CBS Sports - Portland Fire vs. Atlanta Dream preview: Dream seek momentum as Angel Reese is questionable with leg injury</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>https://www.olympics.com/en/news/gout-gout-injury-hamstring-world-athletics-under-20-championships</t>
+          <t>https://www.cbssports.com/wnba/news/portland-fire-atlanta-dream-where-to-watch-angel-reese-injury/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Harshit Rana</t>
+          <t>Brionna Jones</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>India National Cricket Team</t>
+          <t>Atlanta Dream (WNBA)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury sustained during the third T20I vs. England at Trent Bridge</t>
+          <t>Meniscus tear in the right knee suffered in late January while playing overseas for USK Prague; underwent knee surgery at Emory Hospital</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
+          <t>Ruled out to begin the 2026 season and remains sidelined into mid-July; not yet cleared for 5-on-5 drills and has no firm return timetable, though the team says she is expected to make a full recovery</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -656,49 +656,49 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Deepens India's bowling injury crisis on the England tour, with Rana joining Varun Chakaravarthy, Hardik Pandya, and Nitish Kumar Reddy on the unavailable list</t>
+          <t>Four-time All-Star center has yet to play a game for the Dream this season, a significant frontcourt loss to start the year</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
+          <t>CBS News Atlanta - Atlanta Dream's Brionna Jones nearing return, expected back with team soon</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
+          <t>https://www.cbsnews.com/atlanta/news/atlanta-dreams-brionna-jones-nearing-return-expected-back-with-team-next-week/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Varun Chakaravarthy</t>
+          <t>Leonie Fiebich</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>India National Cricket Team</t>
+          <t>New York Liberty (WNBA)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury sustained during the third T20I vs. England at Trent Bridge</t>
+          <t>Left foot soreness</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
+          <t>Ruled out for a second straight game, having missed her first game since May 25; no return timeline given</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -708,49 +708,49 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>India's frontline wrist-spinner is unavailable as the team's injury list grows on the England tour</t>
+          <t>Liberty forward sidelined for consecutive games amid a compressed schedule that includes a quick turnaround for a game in Toronto</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
+          <t>Yahoo Sports - Final Injury Report for Liberty-Mystics: Will Satou Sabally, Leonie Fiebich Play?</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
+          <t>https://sports.yahoo.com/articles/final-injury-report-liberty-mystics-150000047.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Litton Das</t>
+          <t>Johan Manzambi</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh national cricket team</t>
+          <t>Switzerland National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Left calf injury; failed a fitness test ahead of the second ODI</t>
+          <t>Left-knee injury suffered in training on the eve of the Round of 16 match vs. Colombia</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the remainder of the ODI series vs. Zimbabwe; continuing rehab in Dhaka</t>
+          <t>Missed the Round of 16 win over Colombia and ruled out of the quarterfinal vs. Argentina; no return timeline given</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -760,49 +760,49 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh loses their starting wicketkeeper-batter for the series; Parvez Hossain Emon named as replacement for the 2nd and 3rd ODIs</t>
+          <t>Major blow to Switzerland's attack: with Manzambi on the pitch during the group stage the team averaged 3.6 goals per 90 minutes (3 goals, 2 assists for him in 200 minutes); without him, Switzerland have scored just once and averaged 1.4 xG per 90 over 280 minutes</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>The Nation - Injured Litton Das to miss rest of Zimbabwe ODI series</t>
+          <t>ESPN - Switzerland's Johan Manzambi to miss Argentina World Cup quarterfinal clash - Murat Yakin</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>https://www.nation.com.pk/09-Jul-2026/injured-litton-das-miss-rest-zimbabwe-odi-series</t>
+          <t>https://www.espn.com/soccer/story/_/id/49326340/switzerland-johan-manzambi-miss-argentina-world-cup-quarterfinal-clash-murat-yakin</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Ravichandran Ashwin</t>
+          <t>Marc Guehi</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>San Francisco Unicorns (Major League Cricket)</t>
+          <t>England National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Right knee injury</t>
+          <t>Hamstring strain picked up in England's Round of 16 win over Mexico</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of MLC 2026; replaced by Peter Siddle</t>
+          <t>Missed a training session in Kansas City but returned to training Friday and was confirmed available for the quarterfinal vs. Norway</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -812,34 +812,34 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Unicorns lose the veteran spinner after just one appearance this MLC season</t>
+          <t>Created a late fitness scare for England's back line ahead of the quarterfinal, with Newcastle's Dan Burn on standby to deputize had Guehi been unavailable</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>India TV News - Why is Ravichandran Ashwin ruled out of ongoing MLC 2026? San Francisco Unicorns announce replacement</t>
+          <t>Sky Sports - World Cup 2026: England defender Marc Guehi a serious doubt for quarter-final clash with Norway</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>https://www.indiatvnews.com/sports/cricket/why-is-ravichandran-ashwin-ruled-out-of-ongoing-mlc-2026-san-francisco-unicorns-announce-replacement-2026-07-09-1047737</t>
+          <t>https://www.skysports.com/football/news/12016/13562168/world-cup-2026-england-defender-marc-guehi-a-serious-doubt-for-quarter-final-clash-with-norway</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Aaron Judge</t>
+          <t>Nick Kurtz</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>New York Yankees (MLB)</t>
+          <t>Athletics (MLB)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Stress fracture in right rib; has not played since May 31 and went on the injured list June 5</t>
+          <t>Right thumb capsule sprain</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Will have the rib reimaged during the All-Star break; no firm return date, GM Brian Cashman says he must be fully asymptomatic and show healing on imaging before resuming activity</t>
+          <t>Placed on the 10-day injured list, retroactive to July 10</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -864,34 +864,34 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Yankees continue without their three-time AL MVP and captain in the middle of the lineup</t>
+          <t>Keeps the 2025 AL Rookie of the Year and scheduled AL All-Star starting first baseman (.266, 20 HR, 66 RBI, MLB-leading 76 walks) out of the July 14 All-Star Game in Philadelphia; catcher Brian Serven recalled from Triple-A in a corresponding move</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Yankees' Aaron Judge to have rib reimaged during All-Star break</t>
+          <t>ESPN - Athletics All-Star 1B Nick Kurtz placed on IL with thumb sprain</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49317023/yankees-aaron-judge-rib-reimaged-all-star-break</t>
+          <t>https://www.espn.com/mlb/story/_/id/49334996/athletics-all-star-1b-nick-kurtz-placed-il-thumb-sprain</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Mark Vientos</t>
+          <t>Nick Lodolo</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>New York Mets (MLB)</t>
+          <t>Cincinnati Reds (MLB)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -901,12 +901,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Fractured bone in right hand after being hit by a pitch from Michael Wacha</t>
+          <t>Blister on the left index finger (throwing hand); a recurring issue, his fourth stint on the IL for blisters dating back to 2024</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Headed to the injured list; broken bones of this type typically take around six weeks to heal, though the Mets have not given an official timeline and have not yet said whether surgery is needed</t>
+          <t>Placed on the 15-day injured list; eligible to return July 27, though it could take longer depending on severity</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -916,34 +916,34 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Mets lose a regular infielder/DH (.211, 11 HR, 35 RBI in 72 games) just ahead of the trade deadline</t>
+          <t>Reds turn to Rhett Lowder to fill Lodolo's rotation spot</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>amNewYork - Mark Vientos injury: Mets IF/DH headed to IL with hand fracture</t>
+          <t>MLB Trade Rumors - Reds Place Nick Lodolo On IL With Blister, Recall Chase Petty</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>https://www.amny.com/sports/mark-vientos-injury-mets-7-9-26/</t>
+          <t>https://www.mlbtraderumors.com/2026/07/reds-place-nick-lodolo-on-il-with-blister-recall-chase-petty.html</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Athletics (MLB)</t>
+          <t>New York Mets (MLB)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -953,12 +953,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Deep cut underneath the right kneecap after colliding with the left field fence on a sliding catch; came just missed the tendon per the team</t>
+          <t>General leg soreness and right ankle soreness, aggravated by fouling balls off his legs during a series in Atlanta</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Left the July 9 game early; scheduled for an MRI on July 10 to confirm the extent of the injury</t>
+          <t>Held out of the lineup for a second straight game and available only off the bench; expected to use the following day and the All-Star break for a full reset rather than go on the injured list</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -968,49 +968,49 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Athletics risk losing an everyday infielder/outfielder who had an on-base streak of 27 straight games and a 13-game scoring streak snapped by the injury</t>
+          <t>Mets manage his workload during a productive stretch (.320 avg, .788 OPS over his last 25 games) heading into the All-Star break</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Athletics' Gelof to have MRI on knee after sliding into fence</t>
+          <t>Associated Press - Bo Bichette held out of Mets' lineup for second straight game with leg soreness</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49319837/athletics-gelof-mri-knee-sliding-fence</t>
+          <t>https://www.bakersfield.com/ap/sports/bo-bichette-held-out-of-mets-lineup-for-second-straight-game-with-leg-soreness/article_c615803d-891c-57fd-87ef-b86becfaf8cc.html</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Chinelle Henry</t>
+          <t>Collin Murray-Boyles</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>West Indies Women's National Cricket Team</t>
+          <t>Toronto Raptors (NBA) — Las Vegas Summer League</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Exacerbation of a previous injury originally suffered fielding (stretchered off) in a T20 World Cup warm-up match in June</t>
+          <t>Sprained thumb/finger, diagnosed after exiting a Summer League game against the Lakers</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the Women's ODI tour of Ireland beginning July 10; no return timeline disclosed</t>
+          <t>Ruled out of the Raptors' Summer League opener vs. Boston; next possible return targeted for the Houston game; full recovery timeline not specified in available reporting</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1020,49 +1020,49 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>West Indies lose their vice-captain and a key all-rounder; Realeanna Grimmond called up as her replacement for the Ireland series</t>
+          <t>Raptors lose their 2025 first-round pick (9th overall) for early Summer League reps as a point-forward, part of his developmental push</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>ESPNcricinfo - Realeanna Grimmond replaces injured Chinelle Henry in West Indies squad for Ireland Women's ODIs</t>
+          <t>Raptors Republic - Collin Murray-Boyles, Alijah Martin to miss Raptors' Summer League opener</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>https://www.espncricinfo.com/story/slug-1545066</t>
+          <t>https://raptorsrepublic.com/2026/07/10/collin-murray-boyles-alijah-martin-to-miss-raptors-summer-league-opener/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Torstein Træen</t>
+          <t>Shohei Ohtani</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Uno-X Mobility (Tour de France) — Norway</t>
+          <t>Los Angeles Dodgers (MLB)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Cycling</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Concussion and multiple fractured ribs sustained in a crash on the descent of the Col du Tourmalet during stage 6</t>
+          <t>Left knee irritation/swelling, nursed since at least June 11</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Withdrew from the Tour de France (did not start stage 7); no return timeline specified in available reporting</t>
+          <t>Scratched from his Friday, July 10 pitching start vs. Arizona and will skip the All-Star Game; scheduled to have the knee drained and possibly receive a pain-relieving injection during the break</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1072,49 +1072,49 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Uno-X Mobility loses the rider who had been wearing the race's yellow jersey after stage 5; Tadej Pogačar reclaimed the overall race lead the same day</t>
+          <t>Dodgers manage the two-way star's workload heading into the second half; Ohtani continued to DH and homered the same day he was scratched from pitching</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Cyclingnews - 'Not the ending we wanted for this yellow adventure' - Torstein Træen out of Tour de France due to injuries from Tourmalet crash</t>
+          <t>ESPN - Shohei Ohtani dealing with knee irritation, to miss All-Star Game</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://www.cyclingnews.com/pro-cycling/teams-riders/not-the-ending-we-wanted-for-this-yellow-adventure-torstein-traeen-out-of-tour-de-france-due-to-injuries-from-tourmalet-crash/</t>
+          <t>https://www.espn.com/mlb/story/_/id/49327458/shohei-ohtani-dealing-knee-irritation-miss-all-star-game</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Alex Molenaar</t>
+          <t>Gout Gout</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Caja Rural-Seguros RGA (Tour de France) — Netherlands</t>
+          <t>Athletics Australia (Track &amp; Field)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Cycling</t>
+          <t>Athletics (Track &amp; Field)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Fracture of the first metacarpal in his right hand plus multiple contusions, sustained in a high-speed crash roughly 5km from the finish of stage 5; evaluated under concussion protocol after losing memory of the incident</t>
+          <t>Grade-three left hamstring tear suffered in training in Brisbane</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Abandoned the Tour de France; did not start stage 6; recovery timeline not specified in available reporting</t>
+          <t>Ruled out for the remainder of the 2026 season, including the World Athletics U20 Championships (Aug. 5-9, Eugene, Oregon); targeting a return in 2027</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Caja Rural-Seguros RGA loses a rider mid-Tour</t>
+          <t>Removes the U20 200m world record holder from an anticipated showdown with American Tate Taylor at the World U20 Championships</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1134,39 +1134,39 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Cycling Weekly - 'I don't remember the crash' – Caja Rural rider abandons Tour de France with fractured hand</t>
+          <t>Olympics.com - Gout Gout to miss World U20 Championships and rest of the season with hamstring injury</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>https://www.cyclingweekly.com/racing/tour-de-france/i-dont-remember-the-crash-caja-rural-rider-abandons-tour-de-france-with-fractured-hand</t>
+          <t>https://www.olympics.com/en/news/gout-gout-injury-hamstring-world-athletics-under-20-championships</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Arvid de Kleijn</t>
+          <t>Harshit Rana</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Tudor Pro Cycling Team (Tour de France) — Netherlands</t>
+          <t>India National Cricket Team</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Cycling</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Muscle tears sustained during the stage 1 team time trial, which hampered him for the rest of the race</t>
+          <t>Hamstring injury sustained during the third T20I vs. England at Trent Bridge</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Abandoned the Tour de France on stage 6 after struggling since the opening days; recovery timeline not specified in available reporting</t>
+          <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Tudor Pro Cycling Team loses a rider mid-Tour after he battled to beat the time cut on multiple stages</t>
+          <t>Deepens India's bowling injury crisis on the England tour, with Rana joining Varun Chakaravarthy, Hardik Pandya, and Nitish Kumar Reddy on the unavailable list</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1186,39 +1186,39 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>idlprocycling - Suffering ends: Arvid de Kleijn and Cian Uijtdebroeks abandon Tour de France</t>
+          <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.idlprocycling.com/cycling/suffering-ends-arvid-de-kleijn-and-cian-uijtdebroeks-abandon-tour-de-france</t>
+          <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Connor Bedard</t>
+          <t>Varun Chakaravarthy</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Chicago Blackhawks (NHL)</t>
+          <t>India National Cricket Team</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hockey</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Surgery on left shoulder after an injury sustained during a practice session in Vancouver on July 2</t>
+          <t>Hamstring injury sustained during the third T20I vs. England at Trent Bridge</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Expected to need approximately four months to recover; will miss training camp and at least the start of the 2026-27 season</t>
+          <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1228,49 +1228,49 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Blackhawks will open the 2026-27 season, played under the NHL's expanded 84-game schedule, without their No. 1 center for at least the opening month</t>
+          <t>India's frontline wrist-spinner is unavailable as the team's injury list grows on the England tour</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>NHL.com - Bedard to miss start of 2026-27 season for Blackhawks after shoulder surgery</t>
+          <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>https://www.nhl.com/news/connor-bedard-injury-status-update-july-8-2026</t>
+          <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Aliyah Boston</t>
+          <t>Litton Das</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Indiana Fever (WNBA)</t>
+          <t>Bangladesh national cricket team</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Lower right leg injury</t>
+          <t>Left calf injury; failed a fitness test ahead of the second ODI</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Listed out for the Fever's game vs. the LA Sparks; expected to be available for the following game vs. Phoenix</t>
+          <t>Ruled out of the remainder of the ODI series vs. Zimbabwe; continuing rehab in Dhaka</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1280,49 +1280,49 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Fever forced to manage the availability of both Boston and Caitlin Clark during a back-to-back stretch; Boston, a voted-in 2026 All-Star starter, is having a career-best scoring season (17.1 ppg on 50.4% shooting) and was in danger of missing her first game since May 17</t>
+          <t>Bangladesh loses their starting wicketkeeper-batter for the series; Parvez Hossain Emon named as replacement for the 2nd and 3rd ODIs</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Athlon Sports - Indiana Fever Announce Aliyah Boston Injury Update Before LA Sparks Game</t>
+          <t>The Nation - Injured Litton Das to miss rest of Zimbabwe ODI series</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://athlonsports.com/wnba/indiana-fever/indiana-fever-announce-aliyah-boston-injury-update-la-sparks-game</t>
+          <t>https://www.nation.com.pk/09-Jul-2026/injured-litton-das-miss-rest-zimbabwe-odi-series</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Reece James</t>
+          <t>Ravichandran Ashwin</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Chelsea FC (Premier League) / England National Team (2026 FIFA World Cup)</t>
+          <t>San Francisco Unicorns (Major League Cricket)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury sustained in England's final group-stage match vs. Ghana on June 23; described by reporting as worse than first thought</t>
+          <t>Right knee injury</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Touch-and-go for England's July 11 World Cup quarterfinal vs. Norway; has missed England's last three matches and was the sole absentee from the team's final group training session, requiring final medical clearance just to be considered for the bench</t>
+          <t>Ruled out for the remainder of MLC 2026; replaced by Peter Siddle</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1332,49 +1332,49 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Compounds an England right-back crisis that worsened after Jarell Quansah's red card vs. Mexico, leaving manager Thomas Tuchel with very limited options at the position for the quarterfinal</t>
+          <t>Unicorns lose the veteran spinner after just one appearance this MLC season</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Sky Sports - England World Cup latest: Reece James in race to be fit for quarter-final clash with Norway to ease right-back crisis</t>
+          <t>India TV News - Why is Ravichandran Ashwin ruled out of ongoing MLC 2026? San Francisco Unicorns announce replacement</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>https://www.skysports.com/football/news/11095/13561150/england-world-cup-latest-reece-james-in-race-to-be-fit-for-quarter-final-clash-with-norway-to-ease-right-back-crisis</t>
+          <t>https://www.indiatvnews.com/sports/cricket/why-is-ravichandran-ashwin-ruled-out-of-ongoing-mlc-2026-san-francisco-unicorns-announce-replacement-2026-07-09-1047737</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Aurelien Tchouameni</t>
+          <t>Aaron Judge</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Real Madrid (La Liga) / France National Team (2026 FIFA World Cup)</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Muscle tear involving the left adductor and upper thigh, a recurrence of the groin/thigh issue that previously sidelined him for France's group-stage match vs. Iraq</t>
+          <t>Stress fracture in right rib; has not played since May 31 and went on the injured list June 5</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Missed France's Round of 16 win over Paraguay; returned to partial team training on July 8, with a decision on his availability for the July 11 quarterfinal vs. Morocco pending</t>
+          <t>Will have the rib reimaged during the All-Star break; no firm return date, GM Brian Cashman says he must be fully asymptomatic and show healing on imaging before resuming activity</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1384,49 +1384,49 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>France's vice-captain and starting defensive midfielder is a doubt for the quarterfinal, with Manu Kone deputizing in his absence</t>
+          <t>Yankees continue without their three-time AL MVP and captain in the middle of the lineup</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Sportskeeda - France handed huge injury boost as star man returns to training ahead of FIFA World Cup Q/F against Morocco</t>
+          <t>ESPN - Yankees' Aaron Judge to have rib reimaged during All-Star break</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.sportskeeda.com/football/rumor-france-handed-huge-injury-boost-star-man-returns-training-ahead-fifa-world-cup-q-f-morocco-reports</t>
+          <t>https://www.espn.com/mlb/story/_/id/49317023/yankees-aaron-judge-rib-reimaged-all-star-break</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mustafizur Rahman</t>
+          <t>Mark Vientos</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh National Cricket Team</t>
+          <t>New York Mets (MLB)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Grade 1 muscle tear in the right hamstring and meniscal degeneration in the right knee, felt while bowling in the first ODI vs. Zimbabwe</t>
+          <t>Fractured bone in right hand after being hit by a pitch from Michael Wacha</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for four weeks, covering the remainder of Bangladesh's tour of Zimbabwe (concluding July 19), including the T20I series; has returned home for rehab</t>
+          <t>Headed to the injured list; broken bones of this type typically take around six weeks to heal, though the Mets have not given an official timeline and have not yet said whether surgery is needed</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1436,34 +1436,34 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh lose a frontline pace bowler for the rest of the Zimbabwe tour</t>
+          <t>Mets lose a regular infielder/DH (.211, 11 HR, 35 RBI in 72 games) just ahead of the trade deadline</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>ESPNcricinfo - Zim vs Ban: Mustafizur Rahman ruled out for four weeks with hamstring and knee injuries</t>
+          <t>amNewYork - Mark Vientos injury: Mets IF/DH headed to IL with hand fracture</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>https://www.espncricinfo.com/story/zim-vs-ban-mustafizur-rahman-ruled-out-for-four-weeks-with-hamstring-and-knee-injuries-1545065</t>
+          <t>https://www.amny.com/sports/mark-vientos-injury-mets-7-9-26/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Marco Raya</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Twins (MLB)</t>
+          <t>Athletics (MLB)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1473,12 +1473,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Right shoulder impingement</t>
+          <t>Deep cut underneath the right kneecap after colliding with the left field fence on a sliding catch; came just missed the tendon per the team</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Placed on 15-day IL July 8, retroactive to July 5</t>
+          <t>Left the July 9 game early; scheduled for an MRI on July 10 to confirm the extent of the injury</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1488,49 +1488,49 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Twins lose a pitching option for at least 15 days</t>
+          <t>Athletics risk losing an everyday infielder/outfielder who had an on-base streak of 27 straight games and a 13-game scoring streak snapped by the injury</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>MLB.com - Latest Twins injuries &amp; transactions</t>
+          <t>ESPN - Athletics' Gelof to have MRI on knee after sliding into fence</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.mlb.com/news/twins-injuries-and-roster-moves</t>
+          <t>https://www.espn.com/mlb/story/_/id/49319837/athletics-gelof-mri-knee-sliding-fence</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Endy Rodriguez</t>
+          <t>Chinelle Henry</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates (MLB)</t>
+          <t>West Indies Women's National Cricket Team</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Left glute strain</t>
+          <t>Exacerbation of a previous injury originally suffered fielding (stretchered off) in a T20 World Cup warm-up match in June</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Placed on 10-day IL July 8, retroactive to July 6</t>
+          <t>Ruled out of the Women's ODI tour of Ireland beginning July 10; no return timeline disclosed</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1540,49 +1540,49 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Pirates lose their starting catcher for at least 10 days</t>
+          <t>West Indies lose their vice-captain and a key all-rounder; Realeanna Grimmond called up as her replacement for the Ireland series</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>MLB Trade Rumors - Pirates Place Endy Rodriguez On Injured List</t>
+          <t>ESPNcricinfo - Realeanna Grimmond replaces injured Chinelle Henry in West Indies squad for Ireland Women's ODIs</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://www.mlbtraderumors.com/2026/07/pirates-to-place-endy-rodriguez-on-injured-list.html</t>
+          <t>https://www.espncricinfo.com/story/slug-1545066</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Jalen Brunson</t>
+          <t>Torstein Træen</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>New York Knicks (NBA)</t>
+          <t>Uno-X Mobility (Tour de France) — Norway</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Cycling</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Surgery to repair a left wrist injury that he played through during the Knicks' championship playoff run</t>
+          <t>Concussion and multiple fractured ribs sustained in a crash on the descent of the Col du Tourmalet during stage 6</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>At least two months of rehab expected; targeting readiness for the start of the 2026-27 NBA season</t>
+          <t>Withdrew from the Tour de France (did not start stage 7); no return timeline specified in available reporting</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1592,49 +1592,49 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Reigning Finals MVP and starting point guard sidelined for part of the offseason program, though expected back for training camp</t>
+          <t>Uno-X Mobility loses the rider who had been wearing the race's yellow jersey after stage 5; Tadej Pogačar reclaimed the overall race lead the same day</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports - Knicks superstar Jalen Brunson undergoes left wrist surgery, expected to be ready for 2026-27 NBA season</t>
+          <t>Cyclingnews - 'Not the ending we wanted for this yellow adventure' - Torstein Træen out of Tour de France due to injuries from Tourmalet crash</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/nba/breaking-news/article/knicks-superstar-jalen-brunson-undergoes-left-wrist-surgery-expected-to-be-ready-for-2026-27-nba-season-155927234.html</t>
+          <t>https://www.cyclingnews.com/pro-cycling/teams-riders/not-the-ending-we-wanted-for-this-yellow-adventure-torstein-traeen-out-of-tour-de-france-due-to-injuries-from-tourmalet-crash/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Amadou Onana</t>
+          <t>Alex Molenaar</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Aston Villa (Premier League) / Belgium National Team (2026 FIFA World Cup)</t>
+          <t>Caja Rural-Seguros RGA (Tour de France) — Netherlands</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Cycling</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Torn anterior cruciate ligament (ACL), sustained in the 21st minute of Belgium's Round of 16 win over the United States after a challenge with Christian Pulisic</t>
+          <t>Fracture of the first metacarpal in his right hand plus multiple contusions, sustained in a high-speed crash roughly 5km from the finish of stage 5; evaluated under concussion protocol after losing memory of the incident</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of the World Cup; reported to be facing up to eight months out</t>
+          <t>Abandoned the Tour de France; did not start stage 6; recovery timeline not specified in available reporting</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1644,49 +1644,49 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Belgium loses a key defensive midfielder ahead of their World Cup quarterfinal vs. Spain, and Aston Villa will be without him for a significant part of the 2026-27 season</t>
+          <t>Caja Rural-Seguros RGA loses a rider mid-Tour</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Belgium's Amadou Onana out of World Cup after suffering ACL injury</t>
+          <t>Cycling Weekly - 'I don't remember the crash' – Caja Rural rider abandons Tour de France with fractured hand</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49298508/belgium-amadou-onana-world-cup-suffering-acl-injury</t>
+          <t>https://www.cyclingweekly.com/racing/tour-de-france/i-dont-remember-the-crash-caja-rural-rider-abandons-tour-de-france-with-fractured-hand</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Giancarlo Stanton</t>
+          <t>Arvid de Kleijn</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>New York Yankees (MLB)</t>
+          <t>Tudor Pro Cycling Team (Tour de France) — Netherlands</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Cycling</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Right calf strain (originally suffered running the bases on April 24 vs. the Astros); recent rehab setback after re-aggravating the calf during a running progression</t>
+          <t>Muscle tears sustained during the stage 1 team time trial, which hampered him for the rest of the race</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>No firm timeline; has not resumed running since the setback, no target return date given</t>
+          <t>Abandoned the Tour de France on stage 6 after struggling since the opening days; recovery timeline not specified in available reporting</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1696,29 +1696,29 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Yankees continue without their veteran slugger amid an offense that has struggled with injuries; manager Aaron Boone still expects him back at some point in 2026</t>
+          <t>Tudor Pro Cycling Team loses a rider mid-Tour after he battled to beat the time cut on multiple stages</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Last Word on Sports - Stanton Injury Update: Slugger Yet To Resume Rehab On Calf</t>
+          <t>idlprocycling - Suffering ends: Arvid de Kleijn and Cian Uijtdebroeks abandon Tour de France</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://lastwordonsports.com/baseball/2026/07/07/nyy-stanton-injury-update/</t>
+          <t>https://www.idlprocycling.com/cycling/suffering-ends-arvid-de-kleijn-and-cian-uijtdebroeks-abandon-tour-de-france</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Matteo Berrettini</t>
+          <t>Carlos Alcaraz</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1733,64 +1733,64 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Diagnosed with chronic hip pain, a recurrence of the left hip issue that forced his retirement from his Roland Garros quarterfinal in early June</t>
+          <t>Right-wrist tenosynovitis, forcing withdrawals from Madrid, Rome, Roland Garros, Queen's and Wimbledon; has worn a wrist brace since mid-April</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Withdrawing from the ATP tournaments in Gstaad and Kitzbuhel to rest on medical advice, with the goal of being ready for the US hard-court swing culminating in the US Open; no firm return date given</t>
+          <t>Has pulled out of the ATP Montreal entry list and opted to prolong his comeback by two more weeks, targeting Cincinnati or the US Open for his return; recently resumed light on-court practice without a brace</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Forfeits ranking points and prize money from both the Gstaad and Kitzbuhel events</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Removes him from the draw at both tournaments immediately following his third-round Wimbledon loss to Grigor Dimitrov</t>
+          <t>World No. 2 has now missed a full clay and grass swing including two Grand Slams; absence continues into the North American hard-court season</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Puntodebreak - Berrettini withdraws from competing in upcoming tournaments due to "chronic hip pain"</t>
+          <t>Last Word On Tennis - Carlos Alcaraz Injury Update: Spaniard Pulls Out of ATP Montreal Entry List</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://www.puntodebreak.com/en/2026/07/07/berrettini-withdraws-from-competing-in-upcoming-tournaments-due-to-chronic-hip-pain</t>
+          <t>https://lastwordonsports.com/tennis/2026/07/09/carlos-alcaraz-injury-update-spaniard-pulls-out-of-atp-montreal/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Skylar Diggins</t>
+          <t>Connor Bedard</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Chicago Sky (WNBA)</t>
+          <t>Chicago Blackhawks (NHL)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Hockey</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Right knee injury; Diggins has said a knee surgery from last October has contributed to ongoing strain</t>
+          <t>Surgery on left shoulder after an injury sustained during a practice session in Vancouver on July 2</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the July 7 game vs. Phoenix Mercury; no return timeline given</t>
+          <t>Expected to need approximately four months to recover; will miss training camp and at least the start of the 2026-27 season</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1800,86 +1800,86 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Comes as Diggins was moved to the bench for the first time in a decade, ending a streak of 341 consecutive starts; Sky beat Phoenix 77-66 in her absence</t>
+          <t>Blackhawks will open the 2026-27 season, played under the NHL's expanded 84-game schedule, without their No. 1 center for at least the opening month</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports - Sky's Skylar Diggins ruled out (knee) after being benched, Vandersloot starting</t>
+          <t>NHL.com - Bedard to miss start of 2026-27 season for Blackhawks after shoulder surgery</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/articles/skys-skylar-diggins-ruled-vs-010259203.html</t>
+          <t>https://www.nhl.com/news/connor-bedard-injury-status-update-july-8-2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Emma Raducanu</t>
+          <t>Aliyah Boston</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>Indiana Fever (WNBA)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Stress fracture in lower right leg (ankle area); withdrew hours before her scheduled first-round match</t>
+          <t>Lower right leg injury</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of Wimbledon 2026; still on crutches and wearing a protective boot several days after withdrawal, no return timeline given</t>
+          <t>Listed out for the Fever's game vs. the LA Sparks; expected to be available for the following game vs. Phoenix</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Loses out on Wimbledon prize money and ranking points for the event</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Removes a top British draw from the tournament</t>
+          <t>Fever forced to manage the availability of both Boston and Caitlin Clark during a back-to-back stretch; Boston, a voted-in 2026 All-Star starter, is having a career-best scoring season (17.1 ppg on 50.4% shooting) and was in danger of missing her first game since May 17</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - Emma Raducanu setback deepens as British star remains on crutches after Wimbledon withdrawal</t>
+          <t>Athlon Sports - Indiana Fever Announce Aliyah Boston Injury Update Before LA Sparks Game</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/tennis/articles/emma_raducanu_setback_deepens_as_british_star_remains_on_crutches_after_wimbledon_withdrawal/s1_17460_44037038</t>
+          <t>https://athlonsports.com/wnba/indiana-fever/indiana-fever-announce-aliyah-boston-injury-update-la-sparks-game</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Jordan Henderson</t>
+          <t>Reece James</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>England National Team (2026 FIFA World Cup)</t>
+          <t>Chelsea FC (Premier League) / England National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1889,12 +1889,12 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Wrist fracture sustained in a freak fall while celebrating England's Round of 16 win over Mexico; reportedly requires surgery</t>
+          <t>Hamstring injury sustained in England's final group-stage match vs. Ghana on June 23; described by reporting as worse than first thought</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of the 2026 World Cup; exact surgery date and recovery length not yet specified</t>
+          <t>Touch-and-go for England's July 11 World Cup quarterfinal vs. Norway; has missed England's last three matches and was the sole absentee from the team's final group training session, requiring final medical clearance just to be considered for the bench</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1904,34 +1904,34 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>England advance to the quarterfinals without an experienced veteran midfielder, compounding a growing injury list</t>
+          <t>Compounds an England right-back crisis that worsened after Jarell Quansah's red card vs. Mexico, leaving manager Thomas Tuchel with very limited options at the position for the quarterfinal</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>ESPN - England's Henderson hospitalized with wrist injury during celebration</t>
+          <t>Sky Sports - England World Cup latest: Reece James in race to be fit for quarter-final clash with Norway to ease right-back crisis</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49283507/jordan-henderson-taken-hospital-wrist-injury-falling-mexico-victory-celebrations-england-world-cup</t>
+          <t>https://www.skysports.com/football/news/11095/13561150/england-world-cup-latest-reece-james-in-race-to-be-fit-for-quarter-final-clash-with-norway-to-ease-right-back-crisis</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Santiago Gimenez</t>
+          <t>Aurelien Tchouameni</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>AC Milan (Serie A) / Mexico National Team</t>
+          <t>Real Madrid (La Liga) / France National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1941,12 +1941,12 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Grade II right ankle sprain suffered in stoppage time of Mexico's Round of 16 loss to England; hospitalized, but avoided fracture and ligament damage</t>
+          <t>Muscle tear involving the left adductor and upper thigh, a recurrence of the groin/thigh issue that previously sidelined him for France's group-stage match vs. Iraq</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Not yet specified by club or national team</t>
+          <t>Missed France's Round of 16 win over Paraguay; returned to partial team training on July 8, with a decision on his availability for the July 11 quarterfinal vs. Morocco pending</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1956,49 +1956,49 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Injury compounds Mexico's World Cup elimination and raises concern over his fitness for AC Milan's preseason</t>
+          <t>France's vice-captain and starting defensive midfielder is a doubt for the quarterfinal, with Manu Kone deputizing in his absence</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>beIN Sports - Adding insult to injury! Santiago Gimenez suffers injury during Mexico's loss to England</t>
+          <t>Sportskeeda - France handed huge injury boost as star man returns to training ahead of FIFA World Cup Q/F against Morocco</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>https://www.beinsports.com/en-us/soccer/fifa-world-cup-2026/articles/adding-insult-to-injury-santiago-gimenez-suffers-injury-during-mexico-s-loss-to-england-2026-07-06</t>
+          <t>https://www.sportskeeda.com/football/rumor-france-handed-huge-injury-boost-star-man-returns-training-ahead-fifa-world-cup-q-f-morocco-reports</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Ismael Saibari</t>
+          <t>Mustafizur Rahman</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Bayern Munich (Bundesliga, incoming) / Morocco National Team (2026 FIFA World Cup)</t>
+          <t>Bangladesh National Cricket Team</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury (minor muscle issue per medical tests; serious strain ruled out) suffered in the 22nd minute of Morocco's Round of 16 win over Canada</t>
+          <t>Grade 1 muscle tear in the right hamstring and meniscal degeneration in the right knee, felt while bowling in the first ODI vs. Zimbabwe</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Day-to-day pending fitness test; final decision on availability for the World Cup quarterfinal vs. France expected only hours before kickoff</t>
+          <t>Ruled out for four weeks, covering the remainder of Bangladesh's tour of Zimbabwe (concluding July 19), including the T20I series; has returned home for rehab</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2008,49 +2008,49 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Morocco risks losing their top attacking threat (three group-stage goals) for the biggest match of their World Cup run</t>
+          <t>Bangladesh lose a frontline pace bowler for the rest of the Zimbabwe tour</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>The National - Ismael Saibari fitness concern for Morocco ahead of France World Cup quarter-final clash</t>
+          <t>ESPNcricinfo - Zim vs Ban: Mustafizur Rahman ruled out for four weeks with hamstring and knee injuries</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.thenationalnews.com/sport/world-cup-2026/2026/07/06/ismael-saibari-fitness-concern-for-morocco-ahead-of-france-world-cup-quarter-final-clash/</t>
+          <t>https://www.espncricinfo.com/story/zim-vs-ban-mustafizur-rahman-ruled-out-for-four-weeks-with-hamstring-and-knee-injuries-1545065</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>A'ja Wilson</t>
+          <t>Marco Raya</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Las Vegas Aces (WNBA)</t>
+          <t>Minnesota Twins (MLB)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Foot injury sustained in a game against the Chicago Sky</t>
+          <t>Right shoulder impingement</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Missed 3 games; coach Becky Hammon said she could have played if it were a playoff game, suggesting an imminent return</t>
+          <t>Placed on 15-day IL July 8, retroactive to July 5</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2060,49 +2060,49 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Aces without their All-Star forward/center for a short stretch, including a loss to Indiana</t>
+          <t>Twins lose a pitching option for at least 15 days</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>MLB.com - Latest Twins injuries &amp; transactions</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://www.mlb.com/news/twins-injuries-and-roster-moves</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Caitlin Clark</t>
+          <t>Endy Rodriguez</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Indiana Fever (WNBA)</t>
+          <t>Pittsburgh Pirates (MLB)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Aggravated back injury</t>
+          <t>Left glute strain</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Has resumed practicing; no confirmed timeline yet for a game return</t>
+          <t>Placed on 10-day IL July 8, retroactive to July 6</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2112,49 +2112,49 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Fever have played without their All-Star starting guard for an extended stretch</t>
+          <t>Pirates lose their starting catcher for at least 10 days</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>MLB Trade Rumors - Pirates Place Endy Rodriguez On Injured List</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://www.mlbtraderumors.com/2026/07/pirates-to-place-endy-rodriguez-on-injured-list.html</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Napheesa Collier</t>
+          <t>Taylor Fritz</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Lynx (WNBA)</t>
+          <t>ATP Tour</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Tennis</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Offseason surgery on both ankles</t>
+          <t>Knee tendinitis flare-up, a recurring issue, three games into his Wimbledon quarterfinal</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Has yet to play in the 2026 season; recently resumed practicing</t>
+          <t>Played through the flare-up but lost the quarterfinal 6-4, 6-4, 6-2 to Alexander Zverev; no absence or further tournament withdrawal reported</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2164,49 +2164,49 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Lynx have been without their All-Star forward for the entire season to date</t>
+          <t>Eliminated from Wimbledon; dropped to No. 10 in the ATP Live Rankings</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>ESPN - Taylor Fritz loses at Wimbledon after knee tendinitis flares up</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://www.espn.com/tennis/story/_/id/49308826/taylor-fritz-loses-alexander-zverev-wimbledon-quarterfinals-knee-tendonitis-flares-up</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Byron Buxton</t>
+          <t>Jalen Brunson</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Twins (MLB)</t>
+          <t>New York Knicks (NBA)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Aggravated hip injury while being caught stealing in the 1st inning vs. Yankees</t>
+          <t>Surgery to repair a left wrist injury that he played through during the Knicks' championship playoff run</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Day-to-day; had already missed 4 games earlier in the week with the same hip issue</t>
+          <t>At least two months of rehab expected; targeting readiness for the start of the 2026-27 NBA season</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2216,49 +2216,49 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Twins lose their 2026 All-Star outfielder from the lineup for an undetermined stretch</t>
+          <t>Reigning Finals MVP and starting point guard sidelined for part of the offseason program, though expected back for training camp</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>Yahoo Sports - Knicks superstar Jalen Brunson undergoes left wrist surgery, expected to be ready for 2026-27 NBA season</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://sports.yahoo.com/nba/breaking-news/article/knicks-superstar-jalen-brunson-undergoes-left-wrist-surgery-expected-to-be-ready-for-2026-27-nba-season-155927234.html</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Jazz Chisholm Jr.</t>
+          <t>Amadou Onana</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>New York Yankees (MLB)</t>
+          <t>Aston Villa (Premier League) / Belgium National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Right toe discomfort, noticed jogging gingerly to first base after a fly out</t>
+          <t>Torn anterior cruciate ligament (ACL), sustained in the 21st minute of Belgium's Round of 16 win over the United States after a challenge with Christian Pulisic</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Being monitored day-to-day; no IL move confirmed yet</t>
+          <t>Ruled out for the remainder of the World Cup; reported to be facing up to eight months out</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2268,34 +2268,34 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Risk of losing Yankees' starting second baseman if it worsens</t>
+          <t>Belgium loses a key defensive midfielder ahead of their World Cup quarterfinal vs. Spain, and Aston Villa will be without him for a significant part of the 2026-27 season</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>ESPN - Belgium's Amadou Onana out of World Cup after suffering ACL injury</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.espn.com/soccer/story/_/id/49298508/belgium-amadou-onana-world-cup-suffering-acl-injury</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Ranger Suarez</t>
+          <t>Giancarlo Stanton</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies (MLB)</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2305,12 +2305,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Left adductor tightness, pulled early from start vs. Angels</t>
+          <t>Right calf strain (originally suffered running the bases on April 24 vs. the Astros); recent rehab setback after re-aggravating the calf during a running progression</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Undetermined, pending further evaluation</t>
+          <t>No firm timeline; has not resumed running since the setback, no target return date given</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2320,101 +2320,101 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Phillies could lose their 2026 AL All-Star-caliber starter from the rotation</t>
+          <t>Yankees continue without their veteran slugger amid an offense that has struggled with injuries; manager Aaron Boone still expects him back at some point in 2026</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>Last Word on Sports - Stanton Injury Update: Slugger Yet To Resume Rehab On Calf</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://lastwordonsports.com/baseball/2026/07/07/nyy-stanton-injury-update/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Brandon Woodruff</t>
+          <t>Matteo Berrettini</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers (MLB)</t>
+          <t>ATP Tour</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Tennis</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Right shoulder inflammation</t>
+          <t>Diagnosed with chronic hip pain, a recurrence of the left hip issue that forced his retirement from his Roland Garros quarterfinal in early June</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Placed on 15-day Injured List (minimum)</t>
+          <t>Withdrawing from the ATP tournaments in Gstaad and Kitzbuhel to rest on medical advice, with the goal of being ready for the US hard-court swing culminating in the US Open; no firm return date given</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Forfeits ranking points and prize money from both the Gstaad and Kitzbuhel events</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Brewers rotation loses a top starter for at least two full turns</t>
+          <t>Removes him from the draw at both tournaments immediately following his third-round Wimbledon loss to Grigor Dimitrov</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Covers - MLB Injuries 2026</t>
+          <t>Puntodebreak - Berrettini withdraws from competing in upcoming tournaments due to "chronic hip pain"</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>https://www.covers.com/sport/baseball/mlb/injuries</t>
+          <t>https://www.puntodebreak.com/en/2026/07/07/berrettini-withdraws-from-competing-in-upcoming-tournaments-due-to-chronic-hip-pain</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Triston Casas</t>
+          <t>Skylar Diggins</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Boston Red Sox (MLB)</t>
+          <t>Chicago Sky (WNBA)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Torn right patellar tendon (out since May); recently shut down from hitting progression</t>
+          <t>Right knee injury; Diggins has said a knee surgery from last October has contributed to ongoing strain</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Likely season-ending; setback in rehab timeline</t>
+          <t>Ruled out for the July 7 game vs. Phoenix Mercury; no return timeline given</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2424,138 +2424,138 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Red Sox lose starting first baseman for the remainder of the 2026 season</t>
+          <t>Comes as Diggins was moved to the bench for the first time in a decade, ending a streak of 341 consecutive starts; Sky beat Phoenix 77-66 in her absence</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>Yahoo Sports - Sky's Skylar Diggins ruled out (knee) after being benched, Vandersloot starting</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://sports.yahoo.com/articles/skys-skylar-diggins-ruled-vs-010259203.html</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>James Maddison</t>
+          <t>Emma Raducanu</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Tottenham Hotspur (Premier League)</t>
+          <t>WTA Tour</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Tennis</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>ACL reconstruction rehab (returning from tear)</t>
+          <t>Stress fracture in lower right leg (ankle area); withdrew hours before her scheduled first-round match</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Ongoing; currently restricted to 20-25 minutes per match</t>
+          <t>Ruled out of Wimbledon 2026; still on crutches and wearing a protective boot several days after withdrawal, no return timeline given</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Loses out on Wimbledon prize money and ranking points for the event</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Spurs managing his minutes carefully, limiting his impact as a starter</t>
+          <t>Removes a top British draw from the tournament</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>Yardbarker - Emma Raducanu setback deepens as British star remains on crutches after Wimbledon withdrawal</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.yardbarker.com/tennis/articles/emma_raducanu_setback_deepens_as_british_star_remains_on_crutches_after_wimbledon_withdrawal/s1_17460_44037038</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Seamus Power</t>
+          <t>Jordan Henderson</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>PGA Tour</t>
+          <t>England National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Golf</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Recurrence of long-standing back and hip issues he has dealt with since 2023</t>
+          <t>Wrist fracture sustained in a freak fall while celebrating England's Round of 16 win over Mexico; reportedly requires surgery</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Withdrew after an opening-round 6-over 77 at the John Deere Classic on July 2; no return timeline given</t>
+          <t>Ruled out for the remainder of the 2026 World Cup; exact surgery date and recovery length not yet specified</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Forfeits prize money and FedEx Cup points from the John Deere Classic</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Removes a two-time PGA Tour winner from the field partway through the event</t>
+          <t>England advance to the quarterfinals without an experienced veteran midfielder, compounding a growing injury list</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Golfmagic - Two-time PGA Tour winner forced out of John Deere Classic as injury problems strike again</t>
+          <t>ESPN - England's Henderson hospitalized with wrist injury during celebration</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.golfmagic.com/tour/pga-tour/two-time-pga-tour-winner-forced-out-john-deere-classic-injury-problems-strike-again</t>
+          <t>https://www.espn.com/soccer/story/_/id/49283507/jordan-henderson-taken-hospital-wrist-injury-falling-mexico-victory-celebrations-england-world-cup</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Nahikari Garcia</t>
+          <t>Santiago Gimenez</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Denver Summit FC (NWSL)</t>
+          <t>AC Milan (Serie A) / Mexico National Team</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2565,12 +2565,12 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Season-ending knee (ACL) injury</t>
+          <t>Grade II right ankle sprain suffered in stoppage time of Mexico's Round of 16 loss to England; hospitalized, but avoided fracture and ligament damage</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Out for the remainder of the 2026 NWSL season</t>
+          <t>Not yet specified by club or national team</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2580,49 +2580,49 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Denver Summit FC lose a starter for the rest of the season</t>
+          <t>Injury compounds Mexico's World Cup elimination and raises concern over his fitness for AC Milan's preseason</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Spotrac - 2026 NWSL Injured Tracker</t>
+          <t>beIN Sports - Adding insult to injury! Santiago Gimenez suffers injury during Mexico's loss to England</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
+          <t>https://www.beinsports.com/en-us/soccer/fifa-world-cup-2026/articles/adding-insult-to-injury-santiago-gimenez-suffers-injury-during-mexico-s-loss-to-england-2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Brandon Ingram</t>
+          <t>Ismael Saibari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Toronto Raptors (NBA)</t>
+          <t>Bayern Munich (Bundesliga, incoming) / Morocco National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Recovering from offseason surgery (lower body)</t>
+          <t>Hamstring injury (minor muscle issue per medical tests; serious strain ruled out) suffered in the 22nd minute of Morocco's Round of 16 win over Canada</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Expected back for training camp, fall 2026</t>
+          <t>Day-to-day pending fitness test; final decision on availability for the World Cup quarterfinal vs. France expected only hours before kickoff</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2632,34 +2632,34 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Raptors plan around his absence through the offseason program</t>
+          <t>Morocco risks losing their top attacking threat (three group-stage goals) for the biggest match of their World Cup run</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Brandon Ingram Injury Update Provided by Raptors After Surgery</t>
+          <t>The National - Ismael Saibari fitness concern for Morocco ahead of France World Cup quarter-final clash</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25426220-brandon-ingram-injury-update-provided-raptors-after-surgery-latest-timeline-2026-nba-season</t>
+          <t>https://www.thenationalnews.com/sport/world-cup-2026/2026/07/06/ismael-saibari-fitness-concern-for-morocco-ahead-of-france-world-cup-quarter-final-clash/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Josh Giddey</t>
+          <t>A'ja Wilson</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Chicago Bulls (NBA)</t>
+          <t>Las Vegas Aces (WNBA)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2669,12 +2669,12 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Arthroscopic surgery on right ankle</t>
+          <t>Foot injury sustained in a game against the Chicago Sky</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>~3 months to resume basketball activities; targeting training camp</t>
+          <t>Missed 3 games; coach Becky Hammon said she could have played if it were a playoff game, suggesting an imminent return</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2684,49 +2684,49 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Bulls lose a starting guard for the entire offseason program</t>
+          <t>Aces without their All-Star forward/center for a short stretch, including a loss to Indiana</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Josh Giddey Injury Update Provided by Bulls After Ankle Surgery</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25427505-josh-giddey-injury-update-provided-bulls-after-ankle-surgery-latest-timeline-2026-nba-season</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Corey Seager</t>
+          <t>Caitlin Clark</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Texas Rangers (MLB)</t>
+          <t>Indiana Fever (WNBA)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Recurrence of lower back inflammation; his third injured list stint of the 2026 season (previously missed time with the same back issue and with a concussion)</t>
+          <t>Aggravated back injury</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Placed on the 10-day injured list</t>
+          <t>Has resumed practicing; no confirmed timeline yet for a game return</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2736,49 +2736,49 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Rangers lose their star shortstop again, continuing a season of infield instability; Josh Smith recalled from Triple-A as replacement</t>
+          <t>Fever have played without their All-Star starting guard for an extended stretch</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Rangers' Corey Seager back on IL with lower back inflammation</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49238350/rangers-corey-seager-back-il-lower-back-inflammation</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Brent Rooker</t>
+          <t>Napheesa Collier</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Athletics (MLB)</t>
+          <t>Minnesota Lynx (WNBA)</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Cartilage tear in left knee, discovered during an examination at Stanford; requires season-ending surgery</t>
+          <t>Offseason surgery on both ankles</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Season-ending; hadn't played since June 8 and had been on the injured list since June 9</t>
+          <t>Has yet to play in the 2026 season; recently resumed practicing</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2788,49 +2788,49 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Athletics lose their two-time All-Star middle-of-the-order bat for the remainder of the 2026 season</t>
+          <t>Lynx have been without their All-Star forward for the entire season to date</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>ESPN - A's slugger Brent Rooker to have season-ending left knee surgery</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49244022/a-slugger-brent-rooker-season-ending-left-knee-surgery</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>JuJu Watkins</t>
+          <t>Lexi Thompson</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>USC Trojans (NCAA Division I Women's Basketball)</t>
+          <t>LPGA Tour</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Golf</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Recovering from a torn ACL that cost her the entire 2025-26 season</t>
+          <t>Persistent hip pain/suspected hip injury</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Returned to the court roughly 14 months after the injury</t>
+          <t>Withdrew from the KPMG Women's PGA Championship at Hazeltine National, after also sitting out the Meijer LPGA Classic with the same issue; no return timeline given</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2840,49 +2840,49 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>USC gets back its star guard after a full season lost to the injury</t>
+          <t>Ends a 15-tournament appearance streak at the Women's PGA Championship, a run that included four career top-10 finishes; Carolina Chacarra took her place in the field</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Fox Sports - 2026-2027 College Basketball Offseason Buzz</t>
+          <t>Golf Digest - Lexi Thompson withdraws from KPMG Women's PGA Championship</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.foxsports.com/stories/college-basketball/college-basketball-2026-2027-buzz-news-injuries-transfers</t>
+          <t>https://www.golfdigest.com/story/lexi-thompson-withdraws-kpmg-womens-pga-championship</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Jaren Jackson Jr.</t>
+          <t>Byron Buxton</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Memphis Grizzlies (NBA)</t>
+          <t>Minnesota Twins (MLB)</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Turf toe surgery (right foot)</t>
+          <t>Aggravated hip injury while being caught stealing in the 1st inning vs. Yankees</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Re-evaluation in approximately 12 weeks</t>
+          <t>Day-to-day; had already missed 4 games earlier in the week with the same hip issue</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2892,49 +2892,49 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Grizzlies lose their All-Star big man through the offseason and possibly into training camp</t>
+          <t>Twins lose their 2026 All-Star outfielder from the lineup for an undetermined stretch</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>NBA.com - Grizzlies' Jaren Jackson Jr. has surgery to repair turf toe injury</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>https://www.nba.com/news/memphis-grizzlies-jaren-jackson-jr-turf-toe-surgery</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Manuel Ugarte</t>
+          <t>Jazz Chisholm Jr.</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Manchester United (Premier League) / Uruguay National Team</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Knee ligament injury suffered vs. Spain at the World Cup; possible cruciate ligament (ACL) damage</t>
+          <t>Right toe discomfort, noticed jogging gingerly to first base after a fly out</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Potentially several months if ACL is confirmed</t>
+          <t>Being monitored day-to-day; no IL move confirmed yet</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2944,49 +2944,49 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Would be a significant blow to Manchester United's midfield depth heading into 2026-27</t>
+          <t>Risk of losing Yankees' starting second baseman if it worsens</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Rodri</t>
+          <t>Ranger Suarez</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Manchester City (Premier League)</t>
+          <t>Philadelphia Phillies (MLB)</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Undisclosed injury expected to require surgery after the World Cup</t>
+          <t>Left adductor tightness, pulled early from start vs. Angels</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Out for the opening weeks of the 2026-27 season</t>
+          <t>Undetermined, pending further evaluation</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2996,49 +2996,49 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Manchester City to start the new season without their midfield anchor</t>
+          <t>Phillies could lose their 2026 AL All-Star-caliber starter from the rotation</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Kelsey Plum</t>
+          <t>Brandon Woodruff</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks (WNBA)</t>
+          <t>Milwaukee Brewers (MLB)</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Lower leg injury</t>
+          <t>Right shoulder inflammation</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for at least 4 weeks as of late June; All-Star Game (July 25) status still to be decided</t>
+          <t>Placed on 15-day Injured List (minimum)</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3048,49 +3048,49 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Sparks lose a starting guard through their All-Star break stretch</t>
+          <t>Brewers rotation loses a top starter for at least two full turns</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Angel Reese, Kelsey Plum Headline 2026 WNBA All-Star Game Reserves</t>
+          <t>Covers - MLB Injuries 2026</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25452286-angel-reese-kelsey-plum-headline-2026-wnba-all-star-game-reserves-full-roster-announced</t>
+          <t>https://www.covers.com/sport/baseball/mlb/injuries</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Seth Jarvis</t>
+          <t>Triston Casas</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Carolina Hurricanes (NHL)</t>
+          <t>Boston Red Sox (MLB)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Hockey</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Shoulder surgery, the same shoulder that had a torn labrum and rotator cuff during the 2023-24 season</t>
+          <t>Torn right patellar tendon (out since May); recently shut down from hitting progression</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Expected recovery of approximately 4-6 months, meaning the earliest return would be late October</t>
+          <t>Likely season-ending; setback in rehab timeline</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3100,34 +3100,34 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Hurricanes will be without a top-six forward for the start of the 2026-27 season</t>
+          <t>Red Sox lose starting first baseman for the remainder of the 2026 season</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>NHL.com - Jarvis expected to miss start of next season for Hurricanes after shoulder surgery</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>https://www.nhl.com/news/seth-jarvis-to-miss-beginning-of-2026-2027-season-for-hurricanes-after-shoulder-surgery</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Bradley Beal</t>
+          <t>Olivia Miles</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>LA Clippers (NBA)</t>
+          <t>Minnesota Lynx (WNBA)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3137,12 +3137,12 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Hip fracture requiring season-ending surgery</t>
+          <t>Calf strain suffered during a July 3 game vs. the New York Liberty, possibly linked to in-game cramping</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Season-ending; recovery expected to extend into 2026-27 preseason</t>
+          <t>Ruled out of the Lynx's game vs. Connecticut on July 6, the first game of her WNBA career she has missed; no firm timetable given, though signs point to a quick recovery</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3152,29 +3152,29 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Clippers lose a veteran guard for the balance of the season and into next year's planning</t>
+          <t>Costly absence for a Lynx team leaning on its rookie floor general; came a day after Miles was named a starter for the 2026 WNBA All-Star Game and while she remains a near-lock for Rookie of the Year (18.5 ppg, 4.8 rpg, 5.7 apg)</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>NBA.com - Clippers' Bradley Beal (hip) to undergo season-ending surgery</t>
+          <t>ESPN - Olivia Miles sidelined Monday against Sun with calf injury</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://www.nba.com/news/clippers-bradley-beal-out-season-hip-fracture</t>
+          <t>https://www.espn.com/wnba/story/_/id/49287945/olivia-miles-sidelined-monday-sun-calf-injury</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Bejlek</t>
+          <t>Serena Williams</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -3189,49 +3189,49 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Elbow injury</t>
+          <t>Right knee injury tweaked at the end of the first set of her Wimbledon singles match against Maya Joint; postmatch video showed four syringes of fluid drained from the knee</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Withdrew mid-tournament from Eastbourne</t>
+          <t>Withdrew from the Wimbledon doubles draw alongside sister Venus Williams; no return timeline given</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Forfeits Eastbourne prize money/points from the round of withdrawal</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Opponent Zeynep Sonmez advances by walkover</t>
+          <t>Ends a highly anticipated comeback pairing with Venus Williams in doubles, coming during Serena's first singles match in nearly four years</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>RotoWire - Fantasy Tennis Injury News</t>
+          <t>NBC News - Serena Williams withdraws from Wimbledon doubles competition after knee injury</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+          <t>https://www.nbcnews.com/sports/tennis/serena-williams-withdraws-wimbledon-rcna352965</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Matthijs de Ligt</t>
+          <t>James Maddison</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Manchester United (Premier League)</t>
+          <t>Tottenham Hotspur (Premier League)</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3241,12 +3241,12 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Surgery on a long-standing back injury</t>
+          <t>ACL reconstruction rehab (returning from tear)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Will miss the 2026 World Cup; club return timeline unconfirmed</t>
+          <t>Ongoing; currently restricted to 20-25 minutes per match</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3256,12 +3256,12 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>United lose a starting center-back for an extended stretch</t>
+          <t>Spurs managing his minutes carefully, limiting his impact as a starter</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -3278,64 +3278,64 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Elina Svitolina</t>
+          <t>Seamus Power</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>PGA Tour</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Golf</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Hip injury</t>
+          <t>Recurrence of long-standing back and hip issues he has dealt with since 2023</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Withdrew before her Bad Homburg quarterfinal</t>
+          <t>Withdrew after an opening-round 6-over 77 at the John Deere Classic on July 2; no return timeline given</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Forfeits Bad Homburg quarterfinal prize money/points</t>
+          <t>Forfeits prize money and FedEx Cup points from the John Deere Classic</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Opponent Xinyu Wang advances by walkover</t>
+          <t>Removes a two-time PGA Tour winner from the field partway through the event</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>RotoWire - Fantasy Tennis Injury News</t>
+          <t>Golfmagic - Two-time PGA Tour winner forced out of John Deere Classic as injury problems strike again</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+          <t>https://www.golfmagic.com/tour/pga-tour/two-time-pga-tour-winner-forced-out-john-deere-classic-injury-problems-strike-again</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Chris Richards</t>
+          <t>Nahikari Garcia</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Crystal Palace (Premier League) / USMNT</t>
+          <t>Denver Summit FC (NWSL)</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3345,12 +3345,12 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Torn ankle ligaments (two ligaments) suffered vs. Brentford</t>
+          <t>Season-ending knee (ACL) injury</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Expected to recover in time for the 2026 World Cup</t>
+          <t>Out for the remainder of the 2026 NWSL season</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3360,72 +3360,904 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Crystal Palace lose a starting center-back for a multi-week stretch</t>
+          <t>Denver Summit FC lose a starter for the rest of the season</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>Spotrac - 2026 NWSL Injured Tracker</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
+          <t>Brandon Ingram</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Toronto Raptors (NBA)</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Basketball</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Recovering from offseason surgery (lower body)</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Expected back for training camp, fall 2026</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Raptors plan around his absence through the offseason program</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Bleacher Report - Brandon Ingram Injury Update Provided by Raptors After Surgery</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>https://bleacherreport.com/articles/25426220-brandon-ingram-injury-update-provided-raptors-after-surgery-latest-timeline-2026-nba-season</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Josh Giddey</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Chicago Bulls (NBA)</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Basketball</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Arthroscopic surgery on right ankle</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>~3 months to resume basketball activities; targeting training camp</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Bulls lose a starting guard for the entire offseason program</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Bleacher Report - Josh Giddey Injury Update Provided by Bulls After Ankle Surgery</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>https://bleacherreport.com/articles/25427505-josh-giddey-injury-update-provided-bulls-after-ankle-surgery-latest-timeline-2026-nba-season</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Corey Seager</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Texas Rangers (MLB)</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Baseball</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Recurrence of lower back inflammation; his third injured list stint of the 2026 season (previously missed time with the same back issue and with a concussion)</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Placed on the 10-day injured list</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Rangers lose their star shortstop again, continuing a season of infield instability; Josh Smith recalled from Triple-A as replacement</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>ESPN - Rangers' Corey Seager back on IL with lower back inflammation</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.espn.com/mlb/story/_/id/49238350/rangers-corey-seager-back-il-lower-back-inflammation</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Brent Rooker</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Athletics (MLB)</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Baseball</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Cartilage tear in left knee, discovered during an examination at Stanford; requires season-ending surgery</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Season-ending; hadn't played since June 8 and had been on the injured list since June 9</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Athletics lose their two-time All-Star middle-of-the-order bat for the remainder of the 2026 season</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>ESPN - A's slugger Brent Rooker to have season-ending left knee surgery</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.espn.com/mlb/story/_/id/49244022/a-slugger-brent-rooker-season-ending-left-knee-surgery</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>JuJu Watkins</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>USC Trojans (NCAA Division I Women's Basketball)</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Basketball</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Recovering from a torn ACL that cost her the entire 2025-26 season</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Returned to the court roughly 14 months after the injury</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>USC gets back its star guard after a full season lost to the injury</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Fox Sports - 2026-2027 College Basketball Offseason Buzz</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.foxsports.com/stories/college-basketball/college-basketball-2026-2027-buzz-news-injuries-transfers</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Donnie Freeman</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>St. John's University (NCAA Division I Men's Basketball)</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Basketball</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Torn right Achilles tendon, a non-contact injury suffered during a summer workout; underwent successful surgery performed by Dr. Martin O'Malley</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Will miss the entire 2026-27 season</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Major setback for coach Rick Pitino and St. John's, who added the rising junior forward as a transfer-portal pickup this offseason; Freeman averaged 16.5 points and 7.2 rebounds last season at Syracuse</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>The Washington Post - St. John's Donnie Freeman to miss next season following surgery on Achilles tendon</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.washingtonpost.com/sports/colleges/2026/07/01/st-johns-donnie-freeman-achilles-injury-pitino/81e54c60-75c4-11f1-b665-5f8be87f3787_story.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Jaren Jackson Jr.</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Memphis Grizzlies (NBA)</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Basketball</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Turf toe surgery (right foot)</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Re-evaluation in approximately 12 weeks</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Grizzlies lose their All-Star big man through the offseason and possibly into training camp</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>NBA.com - Grizzlies' Jaren Jackson Jr. has surgery to repair turf toe injury</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nba.com/news/memphis-grizzlies-jaren-jackson-jr-turf-toe-surgery</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Manuel Ugarte</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Manchester United (Premier League) / Uruguay National Team</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Soccer</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Knee ligament injury suffered vs. Spain at the World Cup; possible cruciate ligament (ACL) damage</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Potentially several months if ACL is confirmed</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Would be a significant blow to Manchester United's midfield depth heading into 2026-27</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Premier League club injury coverage</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Rodri</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Manchester City (Premier League)</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Soccer</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Undisclosed injury expected to require surgery after the World Cup</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Out for the opening weeks of the 2026-27 season</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Manchester City to start the new season without their midfield anchor</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Premier League club injury coverage</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Kelsey Plum</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks (WNBA)</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Basketball</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Lower leg injury</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Ruled out for at least 4 weeks as of late June; All-Star Game (July 25) status still to be decided</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Sparks lose a starting guard through their All-Star break stretch</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>Bleacher Report - Angel Reese, Kelsey Plum Headline 2026 WNBA All-Star Game Reserves</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>https://bleacherreport.com/articles/25452286-angel-reese-kelsey-plum-headline-2026-wnba-all-star-game-reserves-full-roster-announced</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Seth Jarvis</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Carolina Hurricanes (NHL)</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Hockey</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Shoulder surgery, the same shoulder that had a torn labrum and rotator cuff during the 2023-24 season</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Expected recovery of approximately 4-6 months, meaning the earliest return would be late October</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Hurricanes will be without a top-six forward for the start of the 2026-27 season</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>NHL.com - Jarvis expected to miss start of next season for Hurricanes after shoulder surgery</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nhl.com/news/seth-jarvis-to-miss-beginning-of-2026-2027-season-for-hurricanes-after-shoulder-surgery</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Bradley Beal</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>LA Clippers (NBA)</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Basketball</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Hip fracture requiring season-ending surgery</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Season-ending; recovery expected to extend into 2026-27 preseason</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Clippers lose a veteran guard for the balance of the season and into next year's planning</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>NBA.com - Clippers' Bradley Beal (hip) to undergo season-ending surgery</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nba.com/news/clippers-bradley-beal-out-season-hip-fracture</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Bejlek</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>WTA Tour</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Elbow injury</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Withdrew mid-tournament from Eastbourne</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Forfeits Eastbourne prize money/points from the round of withdrawal</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Opponent Zeynep Sonmez advances by walkover</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>RotoWire - Fantasy Tennis Injury News</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Matthijs de Ligt</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Manchester United (Premier League)</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Soccer</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Surgery on a long-standing back injury</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Will miss the 2026 World Cup; club return timeline unconfirmed</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>United lose a starting center-back for an extended stretch</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>Premier League club injury coverage</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Elina Svitolina</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>WTA Tour</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Hip injury</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Withdrew before her Bad Homburg quarterfinal</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Forfeits Bad Homburg quarterfinal prize money/points</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Opponent Xinyu Wang advances by walkover</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>RotoWire - Fantasy Tennis Injury News</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Chris Richards</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Crystal Palace (Premier League) / USMNT</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Soccer</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Torn ankle ligaments (two ligaments) suffered vs. Brentford</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Expected to recover in time for the 2026 World Cup</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Crystal Palace lose a starting center-back for a multi-week stretch</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>Premier League club injury coverage</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
           <t>Chloe Ricketts</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>Boston Legacy FC (NWSL)</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>Soccer</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>Ankle injury</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Placed on the 45-day short-term injury list</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>Not disclosed in available reporting</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
         <is>
           <t>Boston Legacy FC without a rostered defender for at least 45 days</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr">
+      <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Washington Spirit / NWSL transactions coverage</t>
         </is>
       </c>
-      <c r="J57" s="2" t="inlineStr">
+      <c r="J73" s="2" t="inlineStr">
         <is>
           <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
         </is>
@@ -3489,10 +4321,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId72"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId57"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId73"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Daily injury update: McGregor, Magbegor, Griffin, Bell, Smylie
</commit_message>
<xml_diff>
--- a/injury_report.xlsx
+++ b/injury_report.xlsx
@@ -145,8 +145,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Injuries" displayName="Injuries" ref="A1:J73" headerRowCount="1">
-  <autoFilter ref="A1:J73"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Injuries" displayName="Injuries" ref="A1:J78" headerRowCount="1">
+  <autoFilter ref="A1:J78"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Athlete"/>
     <tableColumn id="2" name="Organization"/>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -522,12 +522,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Satou Sabally</t>
+          <t>Kierstan Bell</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>New York Liberty (WNBA)</t>
+          <t>Las Vegas Aces (WNBA)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -537,12 +537,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Concussion protocol after being elbowed in the face by Aces forward NaLyssa Smith while contesting a rebound; symptoms had delayed onset</t>
+          <t>Right leg injury (specific diagnosis not disclosed in available reporting)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Downgraded from questionable to out; remains in concussion protocol with no return timeline given</t>
+          <t>Ruled out for the Aces' July 13 game vs. the Indiana Fever; no return timeline given</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -552,34 +552,34 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Liberty without their All-Star forward for multiple games as she works through the NBA/WNBA-mandated concussion protocol; notable given she also missed time with a concussion in the 2025 WNBA Finals</t>
+          <t>Aces without a rotation forward who had recently moved into the starting lineup, adding to the team's list of unavailable players</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports - Liberty injury report: Star forward Satou Sabally in concussion protocol</t>
+          <t>Yahoo Sports - Final Injury Report for Fever-Aces: Will Caitlin Clark Play?</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/articles/liberty-injury-report-star-forward-satou-sabally-in-concussion-protocol-224647068.html</t>
+          <t>https://sports.yahoo.com/articles/final-injury-report-fever-aces-210000827.html</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Angel Reese</t>
+          <t>Satou Sabally</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Atlanta Dream (WNBA)</t>
+          <t>New York Liberty (WNBA)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Lower leg/ankle injury sustained falling under the basket late in a win over the Seattle Storm</t>
+          <t>Concussion protocol after being elbowed in the face by Aces forward NaLyssa Smith while contesting a rebound; symptoms had delayed onset</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Listed questionable for the Dream's game vs. the Portland Fire; no firm return timeline given</t>
+          <t>Downgraded from questionable to out; remains in concussion protocol with no return timeline given</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Puts a third-straight All-Star selection and Dream's first year with Reese (acquired in an offseason trade from Chicago) at risk of interruption during a stretch where the team is trying to build momentum after a five-game losing streak</t>
+          <t>Liberty without their All-Star forward for multiple games as she works through the NBA/WNBA-mandated concussion protocol; notable given she also missed time with a concussion in the 2025 WNBA Finals</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -614,19 +614,19 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>CBS Sports - Portland Fire vs. Atlanta Dream preview: Dream seek momentum as Angel Reese is questionable with leg injury</t>
+          <t>Yahoo Sports - Liberty injury report: Star forward Satou Sabally in concussion protocol</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>https://www.cbssports.com/wnba/news/portland-fire-atlanta-dream-where-to-watch-angel-reese-injury/</t>
+          <t>https://sports.yahoo.com/articles/liberty-injury-report-star-forward-satou-sabally-in-concussion-protocol-224647068.html</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Brionna Jones</t>
+          <t>Angel Reese</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -641,12 +641,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Meniscus tear in the right knee suffered in late January while playing overseas for USK Prague; underwent knee surgery at Emory Hospital</t>
+          <t>Lower leg/ankle injury sustained falling under the basket late in a win over the Seattle Storm</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Ruled out to begin the 2026 season and remains sidelined into mid-July; not yet cleared for 5-on-5 drills and has no firm return timetable, though the team says she is expected to make a full recovery</t>
+          <t>Listed questionable for the Dream's game vs. the Portland Fire; no firm return timeline given</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Four-time All-Star center has yet to play a game for the Dream this season, a significant frontcourt loss to start the year</t>
+          <t>Puts a third-straight All-Star selection and Dream's first year with Reese (acquired in an offseason trade from Chicago) at risk of interruption during a stretch where the team is trying to build momentum after a five-game losing streak</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -666,24 +666,24 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>CBS News Atlanta - Atlanta Dream's Brionna Jones nearing return, expected back with team soon</t>
+          <t>CBS Sports - Portland Fire vs. Atlanta Dream preview: Dream seek momentum as Angel Reese is questionable with leg injury</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>https://www.cbsnews.com/atlanta/news/atlanta-dreams-brionna-jones-nearing-return-expected-back-with-team-next-week/</t>
+          <t>https://www.cbssports.com/wnba/news/portland-fire-atlanta-dream-where-to-watch-angel-reese-injury/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Leonie Fiebich</t>
+          <t>Brionna Jones</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>New York Liberty (WNBA)</t>
+          <t>Atlanta Dream (WNBA)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -693,12 +693,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Left foot soreness</t>
+          <t>Meniscus tear in the right knee suffered in late January while playing overseas for USK Prague; underwent knee surgery at Emory Hospital</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for a second straight game, having missed her first game since May 25; no return timeline given</t>
+          <t>Ruled out to begin the 2026 season and remains sidelined into mid-July; not yet cleared for 5-on-5 drills and has no firm return timetable, though the team says she is expected to make a full recovery</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Liberty forward sidelined for consecutive games amid a compressed schedule that includes a quick turnaround for a game in Toronto</t>
+          <t>Four-time All-Star center has yet to play a game for the Dream this season, a significant frontcourt loss to start the year</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -718,39 +718,39 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports - Final Injury Report for Liberty-Mystics: Will Satou Sabally, Leonie Fiebich Play?</t>
+          <t>CBS News Atlanta - Atlanta Dream's Brionna Jones nearing return, expected back with team soon</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/articles/final-injury-report-liberty-mystics-150000047.html</t>
+          <t>https://www.cbsnews.com/atlanta/news/atlanta-dreams-brionna-jones-nearing-return-expected-back-with-team-next-week/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Johan Manzambi</t>
+          <t>Leonie Fiebich</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Switzerland National Team (2026 FIFA World Cup)</t>
+          <t>New York Liberty (WNBA)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Left-knee injury suffered in training on the eve of the Round of 16 match vs. Colombia</t>
+          <t>Left foot soreness</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Missed the Round of 16 win over Colombia and ruled out of the quarterfinal vs. Argentina; no return timeline given</t>
+          <t>Ruled out for a second straight game, having missed her first game since May 25; no return timeline given</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Major blow to Switzerland's attack: with Manzambi on the pitch during the group stage the team averaged 3.6 goals per 90 minutes (3 goals, 2 assists for him in 200 minutes); without him, Switzerland have scored just once and averaged 1.4 xG per 90 over 280 minutes</t>
+          <t>Liberty forward sidelined for consecutive games amid a compressed schedule that includes a quick turnaround for a game in Toronto</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -770,24 +770,24 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Switzerland's Johan Manzambi to miss Argentina World Cup quarterfinal clash - Murat Yakin</t>
+          <t>Yahoo Sports - Final Injury Report for Liberty-Mystics: Will Satou Sabally, Leonie Fiebich Play?</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49326340/switzerland-johan-manzambi-miss-argentina-world-cup-quarterfinal-clash-murat-yakin</t>
+          <t>https://sports.yahoo.com/articles/final-injury-report-liberty-mystics-150000047.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Marc Guehi</t>
+          <t>Johan Manzambi</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>England National Team (2026 FIFA World Cup)</t>
+          <t>Switzerland National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Hamstring strain picked up in England's Round of 16 win over Mexico</t>
+          <t>Left-knee injury suffered in training on the eve of the Round of 16 match vs. Colombia</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Missed a training session in Kansas City but returned to training Friday and was confirmed available for the quarterfinal vs. Norway</t>
+          <t>Missed the Round of 16 win over Colombia and ruled out of the quarterfinal vs. Argentina; no return timeline given</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Created a late fitness scare for England's back line ahead of the quarterfinal, with Newcastle's Dan Burn on standby to deputize had Guehi been unavailable</t>
+          <t>Major blow to Switzerland's attack: with Manzambi on the pitch during the group stage the team averaged 3.6 goals per 90 minutes (3 goals, 2 assists for him in 200 minutes); without him, Switzerland have scored just once and averaged 1.4 xG per 90 over 280 minutes</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -822,39 +822,39 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Sky Sports - World Cup 2026: England defender Marc Guehi a serious doubt for quarter-final clash with Norway</t>
+          <t>ESPN - Switzerland's Johan Manzambi to miss Argentina World Cup quarterfinal clash - Murat Yakin</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>https://www.skysports.com/football/news/12016/13562168/world-cup-2026-england-defender-marc-guehi-a-serious-doubt-for-quarter-final-clash-with-norway</t>
+          <t>https://www.espn.com/soccer/story/_/id/49326340/switzerland-johan-manzambi-miss-argentina-world-cup-quarterfinal-clash-murat-yakin</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Nick Kurtz</t>
+          <t>Marc Guehi</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Athletics (MLB)</t>
+          <t>England National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Right thumb capsule sprain</t>
+          <t>Hamstring strain picked up in England's Round of 16 win over Mexico</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Placed on the 10-day injured list, retroactive to July 10</t>
+          <t>Missed a training session in Kansas City but returned to training Friday and was confirmed available for the quarterfinal vs. Norway</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Keeps the 2025 AL Rookie of the Year and scheduled AL All-Star starting first baseman (.266, 20 HR, 66 RBI, MLB-leading 76 walks) out of the July 14 All-Star Game in Philadelphia; catcher Brian Serven recalled from Triple-A in a corresponding move</t>
+          <t>Created a late fitness scare for England's back line ahead of the quarterfinal, with Newcastle's Dan Burn on standby to deputize had Guehi been unavailable</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -874,24 +874,24 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Athletics All-Star 1B Nick Kurtz placed on IL with thumb sprain</t>
+          <t>Sky Sports - World Cup 2026: England defender Marc Guehi a serious doubt for quarter-final clash with Norway</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49334996/athletics-all-star-1b-nick-kurtz-placed-il-thumb-sprain</t>
+          <t>https://www.skysports.com/football/news/12016/13562168/world-cup-2026-england-defender-marc-guehi-a-serious-doubt-for-quarter-final-clash-with-norway</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Nick Lodolo</t>
+          <t>Nick Kurtz</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Cincinnati Reds (MLB)</t>
+          <t>Athletics (MLB)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -901,12 +901,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Blister on the left index finger (throwing hand); a recurring issue, his fourth stint on the IL for blisters dating back to 2024</t>
+          <t>Right thumb capsule sprain</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Placed on the 15-day injured list; eligible to return July 27, though it could take longer depending on severity</t>
+          <t>Placed on the 10-day injured list, retroactive to July 10</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Reds turn to Rhett Lowder to fill Lodolo's rotation spot</t>
+          <t>Keeps the 2025 AL Rookie of the Year and scheduled AL All-Star starting first baseman (.266, 20 HR, 66 RBI, MLB-leading 76 walks) out of the July 14 All-Star Game in Philadelphia; catcher Brian Serven recalled from Triple-A in a corresponding move</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -926,24 +926,24 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>MLB Trade Rumors - Reds Place Nick Lodolo On IL With Blister, Recall Chase Petty</t>
+          <t>ESPN - Athletics All-Star 1B Nick Kurtz placed on IL with thumb sprain</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>https://www.mlbtraderumors.com/2026/07/reds-place-nick-lodolo-on-il-with-blister-recall-chase-petty.html</t>
+          <t>https://www.espn.com/mlb/story/_/id/49334996/athletics-all-star-1b-nick-kurtz-placed-il-thumb-sprain</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Nick Lodolo</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>New York Mets (MLB)</t>
+          <t>Cincinnati Reds (MLB)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -953,12 +953,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>General leg soreness and right ankle soreness, aggravated by fouling balls off his legs during a series in Atlanta</t>
+          <t>Blister on the left index finger (throwing hand); a recurring issue, his fourth stint on the IL for blisters dating back to 2024</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Held out of the lineup for a second straight game and available only off the bench; expected to use the following day and the All-Star break for a full reset rather than go on the injured list</t>
+          <t>Placed on the 15-day injured list; eligible to return July 27, though it could take longer depending on severity</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Mets manage his workload during a productive stretch (.320 avg, .788 OPS over his last 25 games) heading into the All-Star break</t>
+          <t>Reds turn to Rhett Lowder to fill Lodolo's rotation spot</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -978,39 +978,39 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Associated Press - Bo Bichette held out of Mets' lineup for second straight game with leg soreness</t>
+          <t>MLB Trade Rumors - Reds Place Nick Lodolo On IL With Blister, Recall Chase Petty</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://www.bakersfield.com/ap/sports/bo-bichette-held-out-of-mets-lineup-for-second-straight-game-with-leg-soreness/article_c615803d-891c-57fd-87ef-b86becfaf8cc.html</t>
+          <t>https://www.mlbtraderumors.com/2026/07/reds-place-nick-lodolo-on-il-with-blister-recall-chase-petty.html</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Collin Murray-Boyles</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Toronto Raptors (NBA) — Las Vegas Summer League</t>
+          <t>New York Mets (MLB)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Sprained thumb/finger, diagnosed after exiting a Summer League game against the Lakers</t>
+          <t>General leg soreness and right ankle soreness, aggravated by fouling balls off his legs during a series in Atlanta</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the Raptors' Summer League opener vs. Boston; next possible return targeted for the Houston game; full recovery timeline not specified in available reporting</t>
+          <t>Held out of the lineup for a second straight game and available only off the bench; expected to use the following day and the All-Star break for a full reset rather than go on the injured list</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1020,49 +1020,49 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Raptors lose their 2025 first-round pick (9th overall) for early Summer League reps as a point-forward, part of his developmental push</t>
+          <t>Mets manage his workload during a productive stretch (.320 avg, .788 OPS over his last 25 games) heading into the All-Star break</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Raptors Republic - Collin Murray-Boyles, Alijah Martin to miss Raptors' Summer League opener</t>
+          <t>Associated Press - Bo Bichette held out of Mets' lineup for second straight game with leg soreness</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>https://raptorsrepublic.com/2026/07/10/collin-murray-boyles-alijah-martin-to-miss-raptors-summer-league-opener/</t>
+          <t>https://www.bakersfield.com/ap/sports/bo-bichette-held-out-of-mets-lineup-for-second-straight-game-with-leg-soreness/article_c615803d-891c-57fd-87ef-b86becfaf8cc.html</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Shohei Ohtani</t>
+          <t>Conor McGregor</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers (MLB)</t>
+          <t>UFC</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Mixed Martial Arts</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Left knee irritation/swelling, nursed since at least June 11</t>
+          <t>Suspected torn ACL in the right knee, sustained throwing a kick just 69 seconds into his UFC 329 return bout; official diagnosis pending further medical evaluation</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Scratched from his Friday, July 10 pitching start vs. Arizona and will skip the All-Star Game; scheduled to have the knee drained and possibly receive a pain-relieving injection during the break</t>
+          <t>Fight stopped by the referee at 1:09 of round one; no recovery timeline given pending formal diagnosis</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1072,49 +1072,49 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Dodgers manage the two-way star's workload heading into the second half; Ohtani continued to DH and homered the same day he was scratched from pitching</t>
+          <t>Ends McGregor's much-hyped comeback fight against Max Holloway almost immediately and casts doubt on any near-term return to competition</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Shohei Ohtani dealing with knee irritation, to miss All-Star Game</t>
+          <t>NBC News - Conor McGregor suffers early knee injury in return, loses to Max Holloway at UFC 329</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49327458/shohei-ohtani-dealing-knee-irritation-miss-all-star-game</t>
+          <t>https://www.nbcnews.com/sports/ufc/conor-mcgregor-suffers-early-knee-injury-return-loses-max-holloway-ufc-rcna552729</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Gout Gout</t>
+          <t>Ezi Magbegor</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Athletics Australia (Track &amp; Field)</t>
+          <t>Seattle Storm (WNBA)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Athletics (Track &amp; Field)</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Grade-three left hamstring tear suffered in training in Brisbane</t>
+          <t>Facial fracture</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of the 2026 season, including the World Athletics U20 Championships (Aug. 5-9, Eugene, Oregon); targeting a return in 2027</t>
+          <t>Ruled out of the Storm's game vs. the Washington Mystics; to be reevaluated in the next couple of weeks</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1124,49 +1124,49 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Removes the U20 200m world record holder from an anticipated showdown with American Tate Taylor at the World U20 Championships</t>
+          <t>Storm without their starting center/forward for at least the near term</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Olympics.com - Gout Gout to miss World U20 Championships and rest of the season with hamstring injury</t>
+          <t>Seattle Times - Ezi Magbegor to miss Seattle Storm's game vs. Washington Mystics with face injury</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>https://www.olympics.com/en/news/gout-gout-injury-hamstring-world-athletics-under-20-championships</t>
+          <t>https://www.seattletimes.com/sports/storm/ezi-magbegor-to-miss-seattle-storms-game-vs-washington-mystics-with-face-injury/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Harshit Rana</t>
+          <t>Konnor Griffin</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>India National Cricket Team</t>
+          <t>Pittsburgh Pirates (MLB)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury sustained during the third T20I vs. England at Trent Bridge</t>
+          <t>Torn tendon (sagittal band) in the left ring finger, sustained diving for a ball; initially placed on the 10-day IL and now transferred to the 60-day IL</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
+          <t>8-10 week recovery timeline; ineligible to return until at least September 4; team opted for a non-operative approach, splinting the hand for about six weeks before resuming baseball activities</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1176,49 +1176,49 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Deepens India's bowling injury crisis on the England tour, with Rana joining Varun Chakaravarthy, Hardik Pandya, and Nitish Kumar Reddy on the unavailable list</t>
+          <t>Pirates lose their rookie starting shortstop (the No. 1 overall pick in the 2024 draft) for an extended stretch, his second significant injury of the season after an earlier forearm strain</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
+          <t>CBS Sports - Pirates' Konnor Griffin: Moved to 60-day IL</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
+          <t>https://www.cbssports.com/fantasy/baseball/news/pirates-konnor-griffin-moved-to-60-day-il/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Varun Chakaravarthy</t>
+          <t>Collin Murray-Boyles</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>India National Cricket Team</t>
+          <t>Toronto Raptors (NBA) — Las Vegas Summer League</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury sustained during the third T20I vs. England at Trent Bridge</t>
+          <t>Sprained thumb/finger, diagnosed after exiting a Summer League game against the Lakers</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
+          <t>Ruled out of the Raptors' Summer League opener vs. Boston; next possible return targeted for the Houston game; full recovery timeline not specified in available reporting</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1228,49 +1228,49 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>India's frontline wrist-spinner is unavailable as the team's injury list grows on the England tour</t>
+          <t>Raptors lose their 2025 first-round pick (9th overall) for early Summer League reps as a point-forward, part of his developmental push</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
+          <t>Raptors Republic - Collin Murray-Boyles, Alijah Martin to miss Raptors' Summer League opener</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
+          <t>https://raptorsrepublic.com/2026/07/10/collin-murray-boyles-alijah-martin-to-miss-raptors-summer-league-opener/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Litton Das</t>
+          <t>Shohei Ohtani</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh national cricket team</t>
+          <t>Los Angeles Dodgers (MLB)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Left calf injury; failed a fitness test ahead of the second ODI</t>
+          <t>Left knee irritation/swelling, nursed since at least June 11</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the remainder of the ODI series vs. Zimbabwe; continuing rehab in Dhaka</t>
+          <t>Scratched from his Friday, July 10 pitching start vs. Arizona and will skip the All-Star Game; scheduled to have the knee drained and possibly receive a pain-relieving injection during the break</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1280,49 +1280,49 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh loses their starting wicketkeeper-batter for the series; Parvez Hossain Emon named as replacement for the 2nd and 3rd ODIs</t>
+          <t>Dodgers manage the two-way star's workload heading into the second half; Ohtani continued to DH and homered the same day he was scratched from pitching</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>The Nation - Injured Litton Das to miss rest of Zimbabwe ODI series</t>
+          <t>ESPN - Shohei Ohtani dealing with knee irritation, to miss All-Star Game</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.nation.com.pk/09-Jul-2026/injured-litton-das-miss-rest-zimbabwe-odi-series</t>
+          <t>https://www.espn.com/mlb/story/_/id/49327458/shohei-ohtani-dealing-knee-irritation-miss-all-star-game</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Ravichandran Ashwin</t>
+          <t>Gout Gout</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>San Francisco Unicorns (Major League Cricket)</t>
+          <t>Athletics Australia (Track &amp; Field)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Athletics (Track &amp; Field)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Right knee injury</t>
+          <t>Grade-three left hamstring tear suffered in training in Brisbane</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of MLC 2026; replaced by Peter Siddle</t>
+          <t>Ruled out for the remainder of the 2026 season, including the World Athletics U20 Championships (Aug. 5-9, Eugene, Oregon); targeting a return in 2027</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Unicorns lose the veteran spinner after just one appearance this MLC season</t>
+          <t>Removes the U20 200m world record holder from an anticipated showdown with American Tate Taylor at the World U20 Championships</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1342,39 +1342,39 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>India TV News - Why is Ravichandran Ashwin ruled out of ongoing MLC 2026? San Francisco Unicorns announce replacement</t>
+          <t>Olympics.com - Gout Gout to miss World U20 Championships and rest of the season with hamstring injury</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>https://www.indiatvnews.com/sports/cricket/why-is-ravichandran-ashwin-ruled-out-of-ongoing-mlc-2026-san-francisco-unicorns-announce-replacement-2026-07-09-1047737</t>
+          <t>https://www.olympics.com/en/news/gout-gout-injury-hamstring-world-athletics-under-20-championships</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Aaron Judge</t>
+          <t>Harshit Rana</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>New York Yankees (MLB)</t>
+          <t>India National Cricket Team</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Stress fracture in right rib; has not played since May 31 and went on the injured list June 5</t>
+          <t>Hamstring injury sustained during the third T20I vs. England at Trent Bridge</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Will have the rib reimaged during the All-Star break; no firm return date, GM Brian Cashman says he must be fully asymptomatic and show healing on imaging before resuming activity</t>
+          <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Yankees continue without their three-time AL MVP and captain in the middle of the lineup</t>
+          <t>Deepens India's bowling injury crisis on the England tour, with Rana joining Varun Chakaravarthy, Hardik Pandya, and Nitish Kumar Reddy on the unavailable list</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1394,39 +1394,39 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Yankees' Aaron Judge to have rib reimaged during All-Star break</t>
+          <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49317023/yankees-aaron-judge-rib-reimaged-all-star-break</t>
+          <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mark Vientos</t>
+          <t>Varun Chakaravarthy</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>New York Mets (MLB)</t>
+          <t>India National Cricket Team</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Fractured bone in right hand after being hit by a pitch from Michael Wacha</t>
+          <t>Hamstring injury sustained during the third T20I vs. England at Trent Bridge</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Headed to the injured list; broken bones of this type typically take around six weeks to heal, though the Mets have not given an official timeline and have not yet said whether surgery is needed</t>
+          <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Mets lose a regular infielder/DH (.211, 11 HR, 35 RBI in 72 games) just ahead of the trade deadline</t>
+          <t>India's frontline wrist-spinner is unavailable as the team's injury list grows on the England tour</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1446,39 +1446,39 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>amNewYork - Mark Vientos injury: Mets IF/DH headed to IL with hand fracture</t>
+          <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>https://www.amny.com/sports/mark-vientos-injury-mets-7-9-26/</t>
+          <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Litton Das</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Athletics (MLB)</t>
+          <t>Bangladesh national cricket team</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Deep cut underneath the right kneecap after colliding with the left field fence on a sliding catch; came just missed the tendon per the team</t>
+          <t>Left calf injury; failed a fitness test ahead of the second ODI</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Left the July 9 game early; scheduled for an MRI on July 10 to confirm the extent of the injury</t>
+          <t>Ruled out of the remainder of the ODI series vs. Zimbabwe; continuing rehab in Dhaka</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Athletics risk losing an everyday infielder/outfielder who had an on-base streak of 27 straight games and a 13-game scoring streak snapped by the injury</t>
+          <t>Bangladesh loses their starting wicketkeeper-batter for the series; Parvez Hossain Emon named as replacement for the 2nd and 3rd ODIs</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1498,24 +1498,24 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Athletics' Gelof to have MRI on knee after sliding into fence</t>
+          <t>The Nation - Injured Litton Das to miss rest of Zimbabwe ODI series</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49319837/athletics-gelof-mri-knee-sliding-fence</t>
+          <t>https://www.nation.com.pk/09-Jul-2026/injured-litton-das-miss-rest-zimbabwe-odi-series</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Chinelle Henry</t>
+          <t>Ravichandran Ashwin</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>West Indies Women's National Cricket Team</t>
+          <t>San Francisco Unicorns (Major League Cricket)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1525,12 +1525,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Exacerbation of a previous injury originally suffered fielding (stretchered off) in a T20 World Cup warm-up match in June</t>
+          <t>Right knee injury</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the Women's ODI tour of Ireland beginning July 10; no return timeline disclosed</t>
+          <t>Ruled out for the remainder of MLC 2026; replaced by Peter Siddle</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>West Indies lose their vice-captain and a key all-rounder; Realeanna Grimmond called up as her replacement for the Ireland series</t>
+          <t>Unicorns lose the veteran spinner after just one appearance this MLC season</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1550,39 +1550,39 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>ESPNcricinfo - Realeanna Grimmond replaces injured Chinelle Henry in West Indies squad for Ireland Women's ODIs</t>
+          <t>India TV News - Why is Ravichandran Ashwin ruled out of ongoing MLC 2026? San Francisco Unicorns announce replacement</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://www.espncricinfo.com/story/slug-1545066</t>
+          <t>https://www.indiatvnews.com/sports/cricket/why-is-ravichandran-ashwin-ruled-out-of-ongoing-mlc-2026-san-francisco-unicorns-announce-replacement-2026-07-09-1047737</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Torstein Træen</t>
+          <t>Aaron Judge</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Uno-X Mobility (Tour de France) — Norway</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Cycling</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Concussion and multiple fractured ribs sustained in a crash on the descent of the Col du Tourmalet during stage 6</t>
+          <t>Stress fracture in right rib; has not played since May 31 and went on the injured list June 5</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Withdrew from the Tour de France (did not start stage 7); no return timeline specified in available reporting</t>
+          <t>Will have the rib reimaged during the All-Star break; no firm return date, GM Brian Cashman says he must be fully asymptomatic and show healing on imaging before resuming activity</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Uno-X Mobility loses the rider who had been wearing the race's yellow jersey after stage 5; Tadej Pogačar reclaimed the overall race lead the same day</t>
+          <t>Yankees continue without their three-time AL MVP and captain in the middle of the lineup</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1602,39 +1602,39 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Cyclingnews - 'Not the ending we wanted for this yellow adventure' - Torstein Træen out of Tour de France due to injuries from Tourmalet crash</t>
+          <t>ESPN - Yankees' Aaron Judge to have rib reimaged during All-Star break</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.cyclingnews.com/pro-cycling/teams-riders/not-the-ending-we-wanted-for-this-yellow-adventure-torstein-traeen-out-of-tour-de-france-due-to-injuries-from-tourmalet-crash/</t>
+          <t>https://www.espn.com/mlb/story/_/id/49317023/yankees-aaron-judge-rib-reimaged-all-star-break</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Alex Molenaar</t>
+          <t>Mark Vientos</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Caja Rural-Seguros RGA (Tour de France) — Netherlands</t>
+          <t>New York Mets (MLB)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Cycling</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Fracture of the first metacarpal in his right hand plus multiple contusions, sustained in a high-speed crash roughly 5km from the finish of stage 5; evaluated under concussion protocol after losing memory of the incident</t>
+          <t>Fractured bone in right hand after being hit by a pitch from Michael Wacha</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Abandoned the Tour de France; did not start stage 6; recovery timeline not specified in available reporting</t>
+          <t>Headed to the injured list; broken bones of this type typically take around six weeks to heal, though the Mets have not given an official timeline and have not yet said whether surgery is needed</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Caja Rural-Seguros RGA loses a rider mid-Tour</t>
+          <t>Mets lose a regular infielder/DH (.211, 11 HR, 35 RBI in 72 games) just ahead of the trade deadline</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1654,39 +1654,39 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Cycling Weekly - 'I don't remember the crash' – Caja Rural rider abandons Tour de France with fractured hand</t>
+          <t>amNewYork - Mark Vientos injury: Mets IF/DH headed to IL with hand fracture</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://www.cyclingweekly.com/racing/tour-de-france/i-dont-remember-the-crash-caja-rural-rider-abandons-tour-de-france-with-fractured-hand</t>
+          <t>https://www.amny.com/sports/mark-vientos-injury-mets-7-9-26/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Arvid de Kleijn</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Tudor Pro Cycling Team (Tour de France) — Netherlands</t>
+          <t>Athletics (MLB)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Cycling</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Muscle tears sustained during the stage 1 team time trial, which hampered him for the rest of the race</t>
+          <t>Deep cut underneath the right kneecap after colliding with the left field fence on a sliding catch; came just missed the tendon per the team</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Abandoned the Tour de France on stage 6 after struggling since the opening days; recovery timeline not specified in available reporting</t>
+          <t>Left the July 9 game early; scheduled for an MRI on July 10 to confirm the extent of the injury</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Tudor Pro Cycling Team loses a rider mid-Tour after he battled to beat the time cut on multiple stages</t>
+          <t>Athletics risk losing an everyday infielder/outfielder who had an on-base streak of 27 straight games and a 13-game scoring streak snapped by the injury</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1706,39 +1706,39 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>idlprocycling - Suffering ends: Arvid de Kleijn and Cian Uijtdebroeks abandon Tour de France</t>
+          <t>ESPN - Athletics' Gelof to have MRI on knee after sliding into fence</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.idlprocycling.com/cycling/suffering-ends-arvid-de-kleijn-and-cian-uijtdebroeks-abandon-tour-de-france</t>
+          <t>https://www.espn.com/mlb/story/_/id/49319837/athletics-gelof-mri-knee-sliding-fence</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Carlos Alcaraz</t>
+          <t>Chinelle Henry</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>ATP Tour</t>
+          <t>West Indies Women's National Cricket Team</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Right-wrist tenosynovitis, forcing withdrawals from Madrid, Rome, Roland Garros, Queen's and Wimbledon; has worn a wrist brace since mid-April</t>
+          <t>Exacerbation of a previous injury originally suffered fielding (stretchered off) in a T20 World Cup warm-up match in June</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Has pulled out of the ATP Montreal entry list and opted to prolong his comeback by two more weeks, targeting Cincinnati or the US Open for his return; recently resumed light on-court practice without a brace</t>
+          <t>Ruled out of the Women's ODI tour of Ireland beginning July 10; no return timeline disclosed</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>World No. 2 has now missed a full clay and grass swing including two Grand Slams; absence continues into the North American hard-court season</t>
+          <t>West Indies lose their vice-captain and a key all-rounder; Realeanna Grimmond called up as her replacement for the Ireland series</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1758,39 +1758,39 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Last Word On Tennis - Carlos Alcaraz Injury Update: Spaniard Pulls Out of ATP Montreal Entry List</t>
+          <t>ESPNcricinfo - Realeanna Grimmond replaces injured Chinelle Henry in West Indies squad for Ireland Women's ODIs</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://lastwordonsports.com/tennis/2026/07/09/carlos-alcaraz-injury-update-spaniard-pulls-out-of-atp-montreal/</t>
+          <t>https://www.espncricinfo.com/story/slug-1545066</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Connor Bedard</t>
+          <t>Torstein Træen</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Chicago Blackhawks (NHL)</t>
+          <t>Uno-X Mobility (Tour de France) — Norway</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Hockey</t>
+          <t>Cycling</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Surgery on left shoulder after an injury sustained during a practice session in Vancouver on July 2</t>
+          <t>Concussion and multiple fractured ribs sustained in a crash on the descent of the Col du Tourmalet during stage 6</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Expected to need approximately four months to recover; will miss training camp and at least the start of the 2026-27 season</t>
+          <t>Withdrew from the Tour de France (did not start stage 7); no return timeline specified in available reporting</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1800,49 +1800,49 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Blackhawks will open the 2026-27 season, played under the NHL's expanded 84-game schedule, without their No. 1 center for at least the opening month</t>
+          <t>Uno-X Mobility loses the rider who had been wearing the race's yellow jersey after stage 5; Tadej Pogačar reclaimed the overall race lead the same day</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>NHL.com - Bedard to miss start of 2026-27 season for Blackhawks after shoulder surgery</t>
+          <t>Cyclingnews - 'Not the ending we wanted for this yellow adventure' - Torstein Træen out of Tour de France due to injuries from Tourmalet crash</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.nhl.com/news/connor-bedard-injury-status-update-july-8-2026</t>
+          <t>https://www.cyclingnews.com/pro-cycling/teams-riders/not-the-ending-we-wanted-for-this-yellow-adventure-torstein-traeen-out-of-tour-de-france-due-to-injuries-from-tourmalet-crash/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Aliyah Boston</t>
+          <t>Alex Molenaar</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Indiana Fever (WNBA)</t>
+          <t>Caja Rural-Seguros RGA (Tour de France) — Netherlands</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Cycling</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Lower right leg injury</t>
+          <t>Fracture of the first metacarpal in his right hand plus multiple contusions, sustained in a high-speed crash roughly 5km from the finish of stage 5; evaluated under concussion protocol after losing memory of the incident</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Listed out for the Fever's game vs. the LA Sparks; expected to be available for the following game vs. Phoenix</t>
+          <t>Abandoned the Tour de France; did not start stage 6; recovery timeline not specified in available reporting</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1852,49 +1852,49 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Fever forced to manage the availability of both Boston and Caitlin Clark during a back-to-back stretch; Boston, a voted-in 2026 All-Star starter, is having a career-best scoring season (17.1 ppg on 50.4% shooting) and was in danger of missing her first game since May 17</t>
+          <t>Caja Rural-Seguros RGA loses a rider mid-Tour</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Athlon Sports - Indiana Fever Announce Aliyah Boston Injury Update Before LA Sparks Game</t>
+          <t>Cycling Weekly - 'I don't remember the crash' – Caja Rural rider abandons Tour de France with fractured hand</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://athlonsports.com/wnba/indiana-fever/indiana-fever-announce-aliyah-boston-injury-update-la-sparks-game</t>
+          <t>https://www.cyclingweekly.com/racing/tour-de-france/i-dont-remember-the-crash-caja-rural-rider-abandons-tour-de-france-with-fractured-hand</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Reece James</t>
+          <t>Arvid de Kleijn</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Chelsea FC (Premier League) / England National Team (2026 FIFA World Cup)</t>
+          <t>Tudor Pro Cycling Team (Tour de France) — Netherlands</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Cycling</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury sustained in England's final group-stage match vs. Ghana on June 23; described by reporting as worse than first thought</t>
+          <t>Muscle tears sustained during the stage 1 team time trial, which hampered him for the rest of the race</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Touch-and-go for England's July 11 World Cup quarterfinal vs. Norway; has missed England's last three matches and was the sole absentee from the team's final group training session, requiring final medical clearance just to be considered for the bench</t>
+          <t>Abandoned the Tour de France on stage 6 after struggling since the opening days; recovery timeline not specified in available reporting</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1904,49 +1904,49 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Compounds an England right-back crisis that worsened after Jarell Quansah's red card vs. Mexico, leaving manager Thomas Tuchel with very limited options at the position for the quarterfinal</t>
+          <t>Tudor Pro Cycling Team loses a rider mid-Tour after he battled to beat the time cut on multiple stages</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Sky Sports - England World Cup latest: Reece James in race to be fit for quarter-final clash with Norway to ease right-back crisis</t>
+          <t>idlprocycling - Suffering ends: Arvid de Kleijn and Cian Uijtdebroeks abandon Tour de France</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.skysports.com/football/news/11095/13561150/england-world-cup-latest-reece-james-in-race-to-be-fit-for-quarter-final-clash-with-norway-to-ease-right-back-crisis</t>
+          <t>https://www.idlprocycling.com/cycling/suffering-ends-arvid-de-kleijn-and-cian-uijtdebroeks-abandon-tour-de-france</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Aurelien Tchouameni</t>
+          <t>Carlos Alcaraz</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Real Madrid (La Liga) / France National Team (2026 FIFA World Cup)</t>
+          <t>ATP Tour</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Tennis</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Muscle tear involving the left adductor and upper thigh, a recurrence of the groin/thigh issue that previously sidelined him for France's group-stage match vs. Iraq</t>
+          <t>Right-wrist tenosynovitis, forcing withdrawals from Madrid, Rome, Roland Garros, Queen's and Wimbledon; has worn a wrist brace since mid-April</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Missed France's Round of 16 win over Paraguay; returned to partial team training on July 8, with a decision on his availability for the July 11 quarterfinal vs. Morocco pending</t>
+          <t>Has pulled out of the ATP Montreal entry list and opted to prolong his comeback by two more weeks, targeting Cincinnati or the US Open for his return; recently resumed light on-court practice without a brace</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1956,49 +1956,49 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>France's vice-captain and starting defensive midfielder is a doubt for the quarterfinal, with Manu Kone deputizing in his absence</t>
+          <t>World No. 2 has now missed a full clay and grass swing including two Grand Slams; absence continues into the North American hard-court season</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Sportskeeda - France handed huge injury boost as star man returns to training ahead of FIFA World Cup Q/F against Morocco</t>
+          <t>Last Word On Tennis - Carlos Alcaraz Injury Update: Spaniard Pulls Out of ATP Montreal Entry List</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>https://www.sportskeeda.com/football/rumor-france-handed-huge-injury-boost-star-man-returns-training-ahead-fifa-world-cup-q-f-morocco-reports</t>
+          <t>https://lastwordonsports.com/tennis/2026/07/09/carlos-alcaraz-injury-update-spaniard-pulls-out-of-atp-montreal/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Mustafizur Rahman</t>
+          <t>Connor Bedard</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh National Cricket Team</t>
+          <t>Chicago Blackhawks (NHL)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Cricket</t>
+          <t>Hockey</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Grade 1 muscle tear in the right hamstring and meniscal degeneration in the right knee, felt while bowling in the first ODI vs. Zimbabwe</t>
+          <t>Surgery on left shoulder after an injury sustained during a practice session in Vancouver on July 2</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for four weeks, covering the remainder of Bangladesh's tour of Zimbabwe (concluding July 19), including the T20I series; has returned home for rehab</t>
+          <t>Expected to need approximately four months to recover; will miss training camp and at least the start of the 2026-27 season</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh lose a frontline pace bowler for the rest of the Zimbabwe tour</t>
+          <t>Blackhawks will open the 2026-27 season, played under the NHL's expanded 84-game schedule, without their No. 1 center for at least the opening month</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2018,39 +2018,39 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>ESPNcricinfo - Zim vs Ban: Mustafizur Rahman ruled out for four weeks with hamstring and knee injuries</t>
+          <t>NHL.com - Bedard to miss start of 2026-27 season for Blackhawks after shoulder surgery</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.espncricinfo.com/story/zim-vs-ban-mustafizur-rahman-ruled-out-for-four-weeks-with-hamstring-and-knee-injuries-1545065</t>
+          <t>https://www.nhl.com/news/connor-bedard-injury-status-update-july-8-2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Marco Raya</t>
+          <t>Aliyah Boston</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Twins (MLB)</t>
+          <t>Indiana Fever (WNBA)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Right shoulder impingement</t>
+          <t>Lower right leg injury</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Placed on 15-day IL July 8, retroactive to July 5</t>
+          <t>Listed out for the Fever's game vs. the LA Sparks; expected to be available for the following game vs. Phoenix</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Twins lose a pitching option for at least 15 days</t>
+          <t>Fever forced to manage the availability of both Boston and Caitlin Clark during a back-to-back stretch; Boston, a voted-in 2026 All-Star starter, is having a career-best scoring season (17.1 ppg on 50.4% shooting) and was in danger of missing her first game since May 17</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2070,39 +2070,39 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>MLB.com - Latest Twins injuries &amp; transactions</t>
+          <t>Athlon Sports - Indiana Fever Announce Aliyah Boston Injury Update Before LA Sparks Game</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>https://www.mlb.com/news/twins-injuries-and-roster-moves</t>
+          <t>https://athlonsports.com/wnba/indiana-fever/indiana-fever-announce-aliyah-boston-injury-update-la-sparks-game</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Endy Rodriguez</t>
+          <t>Reece James</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates (MLB)</t>
+          <t>Chelsea FC (Premier League) / England National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Left glute strain</t>
+          <t>Hamstring injury sustained in England's final group-stage match vs. Ghana on June 23; described by reporting as worse than first thought</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Placed on 10-day IL July 8, retroactive to July 6</t>
+          <t>Touch-and-go for England's July 11 World Cup quarterfinal vs. Norway; has missed England's last three matches and was the sole absentee from the team's final group training session, requiring final medical clearance just to be considered for the bench</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Pirates lose their starting catcher for at least 10 days</t>
+          <t>Compounds an England right-back crisis that worsened after Jarell Quansah's red card vs. Mexico, leaving manager Thomas Tuchel with very limited options at the position for the quarterfinal</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2122,39 +2122,39 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>MLB Trade Rumors - Pirates Place Endy Rodriguez On Injured List</t>
+          <t>Sky Sports - England World Cup latest: Reece James in race to be fit for quarter-final clash with Norway to ease right-back crisis</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.mlbtraderumors.com/2026/07/pirates-to-place-endy-rodriguez-on-injured-list.html</t>
+          <t>https://www.skysports.com/football/news/11095/13561150/england-world-cup-latest-reece-james-in-race-to-be-fit-for-quarter-final-clash-with-norway-to-ease-right-back-crisis</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Taylor Fritz</t>
+          <t>Aurelien Tchouameni</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>ATP Tour</t>
+          <t>Real Madrid (La Liga) / France National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Knee tendinitis flare-up, a recurring issue, three games into his Wimbledon quarterfinal</t>
+          <t>Muscle tear involving the left adductor and upper thigh, a recurrence of the groin/thigh issue that previously sidelined him for France's group-stage match vs. Iraq</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Played through the flare-up but lost the quarterfinal 6-4, 6-4, 6-2 to Alexander Zverev; no absence or further tournament withdrawal reported</t>
+          <t>Missed France's Round of 16 win over Paraguay; returned to partial team training on July 8, with a decision on his availability for the July 11 quarterfinal vs. Morocco pending</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Eliminated from Wimbledon; dropped to No. 10 in the ATP Live Rankings</t>
+          <t>France's vice-captain and starting defensive midfielder is a doubt for the quarterfinal, with Manu Kone deputizing in his absence</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2174,39 +2174,39 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Taylor Fritz loses at Wimbledon after knee tendinitis flares up</t>
+          <t>Sportskeeda - France handed huge injury boost as star man returns to training ahead of FIFA World Cup Q/F against Morocco</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/tennis/story/_/id/49308826/taylor-fritz-loses-alexander-zverev-wimbledon-quarterfinals-knee-tendonitis-flares-up</t>
+          <t>https://www.sportskeeda.com/football/rumor-france-handed-huge-injury-boost-star-man-returns-training-ahead-fifa-world-cup-q-f-morocco-reports</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Jalen Brunson</t>
+          <t>Mustafizur Rahman</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>New York Knicks (NBA)</t>
+          <t>Bangladesh National Cricket Team</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Cricket</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Surgery to repair a left wrist injury that he played through during the Knicks' championship playoff run</t>
+          <t>Grade 1 muscle tear in the right hamstring and meniscal degeneration in the right knee, felt while bowling in the first ODI vs. Zimbabwe</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>At least two months of rehab expected; targeting readiness for the start of the 2026-27 NBA season</t>
+          <t>Ruled out for four weeks, covering the remainder of Bangladesh's tour of Zimbabwe (concluding July 19), including the T20I series; has returned home for rehab</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2216,49 +2216,49 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Reigning Finals MVP and starting point guard sidelined for part of the offseason program, though expected back for training camp</t>
+          <t>Bangladesh lose a frontline pace bowler for the rest of the Zimbabwe tour</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports - Knicks superstar Jalen Brunson undergoes left wrist surgery, expected to be ready for 2026-27 NBA season</t>
+          <t>ESPNcricinfo - Zim vs Ban: Mustafizur Rahman ruled out for four weeks with hamstring and knee injuries</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/nba/breaking-news/article/knicks-superstar-jalen-brunson-undergoes-left-wrist-surgery-expected-to-be-ready-for-2026-27-nba-season-155927234.html</t>
+          <t>https://www.espncricinfo.com/story/zim-vs-ban-mustafizur-rahman-ruled-out-for-four-weeks-with-hamstring-and-knee-injuries-1545065</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Amadou Onana</t>
+          <t>Marco Raya</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Aston Villa (Premier League) / Belgium National Team (2026 FIFA World Cup)</t>
+          <t>Minnesota Twins (MLB)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Torn anterior cruciate ligament (ACL), sustained in the 21st minute of Belgium's Round of 16 win over the United States after a challenge with Christian Pulisic</t>
+          <t>Right shoulder impingement</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of the World Cup; reported to be facing up to eight months out</t>
+          <t>Placed on 15-day IL July 8, retroactive to July 5</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2268,34 +2268,34 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Belgium loses a key defensive midfielder ahead of their World Cup quarterfinal vs. Spain, and Aston Villa will be without him for a significant part of the 2026-27 season</t>
+          <t>Twins lose a pitching option for at least 15 days</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Belgium's Amadou Onana out of World Cup after suffering ACL injury</t>
+          <t>MLB.com - Latest Twins injuries &amp; transactions</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49298508/belgium-amadou-onana-world-cup-suffering-acl-injury</t>
+          <t>https://www.mlb.com/news/twins-injuries-and-roster-moves</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Giancarlo Stanton</t>
+          <t>Endy Rodriguez</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>New York Yankees (MLB)</t>
+          <t>Pittsburgh Pirates (MLB)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2305,12 +2305,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Right calf strain (originally suffered running the bases on April 24 vs. the Astros); recent rehab setback after re-aggravating the calf during a running progression</t>
+          <t>Left glute strain</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>No firm timeline; has not resumed running since the setback, no target return date given</t>
+          <t>Placed on 10-day IL July 8, retroactive to July 6</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2320,29 +2320,29 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Yankees continue without their veteran slugger amid an offense that has struggled with injuries; manager Aaron Boone still expects him back at some point in 2026</t>
+          <t>Pirates lose their starting catcher for at least 10 days</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Last Word on Sports - Stanton Injury Update: Slugger Yet To Resume Rehab On Calf</t>
+          <t>MLB Trade Rumors - Pirates Place Endy Rodriguez On Injured List</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://lastwordonsports.com/baseball/2026/07/07/nyy-stanton-injury-update/</t>
+          <t>https://www.mlbtraderumors.com/2026/07/pirates-to-place-endy-rodriguez-on-injured-list.html</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Matteo Berrettini</t>
+          <t>Taylor Fritz</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2357,153 +2357,153 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Diagnosed with chronic hip pain, a recurrence of the left hip issue that forced his retirement from his Roland Garros quarterfinal in early June</t>
+          <t>Knee tendinitis flare-up, a recurring issue, three games into his Wimbledon quarterfinal</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Withdrawing from the ATP tournaments in Gstaad and Kitzbuhel to rest on medical advice, with the goal of being ready for the US hard-court swing culminating in the US Open; no firm return date given</t>
+          <t>Played through the flare-up but lost the quarterfinal 6-4, 6-4, 6-2 to Alexander Zverev; no absence or further tournament withdrawal reported</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Forfeits ranking points and prize money from both the Gstaad and Kitzbuhel events</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Removes him from the draw at both tournaments immediately following his third-round Wimbledon loss to Grigor Dimitrov</t>
+          <t>Eliminated from Wimbledon; dropped to No. 10 in the ATP Live Rankings</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Puntodebreak - Berrettini withdraws from competing in upcoming tournaments due to "chronic hip pain"</t>
+          <t>ESPN - Taylor Fritz loses at Wimbledon after knee tendinitis flares up</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>https://www.puntodebreak.com/en/2026/07/07/berrettini-withdraws-from-competing-in-upcoming-tournaments-due-to-chronic-hip-pain</t>
+          <t>https://www.espn.com/tennis/story/_/id/49308826/taylor-fritz-loses-alexander-zverev-wimbledon-quarterfinals-knee-tendonitis-flares-up</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Skylar Diggins</t>
+          <t>Elvis Smylie</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Chicago Sky (WNBA)</t>
+          <t>LIV Golf (Ripper GC) / DP World Tour</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Golf</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Right knee injury; Diggins has said a knee surgery from last October has contributed to ongoing strain</t>
+          <t>Rib injury</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the July 7 game vs. Phoenix Mercury; no return timeline given</t>
+          <t>Withdrew from the Genesis Scottish Open and The Open Championship at Royal Birkdale; announced an extended break from golf for rehabilitation, with no firm return timeline given</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Forfeits prize money and Race to Dubai/world ranking points from both events</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Comes as Diggins was moved to the bench for the first time in a decade, ending a streak of 341 consecutive starts; Sky beat Phoenix 77-66 in her absence</t>
+          <t>Removes the Australian, who had qualified for his third Open Championship appearance, from the year's final men's major</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports - Sky's Skylar Diggins ruled out (knee) after being benched, Vandersloot starting</t>
+          <t>Today's Golfer - LIV Golf star withdraws on the eve of The Open</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/articles/skys-skylar-diggins-ruled-vs-010259203.html</t>
+          <t>https://www.todays-golfer.com/news-and-events/majors/the-open-championship/elvis-smylie-liv-golf-withdrawal/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Emma Raducanu</t>
+          <t>Jalen Brunson</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>New York Knicks (NBA)</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Stress fracture in lower right leg (ankle area); withdrew hours before her scheduled first-round match</t>
+          <t>Surgery to repair a left wrist injury that he played through during the Knicks' championship playoff run</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of Wimbledon 2026; still on crutches and wearing a protective boot several days after withdrawal, no return timeline given</t>
+          <t>At least two months of rehab expected; targeting readiness for the start of the 2026-27 NBA season</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Loses out on Wimbledon prize money and ranking points for the event</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Removes a top British draw from the tournament</t>
+          <t>Reigning Finals MVP and starting point guard sidelined for part of the offseason program, though expected back for training camp</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - Emma Raducanu setback deepens as British star remains on crutches after Wimbledon withdrawal</t>
+          <t>Yahoo Sports - Knicks superstar Jalen Brunson undergoes left wrist surgery, expected to be ready for 2026-27 NBA season</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/tennis/articles/emma_raducanu_setback_deepens_as_british_star_remains_on_crutches_after_wimbledon_withdrawal/s1_17460_44037038</t>
+          <t>https://sports.yahoo.com/nba/breaking-news/article/knicks-superstar-jalen-brunson-undergoes-left-wrist-surgery-expected-to-be-ready-for-2026-27-nba-season-155927234.html</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Jordan Henderson</t>
+          <t>Amadou Onana</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>England National Team (2026 FIFA World Cup)</t>
+          <t>Aston Villa (Premier League) / Belgium National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2513,12 +2513,12 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Wrist fracture sustained in a freak fall while celebrating England's Round of 16 win over Mexico; reportedly requires surgery</t>
+          <t>Torn anterior cruciate ligament (ACL), sustained in the 21st minute of Belgium's Round of 16 win over the United States after a challenge with Christian Pulisic</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for the remainder of the 2026 World Cup; exact surgery date and recovery length not yet specified</t>
+          <t>Ruled out for the remainder of the World Cup; reported to be facing up to eight months out</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2528,49 +2528,49 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>England advance to the quarterfinals without an experienced veteran midfielder, compounding a growing injury list</t>
+          <t>Belgium loses a key defensive midfielder ahead of their World Cup quarterfinal vs. Spain, and Aston Villa will be without him for a significant part of the 2026-27 season</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>ESPN - England's Henderson hospitalized with wrist injury during celebration</t>
+          <t>ESPN - Belgium's Amadou Onana out of World Cup after suffering ACL injury</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49283507/jordan-henderson-taken-hospital-wrist-injury-falling-mexico-victory-celebrations-england-world-cup</t>
+          <t>https://www.espn.com/soccer/story/_/id/49298508/belgium-amadou-onana-world-cup-suffering-acl-injury</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Santiago Gimenez</t>
+          <t>Giancarlo Stanton</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>AC Milan (Serie A) / Mexico National Team</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Grade II right ankle sprain suffered in stoppage time of Mexico's Round of 16 loss to England; hospitalized, but avoided fracture and ligament damage</t>
+          <t>Right calf strain (originally suffered running the bases on April 24 vs. the Astros); recent rehab setback after re-aggravating the calf during a running progression</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Not yet specified by club or national team</t>
+          <t>No firm timeline; has not resumed running since the setback, no target return date given</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2580,86 +2580,86 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Injury compounds Mexico's World Cup elimination and raises concern over his fitness for AC Milan's preseason</t>
+          <t>Yankees continue without their veteran slugger amid an offense that has struggled with injuries; manager Aaron Boone still expects him back at some point in 2026</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>beIN Sports - Adding insult to injury! Santiago Gimenez suffers injury during Mexico's loss to England</t>
+          <t>Last Word on Sports - Stanton Injury Update: Slugger Yet To Resume Rehab On Calf</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>https://www.beinsports.com/en-us/soccer/fifa-world-cup-2026/articles/adding-insult-to-injury-santiago-gimenez-suffers-injury-during-mexico-s-loss-to-england-2026-07-06</t>
+          <t>https://lastwordonsports.com/baseball/2026/07/07/nyy-stanton-injury-update/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Ismael Saibari</t>
+          <t>Matteo Berrettini</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Bayern Munich (Bundesliga, incoming) / Morocco National Team (2026 FIFA World Cup)</t>
+          <t>ATP Tour</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Tennis</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Hamstring injury (minor muscle issue per medical tests; serious strain ruled out) suffered in the 22nd minute of Morocco's Round of 16 win over Canada</t>
+          <t>Diagnosed with chronic hip pain, a recurrence of the left hip issue that forced his retirement from his Roland Garros quarterfinal in early June</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Day-to-day pending fitness test; final decision on availability for the World Cup quarterfinal vs. France expected only hours before kickoff</t>
+          <t>Withdrawing from the ATP tournaments in Gstaad and Kitzbuhel to rest on medical advice, with the goal of being ready for the US hard-court swing culminating in the US Open; no firm return date given</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Forfeits ranking points and prize money from both the Gstaad and Kitzbuhel events</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Morocco risks losing their top attacking threat (three group-stage goals) for the biggest match of their World Cup run</t>
+          <t>Removes him from the draw at both tournaments immediately following his third-round Wimbledon loss to Grigor Dimitrov</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>The National - Ismael Saibari fitness concern for Morocco ahead of France World Cup quarter-final clash</t>
+          <t>Puntodebreak - Berrettini withdraws from competing in upcoming tournaments due to "chronic hip pain"</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.thenationalnews.com/sport/world-cup-2026/2026/07/06/ismael-saibari-fitness-concern-for-morocco-ahead-of-france-world-cup-quarter-final-clash/</t>
+          <t>https://www.puntodebreak.com/en/2026/07/07/berrettini-withdraws-from-competing-in-upcoming-tournaments-due-to-chronic-hip-pain</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>A'ja Wilson</t>
+          <t>Skylar Diggins</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Las Vegas Aces (WNBA)</t>
+          <t>Chicago Sky (WNBA)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2669,12 +2669,12 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Foot injury sustained in a game against the Chicago Sky</t>
+          <t>Right knee injury; Diggins has said a knee surgery from last October has contributed to ongoing strain</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Missed 3 games; coach Becky Hammon said she could have played if it were a playoff game, suggesting an imminent return</t>
+          <t>Ruled out for the July 7 game vs. Phoenix Mercury; no return timeline given</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2684,59 +2684,59 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Aces without their All-Star forward/center for a short stretch, including a loss to Indiana</t>
+          <t>Comes as Diggins was moved to the bench for the first time in a decade, ending a streak of 341 consecutive starts; Sky beat Phoenix 77-66 in her absence</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>Yahoo Sports - Sky's Skylar Diggins ruled out (knee) after being benched, Vandersloot starting</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://sports.yahoo.com/articles/skys-skylar-diggins-ruled-vs-010259203.html</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Caitlin Clark</t>
+          <t>Emma Raducanu</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Indiana Fever (WNBA)</t>
+          <t>WTA Tour</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Tennis</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Aggravated back injury</t>
+          <t>Stress fracture in lower right leg (ankle area); withdrew hours before her scheduled first-round match</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Has resumed practicing; no confirmed timeline yet for a game return</t>
+          <t>Ruled out of Wimbledon 2026; still on crutches and wearing a protective boot several days after withdrawal, no return timeline given</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Loses out on Wimbledon prize money and ranking points for the event</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Fever have played without their All-Star starting guard for an extended stretch</t>
+          <t>Removes a top British draw from the tournament</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2746,39 +2746,39 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>Yardbarker - Emma Raducanu setback deepens as British star remains on crutches after Wimbledon withdrawal</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://www.yardbarker.com/tennis/articles/emma_raducanu_setback_deepens_as_british_star_remains_on_crutches_after_wimbledon_withdrawal/s1_17460_44037038</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Napheesa Collier</t>
+          <t>Jordan Henderson</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Lynx (WNBA)</t>
+          <t>England National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Offseason surgery on both ankles</t>
+          <t>Wrist fracture sustained in a freak fall while celebrating England's Round of 16 win over Mexico; reportedly requires surgery</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Has yet to play in the 2026 season; recently resumed practicing</t>
+          <t>Ruled out for the remainder of the 2026 World Cup; exact surgery date and recovery length not yet specified</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Lynx have been without their All-Star forward for the entire season to date</t>
+          <t>England advance to the quarterfinals without an experienced veteran midfielder, compounding a growing injury list</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2798,39 +2798,39 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
+          <t>ESPN - England's Henderson hospitalized with wrist injury during celebration</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
+          <t>https://www.espn.com/soccer/story/_/id/49283507/jordan-henderson-taken-hospital-wrist-injury-falling-mexico-victory-celebrations-england-world-cup</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Lexi Thompson</t>
+          <t>Santiago Gimenez</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>LPGA Tour</t>
+          <t>AC Milan (Serie A) / Mexico National Team</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Golf</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Persistent hip pain/suspected hip injury</t>
+          <t>Grade II right ankle sprain suffered in stoppage time of Mexico's Round of 16 loss to England; hospitalized, but avoided fracture and ligament damage</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Withdrew from the KPMG Women's PGA Championship at Hazeltine National, after also sitting out the Meijer LPGA Classic with the same issue; no return timeline given</t>
+          <t>Not yet specified by club or national team</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Ends a 15-tournament appearance streak at the Women's PGA Championship, a run that included four career top-10 finishes; Carolina Chacarra took her place in the field</t>
+          <t>Injury compounds Mexico's World Cup elimination and raises concern over his fitness for AC Milan's preseason</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2850,39 +2850,39 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Golf Digest - Lexi Thompson withdraws from KPMG Women's PGA Championship</t>
+          <t>beIN Sports - Adding insult to injury! Santiago Gimenez suffers injury during Mexico's loss to England</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.golfdigest.com/story/lexi-thompson-withdraws-kpmg-womens-pga-championship</t>
+          <t>https://www.beinsports.com/en-us/soccer/fifa-world-cup-2026/articles/adding-insult-to-injury-santiago-gimenez-suffers-injury-during-mexico-s-loss-to-england-2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Byron Buxton</t>
+          <t>Ismael Saibari</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Twins (MLB)</t>
+          <t>Bayern Munich (Bundesliga, incoming) / Morocco National Team (2026 FIFA World Cup)</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Aggravated hip injury while being caught stealing in the 1st inning vs. Yankees</t>
+          <t>Hamstring injury (minor muscle issue per medical tests; serious strain ruled out) suffered in the 22nd minute of Morocco's Round of 16 win over Canada</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Day-to-day; had already missed 4 games earlier in the week with the same hip issue</t>
+          <t>Day-to-day pending fitness test; final decision on availability for the World Cup quarterfinal vs. France expected only hours before kickoff</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2892,49 +2892,49 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Twins lose their 2026 All-Star outfielder from the lineup for an undetermined stretch</t>
+          <t>Morocco risks losing their top attacking threat (three group-stage goals) for the biggest match of their World Cup run</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>The National - Ismael Saibari fitness concern for Morocco ahead of France World Cup quarter-final clash</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.thenationalnews.com/sport/world-cup-2026/2026/07/06/ismael-saibari-fitness-concern-for-morocco-ahead-of-france-world-cup-quarter-final-clash/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Jazz Chisholm Jr.</t>
+          <t>A'ja Wilson</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>New York Yankees (MLB)</t>
+          <t>Las Vegas Aces (WNBA)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Right toe discomfort, noticed jogging gingerly to first base after a fly out</t>
+          <t>Foot injury sustained in a game against the Chicago Sky</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Being monitored day-to-day; no IL move confirmed yet</t>
+          <t>Missed 3 games; coach Becky Hammon said she could have played if it were a playoff game, suggesting an imminent return</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2944,49 +2944,49 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Risk of losing Yankees' starting second baseman if it worsens</t>
+          <t>Aces without their All-Star forward/center for a short stretch, including a loss to Indiana</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Ranger Suarez</t>
+          <t>Caitlin Clark</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies (MLB)</t>
+          <t>Indiana Fever (WNBA)</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Left adductor tightness, pulled early from start vs. Angels</t>
+          <t>Aggravated back injury</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Undetermined, pending further evaluation</t>
+          <t>Has resumed practicing; no confirmed timeline yet for a game return</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2996,49 +2996,49 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Phillies could lose their 2026 AL All-Star-caliber starter from the rotation</t>
+          <t>Fever have played without their All-Star starting guard for an extended stretch</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Brandon Woodruff</t>
+          <t>Napheesa Collier</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers (MLB)</t>
+          <t>Minnesota Lynx (WNBA)</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Right shoulder inflammation</t>
+          <t>Offseason surgery on both ankles</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Placed on 15-day Injured List (minimum)</t>
+          <t>Has yet to play in the 2026 season; recently resumed practicing</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3048,49 +3048,49 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Brewers rotation loses a top starter for at least two full turns</t>
+          <t>Lynx have been without their All-Star forward for the entire season to date</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Covers - MLB Injuries 2026</t>
+          <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://www.covers.com/sport/baseball/mlb/injuries</t>
+          <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Triston Casas</t>
+          <t>Lexi Thompson</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Boston Red Sox (MLB)</t>
+          <t>LPGA Tour</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Golf</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Torn right patellar tendon (out since May); recently shut down from hitting progression</t>
+          <t>Persistent hip pain/suspected hip injury</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Likely season-ending; setback in rehab timeline</t>
+          <t>Withdrew from the KPMG Women's PGA Championship at Hazeltine National, after also sitting out the Meijer LPGA Classic with the same issue; no return timeline given</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3100,49 +3100,49 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Red Sox lose starting first baseman for the remainder of the 2026 season</t>
+          <t>Ends a 15-tournament appearance streak at the Women's PGA Championship, a run that included four career top-10 finishes; Carolina Chacarra took her place in the field</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
+          <t>Golf Digest - Lexi Thompson withdraws from KPMG Women's PGA Championship</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
+          <t>https://www.golfdigest.com/story/lexi-thompson-withdraws-kpmg-womens-pga-championship</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Olivia Miles</t>
+          <t>Byron Buxton</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Lynx (WNBA)</t>
+          <t>Minnesota Twins (MLB)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Calf strain suffered during a July 3 game vs. the New York Liberty, possibly linked to in-game cramping</t>
+          <t>Aggravated hip injury while being caught stealing in the 1st inning vs. Yankees</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Ruled out of the Lynx's game vs. Connecticut on July 6, the first game of her WNBA career she has missed; no firm timetable given, though signs point to a quick recovery</t>
+          <t>Day-to-day; had already missed 4 games earlier in the week with the same hip issue</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Costly absence for a Lynx team leaning on its rookie floor general; came a day after Miles was named a starter for the 2026 WNBA All-Star Game and while she remains a near-lock for Rookie of the Year (18.5 ppg, 4.8 rpg, 5.7 apg)</t>
+          <t>Twins lose their 2026 All-Star outfielder from the lineup for an undetermined stretch</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3162,39 +3162,39 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Olivia Miles sidelined Monday against Sun with calf injury</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/wnba/story/_/id/49287945/olivia-miles-sidelined-monday-sun-calf-injury</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Serena Williams</t>
+          <t>Jazz Chisholm Jr.</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>New York Yankees (MLB)</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Right knee injury tweaked at the end of the first set of her Wimbledon singles match against Maya Joint; postmatch video showed four syringes of fluid drained from the knee</t>
+          <t>Right toe discomfort, noticed jogging gingerly to first base after a fly out</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Withdrew from the Wimbledon doubles draw alongside sister Venus Williams; no return timeline given</t>
+          <t>Being monitored day-to-day; no IL move confirmed yet</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -3204,49 +3204,49 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Ends a highly anticipated comeback pairing with Venus Williams in doubles, coming during Serena's first singles match in nearly four years</t>
+          <t>Risk of losing Yankees' starting second baseman if it worsens</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>NBC News - Serena Williams withdraws from Wimbledon doubles competition after knee injury</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>https://www.nbcnews.com/sports/tennis/serena-williams-withdraws-wimbledon-rcna352965</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>James Maddison</t>
+          <t>Ranger Suarez</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Tottenham Hotspur (Premier League)</t>
+          <t>Philadelphia Phillies (MLB)</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>ACL reconstruction rehab (returning from tear)</t>
+          <t>Left adductor tightness, pulled early from start vs. Angels</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Ongoing; currently restricted to 20-25 minutes per match</t>
+          <t>Undetermined, pending further evaluation</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3256,101 +3256,101 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Spurs managing his minutes carefully, limiting his impact as a starter</t>
+          <t>Phillies could lose their 2026 AL All-Star-caliber starter from the rotation</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Seamus Power</t>
+          <t>Brandon Woodruff</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>PGA Tour</t>
+          <t>Milwaukee Brewers (MLB)</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Golf</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Recurrence of long-standing back and hip issues he has dealt with since 2023</t>
+          <t>Right shoulder inflammation</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Withdrew after an opening-round 6-over 77 at the John Deere Classic on July 2; no return timeline given</t>
+          <t>Placed on 15-day Injured List (minimum)</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Forfeits prize money and FedEx Cup points from the John Deere Classic</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Removes a two-time PGA Tour winner from the field partway through the event</t>
+          <t>Brewers rotation loses a top starter for at least two full turns</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Golfmagic - Two-time PGA Tour winner forced out of John Deere Classic as injury problems strike again</t>
+          <t>Covers - MLB Injuries 2026</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>https://www.golfmagic.com/tour/pga-tour/two-time-pga-tour-winner-forced-out-john-deere-classic-injury-problems-strike-again</t>
+          <t>https://www.covers.com/sport/baseball/mlb/injuries</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Nahikari Garcia</t>
+          <t>Triston Casas</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Denver Summit FC (NWSL)</t>
+          <t>Boston Red Sox (MLB)</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Season-ending knee (ACL) injury</t>
+          <t>Torn right patellar tendon (out since May); recently shut down from hitting progression</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Out for the remainder of the 2026 NWSL season</t>
+          <t>Likely season-ending; setback in rehab timeline</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3360,34 +3360,34 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Denver Summit FC lose a starter for the rest of the season</t>
+          <t>Red Sox lose starting first baseman for the remainder of the 2026 season</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Spotrac - 2026 NWSL Injured Tracker</t>
+          <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
+          <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Brandon Ingram</t>
+          <t>Olivia Miles</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Toronto Raptors (NBA)</t>
+          <t>Minnesota Lynx (WNBA)</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3397,12 +3397,12 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Recovering from offseason surgery (lower body)</t>
+          <t>Calf strain suffered during a July 3 game vs. the New York Liberty, possibly linked to in-game cramping</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Expected back for training camp, fall 2026</t>
+          <t>Ruled out of the Lynx's game vs. Connecticut on July 6, the first game of her WNBA career she has missed; no firm timetable given, though signs point to a quick recovery</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -3412,49 +3412,49 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Raptors plan around his absence through the offseason program</t>
+          <t>Costly absence for a Lynx team leaning on its rookie floor general; came a day after Miles was named a starter for the 2026 WNBA All-Star Game and while she remains a near-lock for Rookie of the Year (18.5 ppg, 4.8 rpg, 5.7 apg)</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Brandon Ingram Injury Update Provided by Raptors After Surgery</t>
+          <t>ESPN - Olivia Miles sidelined Monday against Sun with calf injury</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25426220-brandon-ingram-injury-update-provided-raptors-after-surgery-latest-timeline-2026-nba-season</t>
+          <t>https://www.espn.com/wnba/story/_/id/49287945/olivia-miles-sidelined-monday-sun-calf-injury</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Josh Giddey</t>
+          <t>Serena Williams</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Chicago Bulls (NBA)</t>
+          <t>WTA Tour</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Tennis</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Arthroscopic surgery on right ankle</t>
+          <t>Right knee injury tweaked at the end of the first set of her Wimbledon singles match against Maya Joint; postmatch video showed four syringes of fluid drained from the knee</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>~3 months to resume basketball activities; targeting training camp</t>
+          <t>Withdrew from the Wimbledon doubles draw alongside sister Venus Williams; no return timeline given</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3464,49 +3464,49 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Bulls lose a starting guard for the entire offseason program</t>
+          <t>Ends a highly anticipated comeback pairing with Venus Williams in doubles, coming during Serena's first singles match in nearly four years</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Josh Giddey Injury Update Provided by Bulls After Ankle Surgery</t>
+          <t>NBC News - Serena Williams withdraws from Wimbledon doubles competition after knee injury</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25427505-josh-giddey-injury-update-provided-bulls-after-ankle-surgery-latest-timeline-2026-nba-season</t>
+          <t>https://www.nbcnews.com/sports/tennis/serena-williams-withdraws-wimbledon-rcna352965</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Corey Seager</t>
+          <t>James Maddison</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Texas Rangers (MLB)</t>
+          <t>Tottenham Hotspur (Premier League)</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Recurrence of lower back inflammation; his third injured list stint of the 2026 season (previously missed time with the same back issue and with a concussion)</t>
+          <t>ACL reconstruction rehab (returning from tear)</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Placed on the 10-day injured list</t>
+          <t>Ongoing; currently restricted to 20-25 minutes per match</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -3516,101 +3516,101 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Rangers lose their star shortstop again, continuing a season of infield instability; Josh Smith recalled from Triple-A as replacement</t>
+          <t>Spurs managing his minutes carefully, limiting his impact as a starter</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>ESPN - Rangers' Corey Seager back on IL with lower back inflammation</t>
+          <t>Premier League club injury coverage</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49238350/rangers-corey-seager-back-il-lower-back-inflammation</t>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Brent Rooker</t>
+          <t>Seamus Power</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Athletics (MLB)</t>
+          <t>PGA Tour</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Baseball</t>
+          <t>Golf</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Cartilage tear in left knee, discovered during an examination at Stanford; requires season-ending surgery</t>
+          <t>Recurrence of long-standing back and hip issues he has dealt with since 2023</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Season-ending; hadn't played since June 8 and had been on the injured list since June 9</t>
+          <t>Withdrew after an opening-round 6-over 77 at the John Deere Classic on July 2; no return timeline given</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Forfeits prize money and FedEx Cup points from the John Deere Classic</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Athletics lose their two-time All-Star middle-of-the-order bat for the remainder of the 2026 season</t>
+          <t>Removes a two-time PGA Tour winner from the field partway through the event</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>ESPN - A's slugger Brent Rooker to have season-ending left knee surgery</t>
+          <t>Golfmagic - Two-time PGA Tour winner forced out of John Deere Classic as injury problems strike again</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/mlb/story/_/id/49244022/a-slugger-brent-rooker-season-ending-left-knee-surgery</t>
+          <t>https://www.golfmagic.com/tour/pga-tour/two-time-pga-tour-winner-forced-out-john-deere-classic-injury-problems-strike-again</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>JuJu Watkins</t>
+          <t>Nahikari Garcia</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>USC Trojans (NCAA Division I Women's Basketball)</t>
+          <t>Denver Summit FC (NWSL)</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Basketball</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Recovering from a torn ACL that cost her the entire 2025-26 season</t>
+          <t>Season-ending knee (ACL) injury</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Returned to the court roughly 14 months after the injury</t>
+          <t>Out for the remainder of the 2026 NWSL season</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -3620,34 +3620,34 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>USC gets back its star guard after a full season lost to the injury</t>
+          <t>Denver Summit FC lose a starter for the rest of the season</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Fox Sports - 2026-2027 College Basketball Offseason Buzz</t>
+          <t>Spotrac - 2026 NWSL Injured Tracker</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>https://www.foxsports.com/stories/college-basketball/college-basketball-2026-2027-buzz-news-injuries-transfers</t>
+          <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Donnie Freeman</t>
+          <t>Brandon Ingram</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>St. John's University (NCAA Division I Men's Basketball)</t>
+          <t>Toronto Raptors (NBA)</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3657,12 +3657,12 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Torn right Achilles tendon, a non-contact injury suffered during a summer workout; underwent successful surgery performed by Dr. Martin O'Malley</t>
+          <t>Recovering from offseason surgery (lower body)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Will miss the entire 2026-27 season</t>
+          <t>Expected back for training camp, fall 2026</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Major setback for coach Rick Pitino and St. John's, who added the rising junior forward as a transfer-portal pickup this offseason; Freeman averaged 16.5 points and 7.2 rebounds last season at Syracuse</t>
+          <t>Raptors plan around his absence through the offseason program</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3682,24 +3682,24 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>The Washington Post - St. John's Donnie Freeman to miss next season following surgery on Achilles tendon</t>
+          <t>Bleacher Report - Brandon Ingram Injury Update Provided by Raptors After Surgery</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://www.washingtonpost.com/sports/colleges/2026/07/01/st-johns-donnie-freeman-achilles-injury-pitino/81e54c60-75c4-11f1-b665-5f8be87f3787_story.html</t>
+          <t>https://bleacherreport.com/articles/25426220-brandon-ingram-injury-update-provided-raptors-after-surgery-latest-timeline-2026-nba-season</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Jaren Jackson Jr.</t>
+          <t>Josh Giddey</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Memphis Grizzlies (NBA)</t>
+          <t>Chicago Bulls (NBA)</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -3709,12 +3709,12 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Turf toe surgery (right foot)</t>
+          <t>Arthroscopic surgery on right ankle</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Re-evaluation in approximately 12 weeks</t>
+          <t>~3 months to resume basketball activities; targeting training camp</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -3724,49 +3724,49 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Grizzlies lose their All-Star big man through the offseason and possibly into training camp</t>
+          <t>Bulls lose a starting guard for the entire offseason program</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>NBA.com - Grizzlies' Jaren Jackson Jr. has surgery to repair turf toe injury</t>
+          <t>Bleacher Report - Josh Giddey Injury Update Provided by Bulls After Ankle Surgery</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>https://www.nba.com/news/memphis-grizzlies-jaren-jackson-jr-turf-toe-surgery</t>
+          <t>https://bleacherreport.com/articles/25427505-josh-giddey-injury-update-provided-bulls-after-ankle-surgery-latest-timeline-2026-nba-season</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Manuel Ugarte</t>
+          <t>Corey Seager</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Manchester United (Premier League) / Uruguay National Team</t>
+          <t>Texas Rangers (MLB)</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Knee ligament injury suffered vs. Spain at the World Cup; possible cruciate ligament (ACL) damage</t>
+          <t>Recurrence of lower back inflammation; his third injured list stint of the 2026 season (previously missed time with the same back issue and with a concussion)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Potentially several months if ACL is confirmed</t>
+          <t>Placed on the 10-day injured list</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -3776,49 +3776,49 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Would be a significant blow to Manchester United's midfield depth heading into 2026-27</t>
+          <t>Rangers lose their star shortstop again, continuing a season of infield instability; Josh Smith recalled from Triple-A as replacement</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>ESPN - Rangers' Corey Seager back on IL with lower back inflammation</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.espn.com/mlb/story/_/id/49238350/rangers-corey-seager-back-il-lower-back-inflammation</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Rodri</t>
+          <t>Brent Rooker</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Manchester City (Premier League)</t>
+          <t>Athletics (MLB)</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Baseball</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Undisclosed injury expected to require surgery after the World Cup</t>
+          <t>Cartilage tear in left knee, discovered during an examination at Stanford; requires season-ending surgery</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Out for the opening weeks of the 2026-27 season</t>
+          <t>Season-ending; hadn't played since June 8 and had been on the injured list since June 9</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -3828,34 +3828,34 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Manchester City to start the new season without their midfield anchor</t>
+          <t>Athletics lose their two-time All-Star middle-of-the-order bat for the remainder of the 2026 season</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>ESPN - A's slugger Brent Rooker to have season-ending left knee surgery</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.espn.com/mlb/story/_/id/49244022/a-slugger-brent-rooker-season-ending-left-knee-surgery</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Kelsey Plum</t>
+          <t>JuJu Watkins</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks (WNBA)</t>
+          <t>USC Trojans (NCAA Division I Women's Basketball)</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3865,12 +3865,12 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Lower leg injury</t>
+          <t>Recovering from a torn ACL that cost her the entire 2025-26 season</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Ruled out for at least 4 weeks as of late June; All-Star Game (July 25) status still to be decided</t>
+          <t>Returned to the court roughly 14 months after the injury</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -3880,49 +3880,49 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Sparks lose a starting guard through their All-Star break stretch</t>
+          <t>USC gets back its star guard after a full season lost to the injury</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Bleacher Report - Angel Reese, Kelsey Plum Headline 2026 WNBA All-Star Game Reserves</t>
+          <t>Fox Sports - 2026-2027 College Basketball Offseason Buzz</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://bleacherreport.com/articles/25452286-angel-reese-kelsey-plum-headline-2026-wnba-all-star-game-reserves-full-roster-announced</t>
+          <t>https://www.foxsports.com/stories/college-basketball/college-basketball-2026-2027-buzz-news-injuries-transfers</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Seth Jarvis</t>
+          <t>Donnie Freeman</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Carolina Hurricanes (NHL)</t>
+          <t>St. John's University (NCAA Division I Men's Basketball)</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Hockey</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Shoulder surgery, the same shoulder that had a torn labrum and rotator cuff during the 2023-24 season</t>
+          <t>Torn right Achilles tendon, a non-contact injury suffered during a summer workout; underwent successful surgery performed by Dr. Martin O'Malley</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Expected recovery of approximately 4-6 months, meaning the earliest return would be late October</t>
+          <t>Will miss the entire 2026-27 season</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -3932,34 +3932,34 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Hurricanes will be without a top-six forward for the start of the 2026-27 season</t>
+          <t>Major setback for coach Rick Pitino and St. John's, who added the rising junior forward as a transfer-portal pickup this offseason; Freeman averaged 16.5 points and 7.2 rebounds last season at Syracuse</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>NHL.com - Jarvis expected to miss start of next season for Hurricanes after shoulder surgery</t>
+          <t>The Washington Post - St. John's Donnie Freeman to miss next season following surgery on Achilles tendon</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>https://www.nhl.com/news/seth-jarvis-to-miss-beginning-of-2026-2027-season-for-hurricanes-after-shoulder-surgery</t>
+          <t>https://www.washingtonpost.com/sports/colleges/2026/07/01/st-johns-donnie-freeman-achilles-injury-pitino/81e54c60-75c4-11f1-b665-5f8be87f3787_story.html</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Bradley Beal</t>
+          <t>Jaren Jackson Jr.</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>LA Clippers (NBA)</t>
+          <t>Memphis Grizzlies (NBA)</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -3969,12 +3969,12 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Hip fracture requiring season-ending surgery</t>
+          <t>Turf toe surgery (right foot)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Season-ending; recovery expected to extend into 2026-27 preseason</t>
+          <t>Re-evaluation in approximately 12 weeks</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -3984,86 +3984,86 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Clippers lose a veteran guard for the balance of the season and into next year's planning</t>
+          <t>Grizzlies lose their All-Star big man through the offseason and possibly into training camp</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>NBA.com - Clippers' Bradley Beal (hip) to undergo season-ending surgery</t>
+          <t>NBA.com - Grizzlies' Jaren Jackson Jr. has surgery to repair turf toe injury</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>https://www.nba.com/news/clippers-bradley-beal-out-season-hip-fracture</t>
+          <t>https://www.nba.com/news/memphis-grizzlies-jaren-jackson-jr-turf-toe-surgery</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Bejlek</t>
+          <t>Manuel Ugarte</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>Manchester United (Premier League) / Uruguay National Team</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Soccer</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Elbow injury</t>
+          <t>Knee ligament injury suffered vs. Spain at the World Cup; possible cruciate ligament (ACL) damage</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Withdrew mid-tournament from Eastbourne</t>
+          <t>Potentially several months if ACL is confirmed</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Forfeits Eastbourne prize money/points from the round of withdrawal</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Opponent Zeynep Sonmez advances by walkover</t>
+          <t>Would be a significant blow to Manchester United's midfield depth heading into 2026-27</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>RotoWire - Fantasy Tennis Injury News</t>
+          <t>Premier League club injury coverage</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Matthijs de Ligt</t>
+          <t>Rodri</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Manchester United (Premier League)</t>
+          <t>Manchester City (Premier League)</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -4073,12 +4073,12 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Surgery on a long-standing back injury</t>
+          <t>Undisclosed injury expected to require surgery after the World Cup</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Will miss the 2026 World Cup; club return timeline unconfirmed</t>
+          <t>Out for the opening weeks of the 2026-27 season</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -4088,12 +4088,12 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>United lose a starting center-back for an extended stretch</t>
+          <t>Manchester City to start the new season without their midfield anchor</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -4110,79 +4110,79 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Elina Svitolina</t>
+          <t>Kelsey Plum</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>WTA Tour</t>
+          <t>Los Angeles Sparks (WNBA)</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Tennis</t>
+          <t>Basketball</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Hip injury</t>
+          <t>Lower leg injury</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Withdrew before her Bad Homburg quarterfinal</t>
+          <t>Ruled out for at least 4 weeks as of late June; All-Star Game (July 25) status still to be decided</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Forfeits Bad Homburg quarterfinal prize money/points</t>
+          <t>Not disclosed in available reporting</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Opponent Xinyu Wang advances by walkover</t>
+          <t>Sparks lose a starting guard through their All-Star break stretch</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>RotoWire - Fantasy Tennis Injury News</t>
+          <t>Bleacher Report - Angel Reese, Kelsey Plum Headline 2026 WNBA All-Star Game Reserves</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+          <t>https://bleacherreport.com/articles/25452286-angel-reese-kelsey-plum-headline-2026-wnba-all-star-game-reserves-full-roster-announced</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Chris Richards</t>
+          <t>Seth Jarvis</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Crystal Palace (Premier League) / USMNT</t>
+          <t>Carolina Hurricanes (NHL)</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>Hockey</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Torn ankle ligaments (two ligaments) suffered vs. Brentford</t>
+          <t>Shoulder surgery, the same shoulder that had a torn labrum and rotator cuff during the 2023-24 season</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Expected to recover in time for the 2026 World Cup</t>
+          <t>Expected recovery of approximately 4-6 months, meaning the earliest return would be late October</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -4192,72 +4192,332 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Crystal Palace lose a starting center-back for a multi-week stretch</t>
+          <t>Hurricanes will be without a top-six forward for the start of the 2026-27 season</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>Premier League club injury coverage</t>
+          <t>NHL.com - Jarvis expected to miss start of next season for Hurricanes after shoulder surgery</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+          <t>https://www.nhl.com/news/seth-jarvis-to-miss-beginning-of-2026-2027-season-for-hurricanes-after-shoulder-surgery</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
+          <t>Bradley Beal</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>LA Clippers (NBA)</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Basketball</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Hip fracture requiring season-ending surgery</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Season-ending; recovery expected to extend into 2026-27 preseason</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Clippers lose a veteran guard for the balance of the season and into next year's planning</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>NBA.com - Clippers' Bradley Beal (hip) to undergo season-ending surgery</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nba.com/news/clippers-bradley-beal-out-season-hip-fracture</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Bejlek</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>WTA Tour</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Elbow injury</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Withdrew mid-tournament from Eastbourne</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Forfeits Eastbourne prize money/points from the round of withdrawal</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Opponent Zeynep Sonmez advances by walkover</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>RotoWire - Fantasy Tennis Injury News</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Matthijs de Ligt</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Manchester United (Premier League)</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Soccer</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Surgery on a long-standing back injury</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Will miss the 2026 World Cup; club return timeline unconfirmed</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>United lose a starting center-back for an extended stretch</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>Premier League club injury coverage</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Elina Svitolina</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>WTA Tour</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Hip injury</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Withdrew before her Bad Homburg quarterfinal</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Forfeits Bad Homburg quarterfinal prize money/points</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Opponent Xinyu Wang advances by walkover</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>RotoWire - Fantasy Tennis Injury News</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Chris Richards</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Crystal Palace (Premier League) / USMNT</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Soccer</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Torn ankle ligaments (two ligaments) suffered vs. Brentford</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Expected to recover in time for the 2026 World Cup</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Crystal Palace lose a starting center-back for a multi-week stretch</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>Premier League club injury coverage</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/latest-player-injuries</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
           <t>Chloe Ricketts</t>
         </is>
       </c>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>Boston Legacy FC (NWSL)</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>Soccer</t>
         </is>
       </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="D78" s="2" t="inlineStr">
         <is>
           <t>Ankle injury</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="E78" s="2" t="inlineStr">
         <is>
           <t>Placed on the 45-day short-term injury list</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>Not disclosed in available reporting</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr">
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Not disclosed in available reporting</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
         <is>
           <t>Boston Legacy FC without a rostered defender for at least 45 days</t>
         </is>
       </c>
-      <c r="H73" s="2" t="inlineStr">
+      <c r="H78" s="2" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr">
+      <c r="I78" s="2" t="inlineStr">
         <is>
           <t>Washington Spirit / NWSL transactions coverage</t>
         </is>
       </c>
-      <c r="J73" s="2" t="inlineStr">
+      <c r="J78" s="2" t="inlineStr">
         <is>
           <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
         </is>
@@ -4337,10 +4597,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId77"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId73"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId78"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Backfill financial_impact as prorated salary sunk cost for all 107 records
</commit_message>
<xml_diff>
--- a/injury_report.xlsx
+++ b/injury_report.xlsx
@@ -547,7 +547,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$2,281 prorated sunk cost (annual salary ~$277,500 per Spotrac ÷ 365 × 3 days out) [assumption: single-game absence, no timeline, day-to-day default]</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$13,020 prorated sunk cost (annual salary ~$678,882 (two-way) per Hoops Rumors ÷ 365 × 7 days out) [assumption: ruled out for remainder of NBA Summer League (~July 13-20); true post-surgery recovery likely longer but not specified]</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$78,272 prorated sunk cost (annual salary ~$9.52M per Spotrac ÷ 365 × 3 days out) [assumption: held out as precaution, no formal diagnosis/timeline, day-to-day default]</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Forfeits prize money and world ranking points from both events</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not disclosed in available reporting — salary not found</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not disclosed in available reporting — salary not found</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$18,942 prorated sunk cost (annual salary ~$493,851 per Spotrac ÷ 365 × 14 days out) [expected out at least two weeks]</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$246,575 prorated sunk cost (annual salary ~$9M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$32,305 prorated sunk cost (annual salary ~$786,100 per Spotrac ÷ 365 × 15 days out)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Forfeits prize money and FedEx Cup points from both events</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Forfeits ranking points and prize money from both events</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Forfeits ranking points and prize money from the event</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$1,553 prorated sunk cost (annual salary ~$113,400 per Capology ÷ 365 × 5 days out; no specific recovery timeline disclosed, conservative 5-day default used)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$30,822 prorated sunk cost (annual salary ~$2.25M per Capology ÷ 365 × 5 days out; no specific recovery timeline disclosed, conservative 5-day default used)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$64,658 prorated sunk cost (annual salary cap hit ~$200,000 per Capology ÷ 365 × 118 days out; days out estimated from date reported to 2026 MLS regular season end ~Nov 7)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$6,520 prorated sunk cost (annual salary ~$793,300 per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$166,685 prorated sunk cost (annual salary ~$780,000 per Spotrac ÷ 365 × 78 days out; possible season-ending surgery, days out estimated from date reported to MLB regular season end ~Sept 28)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Forfeits ranking points and prize money from both events</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$11,164 prorated sunk cost (annual salary ~$815K per Spotrac ÷ 365 × 5 days out) [assumption: concussion protocol with no return timeline, used 5-day undetermined default]</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$2,882 prorated sunk cost (annual salary ~$350,692 per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day questionable status]</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$153,425 prorated sunk cost (annual salary ~$1M per Spotrac ÷ 365 × 56 days out) [assumption: out since ~start of 2026 WNBA season (~May 16) through date reported (July 11), ~56 days]</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$4,021 prorated sunk cost (annual salary ~$293,510 per Spotrac ÷ 365 × 5 days out) [assumption: no return timeline, used 5-day undetermined default]</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$21,507 prorated sunk cost (annual salary ~$785K per Spotrac ÷ 365 × 10 days out) [10-day injured list stint]</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$194,178 prorated sunk cost (annual salary ~$4.725M per Spotrac ÷ 365 × 15 days out) [15-day injured list stint]</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$345,205 prorated sunk cost (annual salary ~$42M (contract AAV) per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day, not placed on IL, used 3-day estimate]</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$47,945 prorated sunk cost (annual salary ~$1.25M per Spotrac ÷ 365 × 14 days out) [assumption: 'reevaluated in the next couple of weeks' = 2 weeks]</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$172,603 prorated sunk cost (annual salary ~$1M base salary per Spotrac ÷ 365 × 63 days out) [8-10 week recovery timeline, used midpoint of 9 weeks = 63 days; excludes one-time signing bonus from prorated base]</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$65,205 prorated sunk cost (annual salary ~$850,000 per Spotrac ÷ 365 × 28 days out)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$356,164 prorated sunk cost (annual salary ~$13M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$86,747 prorated sunk cost (annual salary ~$6.33M per Spotrac ÷ 365 × 5 days out) [assumption: no firm return timeline reported, used 5-day undetermined default]</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$575,342 prorated sunk cost (annual salary ~$70M (contract AAV) per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day knee issue, skipping one start and the All-Star Game, no IL move reported]</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$106,925 prorated sunk cost (annual salary ~$3.9M per Spotrac ÷ 365 × 10 days out) [assumption: ruled out for entire 2026 NBA Summer League, ~July 10-20]</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$684,932 prorated sunk cost (annual salary ~$25M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$10,685 prorated sunk cost (annual salary ~$780,000 per Spotrac ÷ 365 × 5 days out; recovery timeline undisclosed, conservative 5-day default used)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not disclosed in available reporting — salary not found</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$547,945 prorated sunk cost (annual salary ~$40M per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$93,637 prorated sunk cost (annual salary ~$813,750 per Spotrac ÷ 365 × 42 days out)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$10,479 prorated sunk cost (annual salary ~$765,000 per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -3459,7 +3459,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not disclosed in available reporting — salary not found</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$8,219 prorated sunk cost (annual salary ~$1M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$85,479 prorated sunk cost (annual salary ~£10.4M (~$10.4M gross fixed wages) per Capology ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$102,740 prorated sunk cost (annual salary ~€12.5M gross (~$13.5M) per Capology ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -3667,7 +3667,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$32,055 prorated sunk cost (annual salary ~$780,000 MLB minimum per Spotrac ÷ 365 × 15 days out)</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$21,370 prorated sunk cost (annual salary ~$780,000 MLB minimum per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Forfeits prize money and Race to Dubai/world ranking points from both events</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$6,203,757 prorated sunk cost (annual salary ~$37.74M per Spotrac ÷ 365 × 60 days out)</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$6,414,378 prorated sunk cost (annual salary ~$9.76M per Capology (GBP→USD @1.34) ÷ 365 × 240 days out)</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$397,260 prorated sunk cost (annual salary ~$29.00M per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Forfeits ranking points and prize money from both the Gstaad and Kitzbuhel events</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -4135,7 +4135,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$7,562 prorated sunk cost (annual salary ~$920,000 per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Loses out on Wimbledon prize money and ranking points for the event</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$72,304 prorated sunk cost (annual salary ~$5.28M per Capology (EUR→USD @1.14) ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not disclosed in available reporting — salary not found</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$11,507 prorated sunk cost (annual salary ~$1.40M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$4,347 prorated sunk cost (annual salary ~$528,846 per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$11,507 prorated sunk cost (annual salary ~$1.4M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$8,219 prorated sunk cost (annual salary ~$300,000 per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$123,288 prorated sunk cost (annual salary ~$15.00M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$83,836 prorated sunk cost (annual salary ~$10.20M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -4759,7 +4759,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$95,890 prorated sunk cost (annual salary ~$7.00M per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -4811,7 +4811,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$905,137 prorated sunk cost (annual salary ~$22.02M per Spotrac ÷ 365 × 15 days out)</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -4863,7 +4863,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$374,932 prorated sunk cost (annual salary ~$1.61M per Spotrac ÷ 365 × 85 days out)</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$3,838 prorated sunk cost (annual salary ~$466,913 per Spotrac/On3 ÷ 365 × 3 days out) [assumption: day-to-day, signs point to quick recovery]</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -4967,7 +4967,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -5019,7 +5019,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$162,268 prorated sunk cost (annual salary ~$11.85M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -5071,7 +5071,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Forfeits prize money and FedEx Cup points from the John Deere Classic</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not disclosed in available reporting — salary not found</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$9,424,658 prorated sunk cost (annual salary ~$40.00M per Spotrac ÷ 365 × 86 days out)</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$6,164,384 prorated sunk cost (annual salary ~$25.00M per Spotrac ÷ 365 × 90 days out)</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -5279,7 +5279,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$849,315 prorated sunk cost (annual salary ~$31.00M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$1,463,014 prorated sunk cost (annual salary ~$6.00M per Spotrac ÷ 365 × 89 days out)</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -5383,7 +5383,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — NCAA athlete, no fixed salary</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not applicable — NCAA athlete, no fixed salary</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$4,068,493 prorated sunk cost (annual salary ~$4.5M per Spotrac ÷ 365 × 330 days out; 10-12 month recovery timeline, midpoint of 11 months used)</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -5539,7 +5539,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$10,632,329 prorated sunk cost (annual salary ~$46.20M per Spotrac ÷ 365 × 84 days out)</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$2,749,019 prorated sunk cost (annual salary ~$8.36M per Capology (GBP→USD @1.34) ÷ 365 × 120 days out)</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$881,977 prorated sunk cost (annual salary ~$15.33M per Capology (GBP→USD @1.34) ÷ 365 × 21 days out)</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$76,712 prorated sunk cost (annual salary ~$999,999 per Spotrac ÷ 365 × 28 days out)</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$3,246,575 prorated sunk cost (annual salary ~$7.9M AAV per Spotrac ÷ 365 × 150 days out)</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$1,416,976 prorated sunk cost (annual salary ~$5.62M per Spotrac ÷ 365 × 92 days out)</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Forfeits Eastbourne prize money/points from the round of withdrawal</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$185,397 prorated sunk cost (annual salary ~$13.53M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>Forfeits Bad Homburg quarterfinal prize money/points</t>
+          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -6007,7 +6007,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>$52,499 prorated sunk cost (annual salary ~$3.83M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting</t>
+          <t>Not disclosed in available reporting — salary not found</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add prize-money forfeiture to financial_impact for individual/tour sports; fix drifted daily target
</commit_message>
<xml_diff>
--- a/injury_report.xlsx
+++ b/injury_report.xlsx
@@ -819,7 +819,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not applicable — injury occurred during a completed, paid bout (referee stoppage), not a withdrawal from a future event, so no prize money was forfeited</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -3919,7 +3919,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -4539,7 +4539,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -4601,7 +4601,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -4663,7 +4663,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -5655,7 +5655,7 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>£40,000 (~$53,600) forfeited guaranteed prize money — 50% of the £80,000 first-round Wimbledon payout, per WTA withdrawal rules (per GB News / Tennis365)</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
@@ -6709,7 +6709,7 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr">
@@ -7825,7 +7825,7 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Not applicable — earns prize money/appearance fees, no fixed salary to prorate</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add tournament total prize purse as a labeled ceiling for un-forfeited prize-money records
</commit_message>
<xml_diff>
--- a/injury_report.xlsx
+++ b/injury_report.xlsx
@@ -819,7 +819,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €2,302,800 (~$2.6M) total tournament prize purse for the 2026 Tour de France (per Velo/Outside Online).</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $17.75M total tournament prize purse for the 2026 Open Championship at Royal Birkdale (per Forbes/PGA Tour).</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $8.8M total tournament prize purse for the 2026 John Deere Classic (per Golf Channel).</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €612,620 total tournament prize purse for the 2026 EFG Swiss Open Gstaad (per Perfect Tennis).</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $283,347 total tournament prize purse for the 2026 Athens Open (WTA 250) (per Perfect Tennis).</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €612,620 total tournament prize purse for the 2026 EFG Swiss Open Gstaad (per ATP Tour/Perfect Tennis).</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -3919,7 +3919,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): No prize purse — the World Athletics U20 Championships is a non-prize-money junior/development championship; World Athletics only awards prize money at senior-level events.</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €2,302,800 (~$2.6M) total prize fund for the 2026 Tour de France (per Domestique Cycling/Velo/Outside).</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -4539,7 +4539,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €2,302,800 (~$2.6M) total prize fund for the 2026 Tour de France (per Domestique Cycling/Velo/Outside).</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -4601,7 +4601,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €2,302,800 (~$2.6M) total prize fund for the 2026 Tour de France (per Domestique Cycling/Velo/Outside).</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -4663,7 +4663,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $9.42M total ATP prize money for the 2026 National Bank Open (Montreal) (per BetMGM Sports).</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): £64.2M (~$86.1M) total 2026 Wimbledon Championships prize money (per CBS Sports/ATP Tour) — this was a completed quarterfinal loss, not a withdrawal, so no forfeiture occurred.</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $17.75M total tournament prize purse for the 2026 Open Championship at Royal Birkdale (per CBS Sports/Forbes).</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €612,620 total prize money for the 2026 ATP Gstaad (Swiss Open), and €612,620 for the 2026 ATP Kitzbuhel (Generali Open) — both ATP 250 events he withdrew from (per ATP Tour/Perfect Tennis).</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $13M total tournament prize purse for the 2026 KPMG Women's PGA Championship at Hazeltine National (per Golf Channel/GolfDigest).</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): £64.2M (~$86.1M) total 2026 Wimbledon Championships prize money (per CBS Sports/ATP Tour) — she withdrew from the doubles draw specifically, not the whole event's purse.</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
@@ -6709,7 +6709,7 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $8.8M total tournament prize purse for the 2026 John Deere Classic (per Golf Channel/PGA Tour).</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $8.8M total tournament prize purse for the 2026 John Deere Classic (per Golf Channel).</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $499,000 total tournament prize purse for the 2026 Lexus Eastbourne Open (WTA 250) (per LTA/WTA reporting).</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr">
@@ -7825,7 +7825,7 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
+          <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $1.2M total tournament prize purse ($1,206,446 / €1,049,083) for the 2026 Bad Homburg Open (per Perfect Tennis/WTA).</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Fix missed salary lookups (Bedard, Saibari) and clarify structurally-confidential leagues
</commit_message>
<xml_diff>
--- a/injury_report.xlsx
+++ b/injury_report.xlsx
@@ -1501,7 +1501,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — salary not found</t>
+          <t>Not disclosed — individual Super Rugby Pacific player salaries are confidential (New Zealand Rugby publishes only general pay-band ranges, not player-specific figures)</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — salary not found</t>
+          <t>Not disclosed — individual Super Rugby Pacific player salaries are confidential (New Zealand Rugby publishes only general pay-band ranges, not player-specific figures)</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — salary not found</t>
+          <t>Not disclosed — Major League Cricket does not publicly release individual player salaries/signing terms</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -4787,7 +4787,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — salary not found</t>
+          <t>$312,329 prorated sunk cost (2025-26 entry-level contract cap hit ~$950,000 per Spotrac/Puckpedia ÷ 365 × 120 days out [~4-month recovery])</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — salary not found</t>
+          <t>$48,723 prorated sunk cost (annual base salary ~€5.2M / ~$5.93M per Capology (EUR→USD @1.14) ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — salary not found</t>
+          <t>Not disclosed — NWSL player salaries are confidential under the league/NWSLPA collective bargaining agreement and not publicly released</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr">
@@ -7949,7 +7949,7 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Not disclosed in available reporting — salary not found</t>
+          <t>Not disclosed — NWSL player salaries are confidential under the league/NWSLPA collective bargaining agreement and not publicly released</t>
         </is>
       </c>
       <c r="I121" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Split financial_impact into financial_impact_amount (number) and financial_impact_calculation (string)
</commit_message>
<xml_diff>
--- a/injury_report.xlsx
+++ b/injury_report.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -60,12 +62,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -145,9 +150,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Injuries" displayName="Injuries" ref="A1:L121" headerRowCount="1">
-  <autoFilter ref="A1:L121"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Injuries" displayName="Injuries" ref="A1:M121" headerRowCount="1">
+  <autoFilter ref="A1:M121"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="Athlete"/>
     <tableColumn id="2" name="Organization"/>
     <tableColumn id="3" name="Sport"/>
@@ -155,11 +160,12 @@
     <tableColumn id="5" name="League"/>
     <tableColumn id="6" name="Injury"/>
     <tableColumn id="7" name="Expected duration"/>
-    <tableColumn id="8" name="Financial impact"/>
-    <tableColumn id="9" name="Team/game impact"/>
-    <tableColumn id="10" name="Date reported"/>
-    <tableColumn id="11" name="Source"/>
-    <tableColumn id="12" name="Source URL"/>
+    <tableColumn id="8" name="Financial impact ($)"/>
+    <tableColumn id="9" name="Financial impact (calculation)"/>
+    <tableColumn id="10" name="Team/game impact"/>
+    <tableColumn id="11" name="Date reported"/>
+    <tableColumn id="12" name="Source"/>
+    <tableColumn id="13" name="Source URL"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -454,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L121"/>
+  <dimension ref="A1:M121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -464,11 +470,12 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -509,25 +516,30 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Financial impact</t>
+          <t>Financial impact ($)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Financial impact (calculation)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Team/game impact</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Date reported</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Source URL</t>
         </is>
@@ -569,27 +581,30 @@
           <t>Listed questionable for the Sky's July 16 game vs. the Seattle Storm; in danger of missing her first game of the season</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="n">
+        <v>706</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>$706 prorated sunk cost (annual salary ~$85,873 per Spotrac ÷ 365 × 3 days out) [questionable status, day-to-day default]</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Would be the first missed game of the season for the No. 3 overall 2024 pick if she sits; Elizabeth Williams poised for a spot start</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Athlon Sports - Final Injury Report for Storm-Sky: Will Kamilla Cardoso, Skylar Diggins Play?</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>https://athlonsports.com/wnba/chicago-sky/final-injury-report-for-storm-sky-will-kamilla-cardoso-skylar-diggins-play</t>
         </is>
@@ -631,27 +646,30 @@
           <t>Day-to-day; no injured list move reported following negative X-rays</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="n">
+        <v>6532</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>$6,532 prorated sunk cost (annual salary ~$794,800 per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Rays monitor their All-Star third baseman's availability for the second half after the All-Star Game scare</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>DraftKings Network - What happened to Junior Caminero? Injury updates for 2026 MLB All-Star Game</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>https://dknetwork.draftkings.com/2026/07/14/what-happened-to-junior-caminero-injury-updates-for-2026-mlb-all-star-game/</t>
         </is>
@@ -693,27 +711,30 @@
           <t>Not specified in available reporting; team confirmed rib contusion diagnosis a day after the injury</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="n">
+        <v>5579</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>$5,579 prorated sunk cost (annual salary ~$678,882 (two-way) per Hoops Rumors ÷ 365 × 3 days out) [assumption: no timeline given, day-to-day default]</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Jazz lose a newly-signed two-way guard for Summer League evaluation reps after a scary stretcher exit</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Yahoo Sports - Jazz guard Trey Alexander leaves Summer League game on stretcher with rib contusion</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://sports.yahoo.com/nba/breaking-news/article/jazz-guard-trey-alexander-leaves-summer-league-game-on-stretcher-with-rib-contusion-055652310.html</t>
         </is>
@@ -755,27 +776,28 @@
           <t>No diagnosis or return timeline disclosed; had been managing the issue throughout the World Cup</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Compounds France's growing injury list in a 0-2 semifinal defeat; replaced by Crystal Palace's Maxence Lacroix, with Arsenal also monitoring the issue heading into preseason</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>beIN Sports - William Saliba leaves the field injured and in tears during the 2026 World Cup semifinal between France and Spain</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://www.beinsports.com/en-us/soccer/fifa-world-cup-2026/articles/france-suffers-an-unexpected-blow-that-brings-back-a-painful-scene-from-the-last-world-cup-2026-07-14</t>
         </is>
@@ -817,27 +839,28 @@
           <t>Unable to start stage 11; withdrew from the Tour de France; recovery timeline not specified in available reporting</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €2,302,800 (~$2.6M) total tournament prize purse for the 2026 Tour de France (per Velo/Outside Online).</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Q36.5 Pro Cycling Team loses a rider mid-Tour after a dangerous descent that felled multiple riders</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>idlprocycling - Chris Harper withdraws from the Tour de France with a 'serious injury' after crash in same turn as Pidcock</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://www.idlprocycling.com/cycling/chris-harper-withdraws-from-the-tour-de-france-with-a-serious-injury-after-crash-in-same-turn-as-pidcock</t>
         </is>
@@ -879,27 +902,30 @@
           <t>Ruled out for the Aces' July 13 game vs. the Indiana Fever; no return timeline given</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="n">
+        <v>2281</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>$2,281 prorated sunk cost (annual salary ~$277,500 per Spotrac ÷ 365 × 3 days out) [assumption: single-game absence, no timeline, day-to-day default]</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Aces without a rotation forward who had recently moved into the starting lineup, adding to the team's list of unavailable players</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Yahoo Sports - Final Injury Report for Fever-Aces: Will Caitlin Clark Play?</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://sports.yahoo.com/articles/final-injury-report-fever-aces-210000827.html</t>
         </is>
@@ -941,27 +967,30 @@
           <t>Will undergo surgery; ruled out for the remainder of Summer League</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="3" t="n">
+        <v>13020</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>$13,020 prorated sunk cost (annual salary ~$678,882 (two-way) per Hoops Rumors ÷ 365 × 7 days out) [assumption: ruled out for remainder of NBA Summer League (~July 13-20); true post-surgery recovery likely longer but not specified]</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Magic lose their second-round pick's Summer League evaluation window</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>NBC Sports - Magic second-round pick Izaiyah Nelson will have surgery on ankle fracture suffered at Summer League</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://www.nbcsports.com/nba/news/magic-second-round-pick-izaiyah-nelson-will-have-surgery-on-ankle-fracture-suffered-at-summer-league</t>
         </is>
@@ -1003,27 +1032,30 @@
           <t>Did not return after halftime on July 13 vs. Portland; held out of the July 14 game vs. Chicago as the Jazz prioritize long-term health</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="3" t="n">
+        <v>78272</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>$78,272 prorated sunk cost (annual salary ~$9.52M per Spotrac ÷ 365 × 3 days out) [assumption: held out as precaution, no formal diagnosis/timeline, day-to-day default]</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Jazz hold their 2025 lottery pick out of further Summer League action out of caution</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>SI - Ace Bailey's Latest Injury Could End His Jazz Summer League Run</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://www.si.com/nba/jazz/onsi/ace-bailey-s-latest-injury-could-end-his-jazz-summer-league-run</t>
         </is>
@@ -1065,27 +1097,28 @@
           <t>Pulled from his scheduled bout with Jacobe Smith at UFC Oklahoma City (July 18); bout removed from the card</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>UFC.com - Updates To UFC Oklahoma City</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://www.ufc.com/news/updates-ufc-oklahoma-city</t>
         </is>
@@ -1127,27 +1160,28 @@
           <t>Pulled from her flyweight bout with Dione Barbosa at UFC Oklahoma City (July 18); replaced by Anna Melisano</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>UFC.com - Updates To UFC Oklahoma City</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://www.ufc.com/news/updates-ufc-oklahoma-city</t>
         </is>
@@ -1189,27 +1223,28 @@
           <t>Withdrew from the Glasgow 2026 Commonwealth Games (July 23-Aug 2), announced 10 days before the Games began</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Removes the three-time Olympic and 10-time Commonwealth Games medalist pommel horse specialist from Team England's squad</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Olympics.com - Max Whitlock withdraws from Glasgow 2026 Commonwealth Games with hand injury</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://www.olympics.com/en/news/max-whitlock-withdraws-glasgow-2026-commonwealth-games-with-hand-injury</t>
         </is>
@@ -1251,27 +1286,28 @@
           <t>Withdrew from The Open Championship at Royal Birkdale; also pulled out of next week's LIV Golf event at JCB Golf &amp; Country Club</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $17.75M total tournament prize purse for the 2026 Open Championship at Royal Birkdale (per Forbes/PGA Tour).</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Removes the 2010 Open champion from the 156-man field; Aldrich Potgieter promoted as first alternate</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Golf Monthly - Past Champion Louis Oosthuizen Forced To Withdraw From 2026 Open Due To Injury</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://www.golfmonthly.com/news/louis-oosthuizen-forced-to-withdraw-from-2026-open-due-to-injury</t>
         </is>
@@ -1313,27 +1349,28 @@
           <t>Ruled out of England's final Nations Championship match against Argentina in Santiago del Estero</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>England loses its first-choice scrum-half for the climax of the July tour</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>RugbyPass - Steve Borthwick confirms series-ending injury to take sheen off England win</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>https://www.rugbypass.com/news/injured-alex-mitchell-ruled-out-of-argentina-clash-after-england-hammer-fiji/</t>
         </is>
@@ -1375,27 +1412,28 @@
           <t>Withdrew from the final three days of the French Championships to continue treatment</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>His place at the European Aquatics Championships Paris 2026 (Aug 10-16) is not in doubt, as he has already qualified in one event</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>European Aquatics - Marchand withdraws from rest of French Championships to continue treatment on leg muscle injury</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://europeanaquatics.org/marchand-withdraws-from-rest-of-french-championships-to-continue-treatment-on-leg-muscle-injury/</t>
         </is>
@@ -1437,27 +1475,28 @@
           <t>Ruled out of France's remaining Nations Championship matches vs. Australia (July 13, Brisbane) and Japan (July 18, Tokyo)</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>France loses a starting winger for the rest of its Nations Championship campaign</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>NBC Sports - Injured Damian Penaud to miss France games against Australia and Japan in Nations Championship</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://www.nbcsports.com/rugby/news/injured-damian-penaud-to-miss-france-games-against-australia-and-japan-in-nations-championship</t>
         </is>
@@ -1499,27 +1538,28 @@
           <t>Availability for the Super Rugby Pacific Grand Final uncertain pending return-to-play protocols</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Not disclosed — individual Super Rugby Pacific player salaries are confidential (New Zealand Rugby publishes only general pay-band ranges, not player-specific figures)</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Hurricanes risk being without a forward for the Grand Final</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Super Rugby Pacific - Casualty Ward Super Rugby Pacific Grand Final</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://blog.draftrugby.com/p/casualty-ward-super-rugby-pacific-094</t>
         </is>
@@ -1561,27 +1601,28 @@
           <t>Listed as a doubt for the Super Rugby Pacific Grand Final despite hopes of being available</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Not disclosed — individual Super Rugby Pacific player salaries are confidential (New Zealand Rugby publishes only general pay-band ranges, not player-specific figures)</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>Chiefs risk being without a forward for the Grand Final</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Super Rugby Pacific - Casualty Ward Super Rugby Pacific Grand Final</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://blog.draftrugby.com/p/casualty-ward-super-rugby-pacific-094</t>
         </is>
@@ -1623,27 +1664,30 @@
           <t>Resumed throwing daily as of July 13; possible late-July return to the rotation</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="3" t="n">
+        <v>1109589</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>$1,109,589 prorated sunk cost (annual salary ~$27M per Spotrac ÷ 365 × 15 days out) [estimate: ~15 days from July 13 to a "late July" return target]</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>Yankees without a rotation starter for a portion of the stretch run, though a return is targeted before the end of the month</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>MLB.com - Baseball injury updates</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://www.mlb.com/news/baseball-injury-updates</t>
         </is>
@@ -1685,27 +1729,30 @@
           <t>Pulled from his rehab assignment; faces further evaluation before a return timeline is set, having already been out since May with the hernia</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" s="3" t="n">
+        <v>41096</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>$41,096 prorated sunk cost (annual salary ~$3.0M per Spotrac ÷ 365 × 5 days out) [undetermined additional recovery time following the rehab setback]</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Rays' return timeline for their outfielder is pushed back again, prolonging an IL stint that began in May</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Athlon Sports - Rays Player Suffers Unfortunate Injury Setback During Rehab Assignment</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>https://athlonsports.com/mlb/tampa-bay-rays/rays-jake-fraley-rehab-injury-setback</t>
         </is>
@@ -1747,27 +1794,30 @@
           <t>Expected out at least two weeks, to be reevaluated after that; coach indicated it could extend longer</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="3" t="n">
+        <v>18942</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>$18,942 prorated sunk cost (annual salary ~$493,851 per Spotrac ÷ 365 × 14 days out) [expected out at least two weeks]</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>Sparks lose their starting forward for at least two weeks; unrelated to her prior knee issues</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>ESPN - Sparks' Cameron Brink out undetermined time with ankle sprain</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/wnba/story/_/id/49098901/sparks-cameron-brink-undetermined-ankle-sprain</t>
         </is>
@@ -1809,27 +1859,30 @@
           <t>Placed on the 10-day injured list</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H22" s="3" t="n">
+        <v>246575</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>$246,575 prorated sunk cost (annual salary ~$9M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>Braves lose an outfield bat for at least 10 days</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>Yardbarker - 2026 Injury Report: Updates on Bichette, Lodolo, Misiorowski</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_bichette_lodolo_misiorowski/s1_17653_44053323</t>
         </is>
@@ -1871,27 +1924,30 @@
           <t>Placed on the 15-day injured list, retroactive to July 9</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H23" s="3" t="n">
+        <v>32305</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>$32,305 prorated sunk cost (annual salary ~$786,100 per Spotrac ÷ 365 × 15 days out)</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>Brewers lose a starting pitching option for at least 15 days</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>Yardbarker - 2026 Injury Report: Updates on Bichette, Lodolo, Misiorowski</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_bichette_lodolo_misiorowski/s1_17653_44053323</t>
         </is>
@@ -1933,27 +1989,28 @@
           <t>Withdrew from the John Deere Classic and the Genesis Scottish Open</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $8.8M total tournament prize purse for the 2026 John Deere Classic (per Golf Channel).</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>Heavy.com - $45 Million Golfer &amp; Multiple Others Abruptly Withdraw From Genesis Scottish Open</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>https://heavy.com/sports/golf/brooks-koepka-withdraw-jon-rahm-genesis-scottish-open/</t>
         </is>
@@ -1995,27 +2052,28 @@
           <t>Withdrew from the Swiss Open Gstaad; had already missed Wimbledon because of the injury</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €612,620 total tournament prize purse for the 2026 EFG Swiss Open Gstaad (per Perfect Tennis).</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>Last Word on Sports - Five Players Withdraw From the 2026 Swiss Open Gstaad</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>https://lastwordonsports.com/tennis/2026/07/12/five-players-withdraw-from-the-2026-swiss-open-gstaad/</t>
         </is>
@@ -2057,27 +2115,28 @@
           <t>Withdrew from WTA Athens to rest ahead of the second half of the season</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $283,347 total tournament prize purse for the 2026 Athens Open (WTA 250) (per Perfect Tennis).</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>Last Word on Sports - 15 Players Withdraw from WTA Athens and Iasi</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>https://lastwordonsports.com/tennis/2026/07/12/withdraw-wta-athens-iasi/</t>
         </is>
@@ -2119,27 +2178,30 @@
           <t>Will undergo surgery; out for an extended rehabilitation period</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H27" s="3" t="n">
+        <v>1553</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>$1,553 prorated sunk cost (annual salary ~$113,400 per Capology ÷ 365 × 5 days out; no specific recovery timeline disclosed, conservative 5-day default used)</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>NYCFC loses a defender for the remainder of the season</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>MLSsoccer.com - Player Availability Report</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>https://www.mlssoccer.com/news/mlssoccer-com-injury-report</t>
         </is>
@@ -2181,27 +2243,30 @@
           <t>Returning to the U.S. for surgery with Dr. Bert Mandelbaum; out for an extended period</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H28" s="3" t="n">
+        <v>30822</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>$30,822 prorated sunk cost (annual salary ~$2.25M per Capology ÷ 365 × 5 days out; no specific recovery timeline disclosed, conservative 5-day default used)</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Sounders and USMNT lose a veteran forward for an extended stretch</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>MLSsoccer.com - Player Availability Report</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>https://www.mlssoccer.com/news/mlssoccer-com-injury-report</t>
         </is>
@@ -2243,27 +2308,30 @@
           <t>Ruled out for the remainder of the 2026 season</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H29" s="3" t="n">
+        <v>64658</v>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>$64,658 prorated sunk cost (annual salary cap hit ~$200,000 per Capology ÷ 365 × 118 days out; days out estimated from date reported to 2026 MLS regular season end ~Nov 7)</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>Sounders lose a midfielder for the rest of the season</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>MLSsoccer.com - Player Availability Report</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>https://www.mlssoccer.com/news/mlssoccer-com-injury-report</t>
         </is>
@@ -2305,27 +2373,30 @@
           <t>Day-to-day after exiting his start on July 12</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H30" s="3" t="n">
+        <v>6520</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>$6,520 prorated sunk cost (annual salary ~$793,300 per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Mariners monitor a rotation piece heading toward the All-Star break</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>MLB.com - Latest Mariners injuries and transactions</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>https://www.mlb.com/news/mariners-injuries-and-roster-moves</t>
         </is>
@@ -2367,27 +2438,30 @@
           <t>Pulled from his rehab assignment due to pain; may require season-ending surgery</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H31" s="3" t="n">
+        <v>166685</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>$166,685 prorated sunk cost (annual salary ~$780,000 per Spotrac ÷ 365 × 78 days out; possible season-ending surgery, days out estimated from date reported to MLB regular season end ~Sept 28)</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Mariners' infield depth option now faces a possible lost season</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>MLB.com - Latest Mariners injuries and transactions</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>https://www.mlb.com/news/mariners-injuries-and-roster-moves</t>
         </is>
@@ -2429,27 +2503,28 @@
           <t>Withdrew from the Swiss Open Gstaad and a Challenger event in Germany</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €612,620 total tournament prize purse for the 2026 EFG Swiss Open Gstaad (per ATP Tour/Perfect Tennis).</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>Last Word on Sports - Five Players Withdraw From the 2026 Swiss Open Gstaad</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>https://lastwordonsports.com/tennis/2026/07/12/five-players-withdraw-from-the-2026-swiss-open-gstaad/</t>
         </is>
@@ -2491,27 +2566,30 @@
           <t>Expected to miss at least a month; season could be over if surgery is required</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H33" s="3" t="n">
+        <v>65178</v>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>$65,178 prorated sunk cost (annual salary ~$792,800 per Spotrac ÷ 365 × 30 days out) [estimate: 'at least a month' minimum]</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>Orioles lose a middle infielder for at least a month, with a risk of a season-ending outcome pending further evaluation</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>MLB Trade Rumors - Orioles' Blaze Alexander Suffers Fractured Hand On HBP</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>https://www.mlbtraderumors.com/2026/07/orioles-blaze-alexander-suffers-fractured-hand-on-hbp.html</t>
         </is>
@@ -2553,27 +2631,30 @@
           <t>Placed on the 15-day injured list, retroactive to July 9</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H34" s="3" t="n">
+        <v>905205</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>$905,205 prorated sunk cost (annual salary ~$22.025M per Spotrac ÷ 365 × 15 days out)</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>Diamondbacks lose their staff ace for at least two turns through the rotation</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>Arizona Sports - Diamondbacks place RHP Zac Gallen on 15-day IL, recall Mitch Bratt</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>https://arizonasports.com/mlb/arizona-diamondbacks/zac-gallen-15-day-il-recall-mitch-bratt</t>
         </is>
@@ -2615,27 +2696,30 @@
           <t>Downgraded from questionable to out; remains in concussion protocol with no return timeline given</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H35" s="3" t="n">
+        <v>11164</v>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>$11,164 prorated sunk cost (annual salary ~$815K per Spotrac ÷ 365 × 5 days out) [assumption: concussion protocol with no return timeline, used 5-day undetermined default]</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>Liberty without their All-Star forward for multiple games as she works through the NBA/WNBA-mandated concussion protocol; notable given she also missed time with a concussion in the 2025 WNBA Finals</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>Yahoo Sports - Liberty injury report: Star forward Satou Sabally in concussion protocol</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>https://sports.yahoo.com/articles/liberty-injury-report-star-forward-satou-sabally-in-concussion-protocol-224647068.html</t>
         </is>
@@ -2677,27 +2761,30 @@
           <t>Listed questionable for the Dream's game vs. the Portland Fire; no firm return timeline given</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H36" s="3" t="n">
+        <v>2882</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>$2,882 prorated sunk cost (annual salary ~$350,692 per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day questionable status]</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>Puts a third-straight All-Star selection and Dream's first year with Reese (acquired in an offseason trade from Chicago) at risk of interruption during a stretch where the team is trying to build momentum after a five-game losing streak</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>CBS Sports - Portland Fire vs. Atlanta Dream preview: Dream seek momentum as Angel Reese is questionable with leg injury</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>https://www.cbssports.com/wnba/news/portland-fire-atlanta-dream-where-to-watch-angel-reese-injury/</t>
         </is>
@@ -2739,27 +2826,30 @@
           <t>Ruled out to begin the 2026 season and remains sidelined into mid-July; not yet cleared for 5-on-5 drills and has no firm return timetable, though the team says she is expected to make a full recovery</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H37" s="3" t="n">
+        <v>153425</v>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>$153,425 prorated sunk cost (annual salary ~$1M per Spotrac ÷ 365 × 56 days out) [assumption: out since ~start of 2026 WNBA season (~May 16) through date reported (July 11), ~56 days]</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>Four-time All-Star center has yet to play a game for the Dream this season, a significant frontcourt loss to start the year</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>CBS News Atlanta - Atlanta Dream's Brionna Jones nearing return, expected back with team soon</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>https://www.cbsnews.com/atlanta/news/atlanta-dreams-brionna-jones-nearing-return-expected-back-with-team-next-week/</t>
         </is>
@@ -2801,27 +2891,30 @@
           <t>Ruled out for a second straight game, having missed her first game since May 25; no return timeline given</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H38" s="3" t="n">
+        <v>4021</v>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>$4,021 prorated sunk cost (annual salary ~$293,510 per Spotrac ÷ 365 × 5 days out) [assumption: no return timeline, used 5-day undetermined default]</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>Liberty forward sidelined for consecutive games amid a compressed schedule that includes a quick turnaround for a game in Toronto</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>Yahoo Sports - Final Injury Report for Liberty-Mystics: Will Satou Sabally, Leonie Fiebich Play?</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>https://sports.yahoo.com/articles/final-injury-report-liberty-mystics-150000047.html</t>
         </is>
@@ -2863,27 +2956,28 @@
           <t>Missed the Round of 16 win over Colombia and ruled out of the quarterfinal vs. Argentina; no return timeline given</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>Major blow to Switzerland's attack: with Manzambi on the pitch during the group stage the team averaged 3.6 goals per 90 minutes (3 goals, 2 assists for him in 200 minutes); without him, Switzerland have scored just once and averaged 1.4 xG per 90 over 280 minutes</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
         <is>
           <t>ESPN - Switzerland's Johan Manzambi to miss Argentina World Cup quarterfinal clash - Murat Yakin</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/soccer/story/_/id/49326340/switzerland-johan-manzambi-miss-argentina-world-cup-quarterfinal-clash-murat-yakin</t>
         </is>
@@ -2925,27 +3019,28 @@
           <t>Missed a training session in Kansas City but returned to training Friday and was confirmed available for the quarterfinal vs. Norway</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>Created a late fitness scare for England's back line ahead of the quarterfinal, with Newcastle's Dan Burn on standby to deputize had Guehi been unavailable</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>Sky Sports - World Cup 2026: England defender Marc Guehi a serious doubt for quarter-final clash with Norway</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>https://www.skysports.com/football/news/12016/13562168/world-cup-2026-england-defender-marc-guehi-a-serious-doubt-for-quarter-final-clash-with-norway</t>
         </is>
@@ -2987,27 +3082,30 @@
           <t>Placed on the 10-day injured list, retroactive to July 10</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H41" s="3" t="n">
+        <v>21507</v>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>$21,507 prorated sunk cost (annual salary ~$785K per Spotrac ÷ 365 × 10 days out) [10-day injured list stint]</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>Keeps the 2025 AL Rookie of the Year and scheduled AL All-Star starting first baseman (.266, 20 HR, 66 RBI, MLB-leading 76 walks) out of the July 14 All-Star Game in Philadelphia; catcher Brian Serven recalled from Triple-A in a corresponding move</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>ESPN - Athletics All-Star 1B Nick Kurtz placed on IL with thumb sprain</t>
         </is>
       </c>
-      <c r="L41" s="2" t="inlineStr">
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/mlb/story/_/id/49334996/athletics-all-star-1b-nick-kurtz-placed-il-thumb-sprain</t>
         </is>
@@ -3049,27 +3147,30 @@
           <t>Placed on the 15-day injured list; eligible to return July 27, though it could take longer depending on severity</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H42" s="3" t="n">
+        <v>194178</v>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>$194,178 prorated sunk cost (annual salary ~$4.725M per Spotrac ÷ 365 × 15 days out) [15-day injured list stint]</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>Reds turn to Rhett Lowder to fill Lodolo's rotation spot</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>MLB Trade Rumors - Reds Place Nick Lodolo On IL With Blister, Recall Chase Petty</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>https://www.mlbtraderumors.com/2026/07/reds-place-nick-lodolo-on-il-with-blister-recall-chase-petty.html</t>
         </is>
@@ -3111,27 +3212,30 @@
           <t>Held out of the lineup for a second straight game and available only off the bench; expected to use the following day and the All-Star break for a full reset rather than go on the injured list</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H43" s="3" t="n">
+        <v>345205</v>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>$345,205 prorated sunk cost (annual salary ~$42M (contract AAV) per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day, not placed on IL, used 3-day estimate]</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="J43" s="2" t="inlineStr">
         <is>
           <t>Mets manage his workload during a productive stretch (.320 avg, .788 OPS over his last 25 games) heading into the All-Star break</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="L43" s="2" t="inlineStr">
         <is>
           <t>Associated Press - Bo Bichette held out of Mets' lineup for second straight game with leg soreness</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr">
+      <c r="M43" s="2" t="inlineStr">
         <is>
           <t>https://www.bakersfield.com/ap/sports/bo-bichette-held-out-of-mets-lineup-for-second-straight-game-with-leg-soreness/article_c615803d-891c-57fd-87ef-b86becfaf8cc.html</t>
         </is>
@@ -3173,27 +3277,28 @@
           <t>Fight stopped by the referee at 1:09 of round one; no recovery timeline given pending formal diagnosis</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H44" s="2" t="n"/>
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>Not applicable — injury occurred during a completed, paid bout (referee stoppage), not a withdrawal from a future event, so no prize money was forfeited</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>Ends McGregor's much-hyped comeback fight against Max Holloway almost immediately and casts doubt on any near-term return to competition</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K44" s="2" t="inlineStr">
+      <c r="L44" s="2" t="inlineStr">
         <is>
           <t>NBC News - Conor McGregor suffers early knee injury in return, loses to Max Holloway at UFC 329</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr">
+      <c r="M44" s="2" t="inlineStr">
         <is>
           <t>https://www.nbcnews.com/sports/ufc/conor-mcgregor-suffers-early-knee-injury-return-loses-max-holloway-ufc-rcna552729</t>
         </is>
@@ -3235,27 +3340,30 @@
           <t>Ruled out of the Storm's game vs. the Washington Mystics; to be reevaluated in the next couple of weeks</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H45" s="3" t="n">
+        <v>47945</v>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>$47,945 prorated sunk cost (annual salary ~$1.25M per Spotrac ÷ 365 × 14 days out) [assumption: 'reevaluated in the next couple of weeks' = 2 weeks]</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>Storm without their starting center/forward for at least the near term</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K45" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t>Seattle Times - Ezi Magbegor to miss Seattle Storm's game vs. Washington Mystics with face injury</t>
         </is>
       </c>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="M45" s="2" t="inlineStr">
         <is>
           <t>https://www.seattletimes.com/sports/storm/ezi-magbegor-to-miss-seattle-storms-game-vs-washington-mystics-with-face-injury/</t>
         </is>
@@ -3297,27 +3405,30 @@
           <t>8-10 week recovery timeline; ineligible to return until at least September 4; team opted for a non-operative approach, splinting the hand for about six weeks before resuming baseball activities</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H46" s="3" t="n">
+        <v>172603</v>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>$172,603 prorated sunk cost (annual salary ~$1M base salary per Spotrac ÷ 365 × 63 days out) [8-10 week recovery timeline, used midpoint of 9 weeks = 63 days; excludes one-time signing bonus from prorated base]</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>Pirates lose their rookie starting shortstop (the No. 1 overall pick in the 2024 draft) for an extended stretch, his second significant injury of the season after an earlier forearm strain</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="L46" s="2" t="inlineStr">
         <is>
           <t>CBS Sports - Pirates' Konnor Griffin: Moved to 60-day IL</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="M46" s="2" t="inlineStr">
         <is>
           <t>https://www.cbssports.com/fantasy/baseball/news/pirates-konnor-griffin-moved-to-60-day-il/</t>
         </is>
@@ -3359,27 +3470,30 @@
           <t>On the 15-day IL since July 4; received a PRP injection on July 11 with re-evaluation in four weeks</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H47" s="3" t="n">
+        <v>65205</v>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>$65,205 prorated sunk cost (annual salary ~$850,000 per Spotrac ÷ 365 × 28 days out)</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>Giants lose a left-handed relief option for at least a month</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K47" s="2" t="inlineStr">
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>MLB.com - Latest Giants injuries &amp; transactions</t>
         </is>
       </c>
-      <c r="L47" s="2" t="inlineStr">
+      <c r="M47" s="2" t="inlineStr">
         <is>
           <t>https://www.mlb.com/news/giants-injuries-and-roster-moves</t>
         </is>
@@ -3421,27 +3535,30 @@
           <t>Placed on the 10-day injured list</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H48" s="3" t="n">
+        <v>356164</v>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>$356,164 prorated sunk cost (annual salary ~$13M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
         <is>
           <t>Angels lose their outfielder/DH for at least 10 days</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="L48" s="2" t="inlineStr">
         <is>
           <t>CBS Sports - Los Angeles Angels Injury Report and Status 2026</t>
         </is>
       </c>
-      <c r="L48" s="2" t="inlineStr">
+      <c r="M48" s="2" t="inlineStr">
         <is>
           <t>https://www.cbssports.com/mlb/teams/LAA/los-angeles-angels/injuries/</t>
         </is>
@@ -3483,27 +3600,30 @@
           <t>Ruled out of the Raptors' Summer League game vs. Houston on July 11; no firm return timeline given in available reporting</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H49" s="3" t="n">
+        <v>17961</v>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>$17,961 prorated sunk cost (annual salary ~$2.19M per Spotrac [2026-27 base salary on new 2-year deal] ÷ 365 × 3 days out) [assumption: single-game absence, no diagnosis timeline given, day-to-day default]</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr">
+      <c r="J49" s="2" t="inlineStr">
         <is>
           <t>Raptors without a rotation guard for Summer League evaluation reps, joining fellow injury absentee Collin Murray-Boyles on the sideline</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr">
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K49" s="2" t="inlineStr">
+      <c r="L49" s="2" t="inlineStr">
         <is>
           <t>Yardbarker - Collin Murray-Boyles, Alijah Martin to miss Raptors' Summer League opener</t>
         </is>
       </c>
-      <c r="L49" s="2" t="inlineStr">
+      <c r="M49" s="2" t="inlineStr">
         <is>
           <t>https://www.yardbarker.com/nba/articles/collin_murray_boyles_alijah_martin_to_miss_raptors_summer_league_opener/s1_17733_44049064</t>
         </is>
@@ -3545,27 +3665,30 @@
           <t>Substituted in the 77th minute as a precaution; completed training since and expected to be fully available for France's semifinal vs. Spain — described as day-to-day, no games missed</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H50" s="3" t="n">
+        <v>277397</v>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>$277,397 prorated sunk cost (annual salary ~€31.25M / ~$33.75M per Capology [EUR→USD @1.08] ÷ 365 × 3 days out) [day-to-day default; reporting indicates no games were actually missed]</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
         <is>
           <t>Described as a fitness scare for France ahead of the semifinal, but Mbappé and the team said there is no concern about his availability</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="K50" s="2" t="inlineStr">
+      <c r="L50" s="2" t="inlineStr">
         <is>
           <t>Forbes - Kylian Mbappé Injury Update Before France's World Cup Semi Vs. Spain</t>
         </is>
       </c>
-      <c r="L50" s="2" t="inlineStr">
+      <c r="M50" s="2" t="inlineStr">
         <is>
           <t>https://www.forbes.com/sites/brucelee/2026/07/11/kylian-mbapp-ankle-injury-update-before-frances-world-cup-semi-vs-spain/</t>
         </is>
@@ -3607,27 +3730,30 @@
           <t>Ruled out of the Raptors' Summer League opener vs. Boston; next possible return targeted for the Houston game; full recovery timeline not specified in available reporting</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H51" s="3" t="n">
+        <v>86747</v>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
         <is>
           <t>$86,747 prorated sunk cost (annual salary ~$6.33M per Spotrac ÷ 365 × 5 days out) [assumption: no firm return timeline reported, used 5-day undetermined default]</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr">
+      <c r="J51" s="2" t="inlineStr">
         <is>
           <t>Raptors lose their 2025 first-round pick (9th overall) for early Summer League reps as a point-forward, part of his developmental push</t>
         </is>
       </c>
-      <c r="J51" s="2" t="inlineStr">
+      <c r="K51" s="2" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="K51" s="2" t="inlineStr">
+      <c r="L51" s="2" t="inlineStr">
         <is>
           <t>Raptors Republic - Collin Murray-Boyles, Alijah Martin to miss Raptors' Summer League opener</t>
         </is>
       </c>
-      <c r="L51" s="2" t="inlineStr">
+      <c r="M51" s="2" t="inlineStr">
         <is>
           <t>https://raptorsrepublic.com/2026/07/10/collin-murray-boyles-alijah-martin-to-miss-raptors-summer-league-opener/</t>
         </is>
@@ -3669,27 +3795,30 @@
           <t>Scratched from his Friday, July 10 pitching start vs. Arizona and will skip the All-Star Game; scheduled to have the knee drained and possibly receive a pain-relieving injection during the break</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H52" s="3" t="n">
+        <v>575342</v>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
         <is>
           <t>$575,342 prorated sunk cost (annual salary ~$70M (contract AAV) per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day knee issue, skipping one start and the All-Star Game, no IL move reported]</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="J52" s="2" t="inlineStr">
         <is>
           <t>Dodgers manage the two-way star's workload heading into the second half; Ohtani continued to DH and homered the same day he was scratched from pitching</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="K52" s="2" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="K52" s="2" t="inlineStr">
+      <c r="L52" s="2" t="inlineStr">
         <is>
           <t>ESPN - Shohei Ohtani dealing with knee irritation, to miss All-Star Game</t>
         </is>
       </c>
-      <c r="L52" s="2" t="inlineStr">
+      <c r="M52" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/mlb/story/_/id/49327458/shohei-ohtani-dealing-knee-irritation-miss-all-star-game</t>
         </is>
@@ -3731,27 +3860,30 @@
           <t>Will sit out the entire 2026 NBA Summer League</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H53" s="3" t="n">
+        <v>106925</v>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
         <is>
           <t>$106,925 prorated sunk cost (annual salary ~$3.9M per Spotrac ÷ 365 × 10 days out) [assumption: ruled out for entire 2026 NBA Summer League, ~July 10-20]</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="J53" s="2" t="inlineStr">
         <is>
           <t>Spurs lose Summer League evaluation reps for their rookie</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr">
+      <c r="K53" s="2" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="K53" s="2" t="inlineStr">
+      <c r="L53" s="2" t="inlineStr">
         <is>
           <t>Yahoo Sports - San Antonio Spurs Rookie Jayden Quaintance to Sit Out 2026 Summer League</t>
         </is>
       </c>
-      <c r="L53" s="2" t="inlineStr">
+      <c r="M53" s="2" t="inlineStr">
         <is>
           <t>https://sports.yahoo.com/articles/san-antonio-spurs-rookie-jayden-184347004.html</t>
         </is>
@@ -3793,27 +3925,30 @@
           <t>On the 10-day IL since July 1; shut down through the weekend of July 10-12</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="H54" s="3" t="n">
+        <v>684932</v>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>$684,932 prorated sunk cost (annual salary ~$25M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr">
+      <c r="J54" s="2" t="inlineStr">
         <is>
           <t>Giants lose their starting third baseman for an extended stretch</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="K54" s="2" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="K54" s="2" t="inlineStr">
+      <c r="L54" s="2" t="inlineStr">
         <is>
           <t>MLB.com - Latest Giants injuries &amp; transactions</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr">
+      <c r="M54" s="2" t="inlineStr">
         <is>
           <t>https://www.mlb.com/news/giants-injuries-and-roster-moves</t>
         </is>
@@ -3855,27 +3990,30 @@
           <t>Diagnosed July 10; recovery timeline not yet disclosed</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H55" s="3" t="n">
+        <v>10685</v>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
         <is>
           <t>$10,685 prorated sunk cost (annual salary ~$780,000 per Spotrac ÷ 365 × 5 days out; recovery timeline undisclosed, conservative 5-day default used)</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr">
+      <c r="J55" s="2" t="inlineStr">
         <is>
           <t>Giants lose another outfield option amid multiple oblique injuries in the unit</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="K55" s="2" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="K55" s="2" t="inlineStr">
+      <c r="L55" s="2" t="inlineStr">
         <is>
           <t>MLB.com - Latest Giants injuries &amp; transactions</t>
         </is>
       </c>
-      <c r="L55" s="2" t="inlineStr">
+      <c r="M55" s="2" t="inlineStr">
         <is>
           <t>https://www.mlb.com/news/giants-injuries-and-roster-moves</t>
         </is>
@@ -3917,27 +4055,28 @@
           <t>Ruled out for the remainder of the 2026 season, including the World Athletics U20 Championships (Aug. 5-9, Eugene, Oregon); targeting a return in 2027</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H56" s="2" t="n"/>
+      <c r="I56" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): No prize purse — the World Athletics U20 Championships is a non-prize-money junior/development championship; World Athletics only awards prize money at senior-level events.</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr">
+      <c r="J56" s="2" t="inlineStr">
         <is>
           <t>Removes the U20 200m world record holder from an anticipated showdown with American Tate Taylor at the World U20 Championships</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr">
+      <c r="K56" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K56" s="2" t="inlineStr">
+      <c r="L56" s="2" t="inlineStr">
         <is>
           <t>Olympics.com - Gout Gout to miss World U20 Championships and rest of the season with hamstring injury</t>
         </is>
       </c>
-      <c r="L56" s="2" t="inlineStr">
+      <c r="M56" s="2" t="inlineStr">
         <is>
           <t>https://www.olympics.com/en/news/gout-gout-injury-hamstring-world-athletics-under-20-championships</t>
         </is>
@@ -3979,27 +4118,28 @@
           <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H57" s="2" t="n"/>
+      <c r="I57" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr">
+      <c r="J57" s="2" t="inlineStr">
         <is>
           <t>Deepens India's bowling injury crisis on the England tour, with Rana joining Varun Chakaravarthy, Hardik Pandya, and Nitish Kumar Reddy on the unavailable list</t>
         </is>
       </c>
-      <c r="J57" s="2" t="inlineStr">
+      <c r="K57" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K57" s="2" t="inlineStr">
+      <c r="L57" s="2" t="inlineStr">
         <is>
           <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
         </is>
       </c>
-      <c r="L57" s="2" t="inlineStr">
+      <c r="M57" s="2" t="inlineStr">
         <is>
           <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
         </is>
@@ -4041,27 +4181,28 @@
           <t>Ruled out of the remaining 4th and 5th T20Is of the series by the BCCI Medical Team</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H58" s="2" t="n"/>
+      <c r="I58" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
+      <c r="J58" s="2" t="inlineStr">
         <is>
           <t>India's frontline wrist-spinner is unavailable as the team's injury list grows on the England tour</t>
         </is>
       </c>
-      <c r="J58" s="2" t="inlineStr">
+      <c r="K58" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K58" s="2" t="inlineStr">
+      <c r="L58" s="2" t="inlineStr">
         <is>
           <t>IANS - 4th T20I: Injured Rana, Chakaravarthy ruled out of remaining games against England</t>
         </is>
       </c>
-      <c r="L58" s="2" t="inlineStr">
+      <c r="M58" s="2" t="inlineStr">
         <is>
           <t>https://ianslive.in/4th-t20i-injured-rana-chakaravarthy-ruled-out-of-remaining-games-against-england--20260709215924</t>
         </is>
@@ -4103,27 +4244,28 @@
           <t>Ruled out of the remainder of the ODI series vs. Zimbabwe; continuing rehab in Dhaka</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H59" s="2" t="n"/>
+      <c r="I59" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
+      <c r="J59" s="2" t="inlineStr">
         <is>
           <t>Bangladesh loses their starting wicketkeeper-batter for the series; Parvez Hossain Emon named as replacement for the 2nd and 3rd ODIs</t>
         </is>
       </c>
-      <c r="J59" s="2" t="inlineStr">
+      <c r="K59" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K59" s="2" t="inlineStr">
+      <c r="L59" s="2" t="inlineStr">
         <is>
           <t>The Nation - Injured Litton Das to miss rest of Zimbabwe ODI series</t>
         </is>
       </c>
-      <c r="L59" s="2" t="inlineStr">
+      <c r="M59" s="2" t="inlineStr">
         <is>
           <t>https://www.nation.com.pk/09-Jul-2026/injured-litton-das-miss-rest-zimbabwe-odi-series</t>
         </is>
@@ -4165,27 +4307,28 @@
           <t>Ruled out for the remainder of MLC 2026; replaced by Peter Siddle</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H60" s="2" t="n"/>
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>Not disclosed — Major League Cricket does not publicly release individual player salaries/signing terms</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
+      <c r="J60" s="2" t="inlineStr">
         <is>
           <t>Unicorns lose the veteran spinner after just one appearance this MLC season</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr">
+      <c r="K60" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K60" s="2" t="inlineStr">
+      <c r="L60" s="2" t="inlineStr">
         <is>
           <t>India TV News - Why is Ravichandran Ashwin ruled out of ongoing MLC 2026? San Francisco Unicorns announce replacement</t>
         </is>
       </c>
-      <c r="L60" s="2" t="inlineStr">
+      <c r="M60" s="2" t="inlineStr">
         <is>
           <t>https://www.indiatvnews.com/sports/cricket/why-is-ravichandran-ashwin-ruled-out-of-ongoing-mlc-2026-san-francisco-unicorns-announce-replacement-2026-07-09-1047737</t>
         </is>
@@ -4227,27 +4370,30 @@
           <t>Will have the rib reimaged during the All-Star break; no firm return date, GM Brian Cashman says he must be fully asymptomatic and show healing on imaging before resuming activity</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H61" s="3" t="n">
+        <v>547945</v>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
         <is>
           <t>$547,945 prorated sunk cost (annual salary ~$40M per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr">
+      <c r="J61" s="2" t="inlineStr">
         <is>
           <t>Yankees continue without their three-time AL MVP and captain in the middle of the lineup</t>
         </is>
       </c>
-      <c r="J61" s="2" t="inlineStr">
+      <c r="K61" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K61" s="2" t="inlineStr">
+      <c r="L61" s="2" t="inlineStr">
         <is>
           <t>ESPN - Yankees' Aaron Judge to have rib reimaged during All-Star break</t>
         </is>
       </c>
-      <c r="L61" s="2" t="inlineStr">
+      <c r="M61" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/mlb/story/_/id/49317023/yankees-aaron-judge-rib-reimaged-all-star-break</t>
         </is>
@@ -4289,27 +4435,30 @@
           <t>Headed to the injured list; broken bones of this type typically take around six weeks to heal, though the Mets have not given an official timeline and have not yet said whether surgery is needed</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H62" s="3" t="n">
+        <v>93637</v>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
         <is>
           <t>$93,637 prorated sunk cost (annual salary ~$813,750 per Spotrac ÷ 365 × 42 days out)</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr">
+      <c r="J62" s="2" t="inlineStr">
         <is>
           <t>Mets lose a regular infielder/DH (.211, 11 HR, 35 RBI in 72 games) just ahead of the trade deadline</t>
         </is>
       </c>
-      <c r="J62" s="2" t="inlineStr">
+      <c r="K62" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K62" s="2" t="inlineStr">
+      <c r="L62" s="2" t="inlineStr">
         <is>
           <t>amNewYork - Mark Vientos injury: Mets IF/DH headed to IL with hand fracture</t>
         </is>
       </c>
-      <c r="L62" s="2" t="inlineStr">
+      <c r="M62" s="2" t="inlineStr">
         <is>
           <t>https://www.amny.com/sports/mark-vientos-injury-mets-7-9-26/</t>
         </is>
@@ -4351,27 +4500,30 @@
           <t>Left the July 9 game early; scheduled for an MRI on July 10 to confirm the extent of the injury</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H63" s="3" t="n">
+        <v>10479</v>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
         <is>
           <t>$10,479 prorated sunk cost (annual salary ~$765,000 per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr">
+      <c r="J63" s="2" t="inlineStr">
         <is>
           <t>Athletics risk losing an everyday infielder/outfielder who had an on-base streak of 27 straight games and a 13-game scoring streak snapped by the injury</t>
         </is>
       </c>
-      <c r="J63" s="2" t="inlineStr">
+      <c r="K63" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K63" s="2" t="inlineStr">
+      <c r="L63" s="2" t="inlineStr">
         <is>
           <t>ESPN - Athletics' Gelof to have MRI on knee after sliding into fence</t>
         </is>
       </c>
-      <c r="L63" s="2" t="inlineStr">
+      <c r="M63" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/mlb/story/_/id/49319837/athletics-gelof-mri-knee-sliding-fence</t>
         </is>
@@ -4413,27 +4565,28 @@
           <t>Ruled out of the Women's ODI tour of Ireland beginning July 10; no return timeline disclosed</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H64" s="2" t="n"/>
+      <c r="I64" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr">
+      <c r="J64" s="2" t="inlineStr">
         <is>
           <t>West Indies lose their vice-captain and a key all-rounder; Realeanna Grimmond called up as her replacement for the Ireland series</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr">
+      <c r="K64" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K64" s="2" t="inlineStr">
+      <c r="L64" s="2" t="inlineStr">
         <is>
           <t>ESPNcricinfo - Realeanna Grimmond replaces injured Chinelle Henry in West Indies squad for Ireland Women's ODIs</t>
         </is>
       </c>
-      <c r="L64" s="2" t="inlineStr">
+      <c r="M64" s="2" t="inlineStr">
         <is>
           <t>https://www.espncricinfo.com/story/slug-1545066</t>
         </is>
@@ -4475,27 +4628,28 @@
           <t>Withdrew from the Tour de France (did not start stage 7); no return timeline specified in available reporting</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H65" s="2" t="n"/>
+      <c r="I65" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €2,302,800 (~$2.6M) total prize fund for the 2026 Tour de France (per Domestique Cycling/Velo/Outside).</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr">
+      <c r="J65" s="2" t="inlineStr">
         <is>
           <t>Uno-X Mobility loses the rider who had been wearing the race's yellow jersey after stage 5; Tadej Pogačar reclaimed the overall race lead the same day</t>
         </is>
       </c>
-      <c r="J65" s="2" t="inlineStr">
+      <c r="K65" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K65" s="2" t="inlineStr">
+      <c r="L65" s="2" t="inlineStr">
         <is>
           <t>Cyclingnews - 'Not the ending we wanted for this yellow adventure' - Torstein Træen out of Tour de France due to injuries from Tourmalet crash</t>
         </is>
       </c>
-      <c r="L65" s="2" t="inlineStr">
+      <c r="M65" s="2" t="inlineStr">
         <is>
           <t>https://www.cyclingnews.com/pro-cycling/teams-riders/not-the-ending-we-wanted-for-this-yellow-adventure-torstein-traeen-out-of-tour-de-france-due-to-injuries-from-tourmalet-crash/</t>
         </is>
@@ -4537,27 +4691,28 @@
           <t>Abandoned the Tour de France; did not start stage 6; recovery timeline not specified in available reporting</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H66" s="2" t="n"/>
+      <c r="I66" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €2,302,800 (~$2.6M) total prize fund for the 2026 Tour de France (per Domestique Cycling/Velo/Outside).</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr">
+      <c r="J66" s="2" t="inlineStr">
         <is>
           <t>Caja Rural-Seguros RGA loses a rider mid-Tour</t>
         </is>
       </c>
-      <c r="J66" s="2" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K66" s="2" t="inlineStr">
+      <c r="L66" s="2" t="inlineStr">
         <is>
           <t>Cycling Weekly - 'I don't remember the crash' – Caja Rural rider abandons Tour de France with fractured hand</t>
         </is>
       </c>
-      <c r="L66" s="2" t="inlineStr">
+      <c r="M66" s="2" t="inlineStr">
         <is>
           <t>https://www.cyclingweekly.com/racing/tour-de-france/i-dont-remember-the-crash-caja-rural-rider-abandons-tour-de-france-with-fractured-hand</t>
         </is>
@@ -4599,27 +4754,28 @@
           <t>Abandoned the Tour de France on stage 6 after struggling since the opening days; recovery timeline not specified in available reporting</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="H67" s="2" t="n"/>
+      <c r="I67" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €2,302,800 (~$2.6M) total prize fund for the 2026 Tour de France (per Domestique Cycling/Velo/Outside).</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr">
+      <c r="J67" s="2" t="inlineStr">
         <is>
           <t>Tudor Pro Cycling Team loses a rider mid-Tour after he battled to beat the time cut on multiple stages</t>
         </is>
       </c>
-      <c r="J67" s="2" t="inlineStr">
+      <c r="K67" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K67" s="2" t="inlineStr">
+      <c r="L67" s="2" t="inlineStr">
         <is>
           <t>idlprocycling - Suffering ends: Arvid de Kleijn and Cian Uijtdebroeks abandon Tour de France</t>
         </is>
       </c>
-      <c r="L67" s="2" t="inlineStr">
+      <c r="M67" s="2" t="inlineStr">
         <is>
           <t>https://www.idlprocycling.com/cycling/suffering-ends-arvid-de-kleijn-and-cian-uijtdebroeks-abandon-tour-de-france</t>
         </is>
@@ -4661,27 +4817,28 @@
           <t>Has pulled out of the ATP Montreal entry list and opted to prolong his comeback by two more weeks, targeting Cincinnati or the US Open for his return; recently resumed light on-court practice without a brace</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H68" s="2" t="n"/>
+      <c r="I68" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $9.42M total ATP prize money for the 2026 National Bank Open (Montreal) (per BetMGM Sports).</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr">
+      <c r="J68" s="2" t="inlineStr">
         <is>
           <t>World No. 2 has now missed a full clay and grass swing including two Grand Slams; absence continues into the North American hard-court season</t>
         </is>
       </c>
-      <c r="J68" s="2" t="inlineStr">
+      <c r="K68" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K68" s="2" t="inlineStr">
+      <c r="L68" s="2" t="inlineStr">
         <is>
           <t>Last Word On Tennis - Carlos Alcaraz Injury Update: Spaniard Pulls Out of ATP Montreal Entry List</t>
         </is>
       </c>
-      <c r="L68" s="2" t="inlineStr">
+      <c r="M68" s="2" t="inlineStr">
         <is>
           <t>https://lastwordonsports.com/tennis/2026/07/09/carlos-alcaraz-injury-update-spaniard-pulls-out-of-atp-montreal/</t>
         </is>
@@ -4723,27 +4880,30 @@
           <t>Out indefinitely; will be re-evaluated at the start of training camp in September, with availability for the 2026-27 season in question</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H69" s="3" t="n">
+        <v>616438</v>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
         <is>
           <t>$616,438 prorated sunk cost (annual salary ~$3.75M AAV per Spotrac ÷ 365 × 60 days out) [assumption: 60 days used as the near-term horizon to the September training-camp re-evaluation date; reporting indicates his full 2026-27 season could be at risk if complications persist, which would raise this figure substantially]</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
+      <c r="J69" s="2" t="inlineStr">
         <is>
           <t>Maple Leafs face uncertainty over a key veteran forward's availability for training camp and potentially the start of next season</t>
         </is>
       </c>
-      <c r="J69" s="2" t="inlineStr">
+      <c r="K69" s="2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="K69" s="2" t="inlineStr">
+      <c r="L69" s="2" t="inlineStr">
         <is>
           <t>NHL.com - Max Domi has 'complications' after surgery, out indefinitely for Maple Leafs</t>
         </is>
       </c>
-      <c r="L69" s="2" t="inlineStr">
+      <c r="M69" s="2" t="inlineStr">
         <is>
           <t>https://www.nhl.com/news/max-domi-has-complications-after-surgery-out-indefinitely-for-maple-leafs</t>
         </is>
@@ -4785,27 +4945,30 @@
           <t>Expected to need approximately four months to recover; will miss training camp and at least the start of the 2026-27 season</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="H70" s="3" t="n">
+        <v>312329</v>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
         <is>
           <t>$312,329 prorated sunk cost (2025-26 entry-level contract cap hit ~$950,000 per Spotrac/Puckpedia ÷ 365 × 120 days out [~4-month recovery])</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr">
+      <c r="J70" s="2" t="inlineStr">
         <is>
           <t>Blackhawks will open the 2026-27 season, played under the NHL's expanded 84-game schedule, without their No. 1 center for at least the opening month</t>
         </is>
       </c>
-      <c r="J70" s="2" t="inlineStr">
+      <c r="K70" s="2" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="K70" s="2" t="inlineStr">
+      <c r="L70" s="2" t="inlineStr">
         <is>
           <t>NHL.com - Bedard to miss start of 2026-27 season for Blackhawks after shoulder surgery</t>
         </is>
       </c>
-      <c r="L70" s="2" t="inlineStr">
+      <c r="M70" s="2" t="inlineStr">
         <is>
           <t>https://www.nhl.com/news/connor-bedard-injury-status-update-july-8-2026</t>
         </is>
@@ -4847,27 +5010,30 @@
           <t>Listed out for the Fever's game vs. the LA Sparks; expected to be available for the following game vs. Phoenix</t>
         </is>
       </c>
-      <c r="H71" s="2" t="inlineStr">
+      <c r="H71" s="3" t="n">
+        <v>8219</v>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
         <is>
           <t>$8,219 prorated sunk cost (annual salary ~$1M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr">
+      <c r="J71" s="2" t="inlineStr">
         <is>
           <t>Fever forced to manage the availability of both Boston and Caitlin Clark during a back-to-back stretch; Boston, a voted-in 2026 All-Star starter, is having a career-best scoring season (17.1 ppg on 50.4% shooting) and was in danger of missing her first game since May 17</t>
         </is>
       </c>
-      <c r="J71" s="2" t="inlineStr">
+      <c r="K71" s="2" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="K71" s="2" t="inlineStr">
+      <c r="L71" s="2" t="inlineStr">
         <is>
           <t>Athlon Sports - Indiana Fever Announce Aliyah Boston Injury Update Before LA Sparks Game</t>
         </is>
       </c>
-      <c r="L71" s="2" t="inlineStr">
+      <c r="M71" s="2" t="inlineStr">
         <is>
           <t>https://athlonsports.com/wnba/indiana-fever/indiana-fever-announce-aliyah-boston-injury-update-la-sparks-game</t>
         </is>
@@ -4909,27 +5075,30 @@
           <t>Touch-and-go for England's July 11 World Cup quarterfinal vs. Norway; has missed England's last three matches and was the sole absentee from the team's final group training session, requiring final medical clearance just to be considered for the bench</t>
         </is>
       </c>
-      <c r="H72" s="2" t="inlineStr">
+      <c r="H72" s="3" t="n">
+        <v>85479</v>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
         <is>
           <t>$85,479 prorated sunk cost (annual salary ~£10.4M (~$10.4M gross fixed wages) per Capology ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I72" s="2" t="inlineStr">
+      <c r="J72" s="2" t="inlineStr">
         <is>
           <t>Compounds an England right-back crisis that worsened after Jarell Quansah's red card vs. Mexico, leaving manager Thomas Tuchel with very limited options at the position for the quarterfinal</t>
         </is>
       </c>
-      <c r="J72" s="2" t="inlineStr">
+      <c r="K72" s="2" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="K72" s="2" t="inlineStr">
+      <c r="L72" s="2" t="inlineStr">
         <is>
           <t>Sky Sports - England World Cup latest: Reece James in race to be fit for quarter-final clash with Norway to ease right-back crisis</t>
         </is>
       </c>
-      <c r="L72" s="2" t="inlineStr">
+      <c r="M72" s="2" t="inlineStr">
         <is>
           <t>https://www.skysports.com/football/news/11095/13561150/england-world-cup-latest-reece-james-in-race-to-be-fit-for-quarter-final-clash-with-norway-to-ease-right-back-crisis</t>
         </is>
@@ -4971,27 +5140,30 @@
           <t>Missed France's Round of 16 win over Paraguay; returned to partial team training on July 8, with a decision on his availability for the July 11 quarterfinal vs. Morocco pending</t>
         </is>
       </c>
-      <c r="H73" s="2" t="inlineStr">
+      <c r="H73" s="3" t="n">
+        <v>102740</v>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
         <is>
           <t>$102,740 prorated sunk cost (annual salary ~€12.5M gross (~$13.5M) per Capology ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr">
+      <c r="J73" s="2" t="inlineStr">
         <is>
           <t>France's vice-captain and starting defensive midfielder is a doubt for the quarterfinal, with Manu Kone deputizing in his absence</t>
         </is>
       </c>
-      <c r="J73" s="2" t="inlineStr">
+      <c r="K73" s="2" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="K73" s="2" t="inlineStr">
+      <c r="L73" s="2" t="inlineStr">
         <is>
           <t>Sportskeeda - France handed huge injury boost as star man returns to training ahead of FIFA World Cup Q/F against Morocco</t>
         </is>
       </c>
-      <c r="L73" s="2" t="inlineStr">
+      <c r="M73" s="2" t="inlineStr">
         <is>
           <t>https://www.sportskeeda.com/football/rumor-france-handed-huge-injury-boost-star-man-returns-training-ahead-fifa-world-cup-q-f-morocco-reports</t>
         </is>
@@ -5033,27 +5205,28 @@
           <t>Ruled out for four weeks, covering the remainder of Bangladesh's tour of Zimbabwe (concluding July 19), including the T20I series; has returned home for rehab</t>
         </is>
       </c>
-      <c r="H74" s="2" t="inlineStr">
+      <c r="H74" s="2" t="n"/>
+      <c r="I74" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr">
+      <c r="J74" s="2" t="inlineStr">
         <is>
           <t>Bangladesh lose a frontline pace bowler for the rest of the Zimbabwe tour</t>
         </is>
       </c>
-      <c r="J74" s="2" t="inlineStr">
+      <c r="K74" s="2" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="K74" s="2" t="inlineStr">
+      <c r="L74" s="2" t="inlineStr">
         <is>
           <t>ESPNcricinfo - Zim vs Ban: Mustafizur Rahman ruled out for four weeks with hamstring and knee injuries</t>
         </is>
       </c>
-      <c r="L74" s="2" t="inlineStr">
+      <c r="M74" s="2" t="inlineStr">
         <is>
           <t>https://www.espncricinfo.com/story/zim-vs-ban-mustafizur-rahman-ruled-out-for-four-weeks-with-hamstring-and-knee-injuries-1545065</t>
         </is>
@@ -5095,27 +5268,30 @@
           <t>Placed on 15-day IL July 8, retroactive to July 5</t>
         </is>
       </c>
-      <c r="H75" s="2" t="inlineStr">
+      <c r="H75" s="3" t="n">
+        <v>32055</v>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
         <is>
           <t>$32,055 prorated sunk cost (annual salary ~$780,000 MLB minimum per Spotrac ÷ 365 × 15 days out)</t>
         </is>
       </c>
-      <c r="I75" s="2" t="inlineStr">
+      <c r="J75" s="2" t="inlineStr">
         <is>
           <t>Twins lose a pitching option for at least 15 days</t>
         </is>
       </c>
-      <c r="J75" s="2" t="inlineStr">
+      <c r="K75" s="2" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="K75" s="2" t="inlineStr">
+      <c r="L75" s="2" t="inlineStr">
         <is>
           <t>MLB.com - Latest Twins injuries &amp; transactions</t>
         </is>
       </c>
-      <c r="L75" s="2" t="inlineStr">
+      <c r="M75" s="2" t="inlineStr">
         <is>
           <t>https://www.mlb.com/news/twins-injuries-and-roster-moves</t>
         </is>
@@ -5157,27 +5333,30 @@
           <t>Placed on 10-day IL July 8, retroactive to July 6</t>
         </is>
       </c>
-      <c r="H76" s="2" t="inlineStr">
+      <c r="H76" s="3" t="n">
+        <v>21370</v>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
         <is>
           <t>$21,370 prorated sunk cost (annual salary ~$780,000 MLB minimum per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr">
+      <c r="J76" s="2" t="inlineStr">
         <is>
           <t>Pirates lose their starting catcher for at least 10 days</t>
         </is>
       </c>
-      <c r="J76" s="2" t="inlineStr">
+      <c r="K76" s="2" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="K76" s="2" t="inlineStr">
+      <c r="L76" s="2" t="inlineStr">
         <is>
           <t>MLB Trade Rumors - Pirates Place Endy Rodriguez On Injured List</t>
         </is>
       </c>
-      <c r="L76" s="2" t="inlineStr">
+      <c r="M76" s="2" t="inlineStr">
         <is>
           <t>https://www.mlbtraderumors.com/2026/07/pirates-to-place-endy-rodriguez-on-injured-list.html</t>
         </is>
@@ -5219,27 +5398,28 @@
           <t>Played through the flare-up but lost the quarterfinal 6-4, 6-4, 6-2 to Alexander Zverev; no absence or further tournament withdrawal reported</t>
         </is>
       </c>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="H77" s="2" t="n"/>
+      <c r="I77" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): £64.2M (~$86.1M) total 2026 Wimbledon Championships prize money (per CBS Sports/ATP Tour) — this was a completed quarterfinal loss, not a withdrawal, so no forfeiture occurred.</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr">
+      <c r="J77" s="2" t="inlineStr">
         <is>
           <t>Eliminated from Wimbledon; dropped to No. 10 in the ATP Live Rankings</t>
         </is>
       </c>
-      <c r="J77" s="2" t="inlineStr">
+      <c r="K77" s="2" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="K77" s="2" t="inlineStr">
+      <c r="L77" s="2" t="inlineStr">
         <is>
           <t>ESPN - Taylor Fritz loses at Wimbledon after knee tendinitis flares up</t>
         </is>
       </c>
-      <c r="L77" s="2" t="inlineStr">
+      <c r="M77" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/tennis/story/_/id/49308826/taylor-fritz-loses-alexander-zverev-wimbledon-quarterfinals-knee-tendonitis-flares-up</t>
         </is>
@@ -5281,27 +5461,28 @@
           <t>Withdrew from the Genesis Scottish Open and The Open Championship at Royal Birkdale; announced an extended break from golf for rehabilitation, with no firm return timeline given</t>
         </is>
       </c>
-      <c r="H78" s="2" t="inlineStr">
+      <c r="H78" s="2" t="n"/>
+      <c r="I78" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $17.75M total tournament prize purse for the 2026 Open Championship at Royal Birkdale (per CBS Sports/Forbes).</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr">
+      <c r="J78" s="2" t="inlineStr">
         <is>
           <t>Removes the Australian, who had qualified for his third Open Championship appearance, from the year's final men's major</t>
         </is>
       </c>
-      <c r="J78" s="2" t="inlineStr">
+      <c r="K78" s="2" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="K78" s="2" t="inlineStr">
+      <c r="L78" s="2" t="inlineStr">
         <is>
           <t>Today's Golfer - LIV Golf star withdraws on the eve of The Open</t>
         </is>
       </c>
-      <c r="L78" s="2" t="inlineStr">
+      <c r="M78" s="2" t="inlineStr">
         <is>
           <t>https://www.todays-golfer.com/news-and-events/majors/the-open-championship/elvis-smylie-liv-golf-withdrawal/</t>
         </is>
@@ -5343,27 +5524,30 @@
           <t>At least two months of rehab expected; targeting readiness for the start of the 2026-27 NBA season</t>
         </is>
       </c>
-      <c r="H79" s="2" t="inlineStr">
+      <c r="H79" s="3" t="n">
+        <v>6203757</v>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
         <is>
           <t>$6,203,757 prorated sunk cost (annual salary ~$37.74M per Spotrac ÷ 365 × 60 days out)</t>
         </is>
       </c>
-      <c r="I79" s="2" t="inlineStr">
+      <c r="J79" s="2" t="inlineStr">
         <is>
           <t>Reigning Finals MVP and starting point guard sidelined for part of the offseason program, though expected back for training camp</t>
         </is>
       </c>
-      <c r="J79" s="2" t="inlineStr">
+      <c r="K79" s="2" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="K79" s="2" t="inlineStr">
+      <c r="L79" s="2" t="inlineStr">
         <is>
           <t>Yahoo Sports - Knicks superstar Jalen Brunson undergoes left wrist surgery, expected to be ready for 2026-27 NBA season</t>
         </is>
       </c>
-      <c r="L79" s="2" t="inlineStr">
+      <c r="M79" s="2" t="inlineStr">
         <is>
           <t>https://sports.yahoo.com/nba/breaking-news/article/knicks-superstar-jalen-brunson-undergoes-left-wrist-surgery-expected-to-be-ready-for-2026-27-nba-season-155927234.html</t>
         </is>
@@ -5405,27 +5589,30 @@
           <t>Ruled out for the remainder of the World Cup; reported to be facing up to eight months out</t>
         </is>
       </c>
-      <c r="H80" s="2" t="inlineStr">
+      <c r="H80" s="3" t="n">
+        <v>6414378</v>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
         <is>
           <t>$6,414,378 prorated sunk cost (annual salary ~$9.76M per Capology (GBP→USD @1.34) ÷ 365 × 240 days out)</t>
         </is>
       </c>
-      <c r="I80" s="2" t="inlineStr">
+      <c r="J80" s="2" t="inlineStr">
         <is>
           <t>Belgium loses a key defensive midfielder ahead of their World Cup quarterfinal vs. Spain, and Aston Villa will be without him for a significant part of the 2026-27 season</t>
         </is>
       </c>
-      <c r="J80" s="2" t="inlineStr">
+      <c r="K80" s="2" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="K80" s="2" t="inlineStr">
+      <c r="L80" s="2" t="inlineStr">
         <is>
           <t>ESPN - Belgium's Amadou Onana out of World Cup after suffering ACL injury</t>
         </is>
       </c>
-      <c r="L80" s="2" t="inlineStr">
+      <c r="M80" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/soccer/story/_/id/49298508/belgium-amadou-onana-world-cup-suffering-acl-injury</t>
         </is>
@@ -5467,27 +5654,30 @@
           <t>No firm timeline; has not resumed running since the setback, no target return date given</t>
         </is>
       </c>
-      <c r="H81" s="2" t="inlineStr">
+      <c r="H81" s="3" t="n">
+        <v>397260</v>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
         <is>
           <t>$397,260 prorated sunk cost (annual salary ~$29.00M per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
-      <c r="I81" s="2" t="inlineStr">
+      <c r="J81" s="2" t="inlineStr">
         <is>
           <t>Yankees continue without their veteran slugger amid an offense that has struggled with injuries; manager Aaron Boone still expects him back at some point in 2026</t>
         </is>
       </c>
-      <c r="J81" s="2" t="inlineStr">
+      <c r="K81" s="2" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="K81" s="2" t="inlineStr">
+      <c r="L81" s="2" t="inlineStr">
         <is>
           <t>Last Word on Sports - Stanton Injury Update: Slugger Yet To Resume Rehab On Calf</t>
         </is>
       </c>
-      <c r="L81" s="2" t="inlineStr">
+      <c r="M81" s="2" t="inlineStr">
         <is>
           <t>https://lastwordonsports.com/baseball/2026/07/07/nyy-stanton-injury-update/</t>
         </is>
@@ -5529,27 +5719,28 @@
           <t>Withdrawing from the ATP tournaments in Gstaad and Kitzbuhel to rest on medical advice, with the goal of being ready for the US hard-court swing culminating in the US Open; no firm return date given</t>
         </is>
       </c>
-      <c r="H82" s="2" t="inlineStr">
+      <c r="H82" s="2" t="n"/>
+      <c r="I82" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): €612,620 total prize money for the 2026 ATP Gstaad (Swiss Open), and €612,620 for the 2026 ATP Kitzbuhel (Generali Open) — both ATP 250 events he withdrew from (per ATP Tour/Perfect Tennis).</t>
         </is>
       </c>
-      <c r="I82" s="2" t="inlineStr">
+      <c r="J82" s="2" t="inlineStr">
         <is>
           <t>Removes him from the draw at both tournaments immediately following his third-round Wimbledon loss to Grigor Dimitrov</t>
         </is>
       </c>
-      <c r="J82" s="2" t="inlineStr">
+      <c r="K82" s="2" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="K82" s="2" t="inlineStr">
+      <c r="L82" s="2" t="inlineStr">
         <is>
           <t>Puntodebreak - Berrettini withdraws from competing in upcoming tournaments due to "chronic hip pain"</t>
         </is>
       </c>
-      <c r="L82" s="2" t="inlineStr">
+      <c r="M82" s="2" t="inlineStr">
         <is>
           <t>https://www.puntodebreak.com/en/2026/07/07/berrettini-withdraws-from-competing-in-upcoming-tournaments-due-to-chronic-hip-pain</t>
         </is>
@@ -5591,27 +5782,30 @@
           <t>Ruled out for the July 7 game vs. Phoenix Mercury; no return timeline given</t>
         </is>
       </c>
-      <c r="H83" s="2" t="inlineStr">
+      <c r="H83" s="3" t="n">
+        <v>7562</v>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
         <is>
           <t>$7,562 prorated sunk cost (annual salary ~$920,000 per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I83" s="2" t="inlineStr">
+      <c r="J83" s="2" t="inlineStr">
         <is>
           <t>Comes as Diggins was moved to the bench for the first time in a decade, ending a streak of 341 consecutive starts; Sky beat Phoenix 77-66 in her absence</t>
         </is>
       </c>
-      <c r="J83" s="2" t="inlineStr">
+      <c r="K83" s="2" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="K83" s="2" t="inlineStr">
+      <c r="L83" s="2" t="inlineStr">
         <is>
           <t>Yahoo Sports - Sky's Skylar Diggins ruled out (knee) after being benched, Vandersloot starting</t>
         </is>
       </c>
-      <c r="L83" s="2" t="inlineStr">
+      <c r="M83" s="2" t="inlineStr">
         <is>
           <t>https://sports.yahoo.com/articles/skys-skylar-diggins-ruled-vs-010259203.html</t>
         </is>
@@ -5653,27 +5847,30 @@
           <t>Ruled out of Wimbledon 2026; still on crutches and wearing a protective boot several days after withdrawal, no return timeline given</t>
         </is>
       </c>
-      <c r="H84" s="2" t="inlineStr">
+      <c r="H84" s="3" t="n">
+        <v>53600</v>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
         <is>
           <t>£40,000 (~$53,600) forfeited guaranteed prize money — 50% of the £80,000 first-round Wimbledon payout, per WTA withdrawal rules (per GB News / Tennis365)</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr">
+      <c r="J84" s="2" t="inlineStr">
         <is>
           <t>Removes a top British draw from the tournament</t>
         </is>
       </c>
-      <c r="J84" s="2" t="inlineStr">
+      <c r="K84" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="K84" s="2" t="inlineStr">
+      <c r="L84" s="2" t="inlineStr">
         <is>
           <t>Yardbarker - Emma Raducanu setback deepens as British star remains on crutches after Wimbledon withdrawal</t>
         </is>
       </c>
-      <c r="L84" s="2" t="inlineStr">
+      <c r="M84" s="2" t="inlineStr">
         <is>
           <t>https://www.yardbarker.com/tennis/articles/emma_raducanu_setback_deepens_as_british_star_remains_on_crutches_after_wimbledon_withdrawal/s1_17460_44037038</t>
         </is>
@@ -5715,27 +5912,28 @@
           <t>Ruled out for the remainder of the 2026 World Cup; exact surgery date and recovery length not yet specified</t>
         </is>
       </c>
-      <c r="H85" s="2" t="inlineStr">
+      <c r="H85" s="2" t="n"/>
+      <c r="I85" s="2" t="inlineStr">
         <is>
           <t>Not applicable — no fixed salary information available for this national-team context</t>
         </is>
       </c>
-      <c r="I85" s="2" t="inlineStr">
+      <c r="J85" s="2" t="inlineStr">
         <is>
           <t>England advance to the quarterfinals without an experienced veteran midfielder, compounding a growing injury list</t>
         </is>
       </c>
-      <c r="J85" s="2" t="inlineStr">
+      <c r="K85" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="K85" s="2" t="inlineStr">
+      <c r="L85" s="2" t="inlineStr">
         <is>
           <t>ESPN - England's Henderson hospitalized with wrist injury during celebration</t>
         </is>
       </c>
-      <c r="L85" s="2" t="inlineStr">
+      <c r="M85" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/soccer/story/_/id/49283507/jordan-henderson-taken-hospital-wrist-injury-falling-mexico-victory-celebrations-england-world-cup</t>
         </is>
@@ -5777,27 +5975,30 @@
           <t>Not yet specified by club or national team</t>
         </is>
       </c>
-      <c r="H86" s="2" t="inlineStr">
+      <c r="H86" s="3" t="n">
+        <v>72304</v>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
         <is>
           <t>$72,304 prorated sunk cost (annual salary ~$5.28M per Capology (EUR→USD @1.14) ÷ 365 × 5 days out)</t>
         </is>
       </c>
-      <c r="I86" s="2" t="inlineStr">
+      <c r="J86" s="2" t="inlineStr">
         <is>
           <t>Injury compounds Mexico's World Cup elimination and raises concern over his fitness for AC Milan's preseason</t>
         </is>
       </c>
-      <c r="J86" s="2" t="inlineStr">
+      <c r="K86" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="K86" s="2" t="inlineStr">
+      <c r="L86" s="2" t="inlineStr">
         <is>
           <t>beIN Sports - Adding insult to injury! Santiago Gimenez suffers injury during Mexico's loss to England</t>
         </is>
       </c>
-      <c r="L86" s="2" t="inlineStr">
+      <c r="M86" s="2" t="inlineStr">
         <is>
           <t>https://www.beinsports.com/en-us/soccer/fifa-world-cup-2026/articles/adding-insult-to-injury-santiago-gimenez-suffers-injury-during-mexico-s-loss-to-england-2026-07-06</t>
         </is>
@@ -5839,27 +6040,30 @@
           <t>Day-to-day pending fitness test; final decision on availability for the World Cup quarterfinal vs. France expected only hours before kickoff</t>
         </is>
       </c>
-      <c r="H87" s="2" t="inlineStr">
+      <c r="H87" s="3" t="n">
+        <v>48723</v>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
         <is>
           <t>$48,723 prorated sunk cost (annual base salary ~€5.2M / ~$5.93M per Capology (EUR→USD @1.14) ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I87" s="2" t="inlineStr">
+      <c r="J87" s="2" t="inlineStr">
         <is>
           <t>Morocco risks losing their top attacking threat (three group-stage goals) for the biggest match of their World Cup run</t>
         </is>
       </c>
-      <c r="J87" s="2" t="inlineStr">
+      <c r="K87" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="K87" s="2" t="inlineStr">
+      <c r="L87" s="2" t="inlineStr">
         <is>
           <t>The National - Ismael Saibari fitness concern for Morocco ahead of France World Cup quarter-final clash</t>
         </is>
       </c>
-      <c r="L87" s="2" t="inlineStr">
+      <c r="M87" s="2" t="inlineStr">
         <is>
           <t>https://www.thenationalnews.com/sport/world-cup-2026/2026/07/06/ismael-saibari-fitness-concern-for-morocco-ahead-of-france-world-cup-quarter-final-clash/</t>
         </is>
@@ -5901,27 +6105,30 @@
           <t>Missed 3 games; coach Becky Hammon said she could have played if it were a playoff game, suggesting an imminent return</t>
         </is>
       </c>
-      <c r="H88" s="2" t="inlineStr">
+      <c r="H88" s="3" t="n">
+        <v>11507</v>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
         <is>
           <t>$11,507 prorated sunk cost (annual salary ~$1.40M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I88" s="2" t="inlineStr">
+      <c r="J88" s="2" t="inlineStr">
         <is>
           <t>Aces without their All-Star forward/center for a short stretch, including a loss to Indiana</t>
         </is>
       </c>
-      <c r="J88" s="2" t="inlineStr">
+      <c r="K88" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="K88" s="2" t="inlineStr">
+      <c r="L88" s="2" t="inlineStr">
         <is>
           <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
-      <c r="L88" s="2" t="inlineStr">
+      <c r="M88" s="2" t="inlineStr">
         <is>
           <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
@@ -5963,27 +6170,30 @@
           <t>Has resumed practicing; no confirmed timeline yet for a game return</t>
         </is>
       </c>
-      <c r="H89" s="2" t="inlineStr">
+      <c r="H89" s="3" t="n">
+        <v>4347</v>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
         <is>
           <t>$4,347 prorated sunk cost (annual salary ~$528,846 per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I89" s="2" t="inlineStr">
+      <c r="J89" s="2" t="inlineStr">
         <is>
           <t>Fever have played without their All-Star starting guard for an extended stretch</t>
         </is>
       </c>
-      <c r="J89" s="2" t="inlineStr">
+      <c r="K89" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="K89" s="2" t="inlineStr">
+      <c r="L89" s="2" t="inlineStr">
         <is>
           <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
-      <c r="L89" s="2" t="inlineStr">
+      <c r="M89" s="2" t="inlineStr">
         <is>
           <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
@@ -6025,27 +6235,30 @@
           <t>Has yet to play in the 2026 season; recently resumed practicing</t>
         </is>
       </c>
-      <c r="H90" s="2" t="inlineStr">
+      <c r="H90" s="3" t="n">
+        <v>11507</v>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
         <is>
           <t>$11,507 prorated sunk cost (annual salary ~$1.4M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I90" s="2" t="inlineStr">
+      <c r="J90" s="2" t="inlineStr">
         <is>
           <t>Lynx have been without their All-Star forward for the entire season to date</t>
         </is>
       </c>
-      <c r="J90" s="2" t="inlineStr">
+      <c r="K90" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="K90" s="2" t="inlineStr">
+      <c r="L90" s="2" t="inlineStr">
         <is>
           <t>Northwest Arkansas Democrat-Gazette - Injuries taking toll throughout WNBA</t>
         </is>
       </c>
-      <c r="L90" s="2" t="inlineStr">
+      <c r="M90" s="2" t="inlineStr">
         <is>
           <t>https://www.nwaonline.com/news/2026/jul/07/injuries-taking-toll-throughout-wnba/</t>
         </is>
@@ -6087,27 +6300,28 @@
           <t>Withdrew from the KPMG Women's PGA Championship at Hazeltine National, after also sitting out the Meijer LPGA Classic with the same issue; no return timeline given</t>
         </is>
       </c>
-      <c r="H91" s="2" t="inlineStr">
+      <c r="H91" s="2" t="n"/>
+      <c r="I91" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $13M total tournament prize purse for the 2026 KPMG Women's PGA Championship at Hazeltine National (per Golf Channel/GolfDigest).</t>
         </is>
       </c>
-      <c r="I91" s="2" t="inlineStr">
+      <c r="J91" s="2" t="inlineStr">
         <is>
           <t>Ends a 15-tournament appearance streak at the Women's PGA Championship, a run that included four career top-10 finishes; Carolina Chacarra took her place in the field</t>
         </is>
       </c>
-      <c r="J91" s="2" t="inlineStr">
+      <c r="K91" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="K91" s="2" t="inlineStr">
+      <c r="L91" s="2" t="inlineStr">
         <is>
           <t>Golf Digest - Lexi Thompson withdraws from KPMG Women's PGA Championship</t>
         </is>
       </c>
-      <c r="L91" s="2" t="inlineStr">
+      <c r="M91" s="2" t="inlineStr">
         <is>
           <t>https://www.golfdigest.com/story/lexi-thompson-withdraws-kpmg-womens-pga-championship</t>
         </is>
@@ -6149,27 +6363,30 @@
           <t>Placed on the 10-day injured list, retroactive to July 6; expected return in the second half of the season</t>
         </is>
       </c>
-      <c r="H92" s="2" t="inlineStr">
+      <c r="H92" s="3" t="n">
+        <v>8219</v>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
         <is>
           <t>$8,219 prorated sunk cost (annual salary ~$300,000 per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
-      <c r="I92" s="2" t="inlineStr">
+      <c r="J92" s="2" t="inlineStr">
         <is>
           <t>Giants lose an outfielder for at least the minimum IL stint</t>
         </is>
       </c>
-      <c r="J92" s="2" t="inlineStr">
+      <c r="K92" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="K92" s="2" t="inlineStr">
+      <c r="L92" s="2" t="inlineStr">
         <is>
           <t>MLB.com - Latest Giants injuries &amp; transactions</t>
         </is>
       </c>
-      <c r="L92" s="2" t="inlineStr">
+      <c r="M92" s="2" t="inlineStr">
         <is>
           <t>https://www.mlb.com/news/giants-injuries-and-roster-moves</t>
         </is>
@@ -6211,27 +6428,30 @@
           <t>Day-to-day; had already missed 4 games earlier in the week with the same hip issue</t>
         </is>
       </c>
-      <c r="H93" s="2" t="inlineStr">
+      <c r="H93" s="3" t="n">
+        <v>123288</v>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
         <is>
           <t>$123,288 prorated sunk cost (annual salary ~$15.00M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I93" s="2" t="inlineStr">
+      <c r="J93" s="2" t="inlineStr">
         <is>
           <t>Twins lose their 2026 All-Star outfielder from the lineup for an undetermined stretch</t>
         </is>
       </c>
-      <c r="J93" s="2" t="inlineStr">
+      <c r="K93" s="2" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="K93" s="2" t="inlineStr">
+      <c r="L93" s="2" t="inlineStr">
         <is>
           <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
-      <c r="L93" s="2" t="inlineStr">
+      <c r="M93" s="2" t="inlineStr">
         <is>
           <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
@@ -6273,27 +6493,30 @@
           <t>Being monitored day-to-day; no IL move confirmed yet</t>
         </is>
       </c>
-      <c r="H94" s="2" t="inlineStr">
+      <c r="H94" s="3" t="n">
+        <v>83836</v>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
         <is>
           <t>$83,836 prorated sunk cost (annual salary ~$10.20M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
-      <c r="I94" s="2" t="inlineStr">
+      <c r="J94" s="2" t="inlineStr">
         <is>
           <t>Risk of losing Yankees' starting second baseman if it worsens</t>
         </is>
       </c>
-      <c r="J94" s="2" t="inlineStr">
+      <c r="K94" s="2" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="K94" s="2" t="inlineStr">
+      <c r="L94" s="2" t="inlineStr">
         <is>
           <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
-      <c r="L94" s="2" t="inlineStr">
+      <c r="M94" s="2" t="inlineStr">
         <is>
           <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
@@ -6335,27 +6558,30 @@
           <t>Undetermined, pending further evaluation</t>
         </is>
       </c>
-      <c r="H95" s="2" t="inlineStr">
+      <c r="H95" s="3" t="n">
+        <v>95890</v>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
         <is>
           <t>$95,890 prorated sunk cost (annual salary ~$7.00M per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
-      <c r="I95" s="2" t="inlineStr">
+      <c r="J95" s="2" t="inlineStr">
         <is>
           <t>Phillies could lose their 2026 AL All-Star-caliber starter from the rotation</t>
         </is>
       </c>
-      <c r="J95" s="2" t="inlineStr">
+      <c r="K95" s="2" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="K95" s="2" t="inlineStr">
+      <c r="L95" s="2" t="inlineStr">
         <is>
           <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
-      <c r="L95" s="2" t="inlineStr">
+      <c r="M95" s="2" t="inlineStr">
         <is>
           <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
@@ -6397,27 +6623,30 @@
           <t>Placed on 15-day Injured List (minimum)</t>
         </is>
       </c>
-      <c r="H96" s="2" t="inlineStr">
+      <c r="H96" s="3" t="n">
+        <v>905137</v>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
         <is>
           <t>$905,137 prorated sunk cost (annual salary ~$22.02M per Spotrac ÷ 365 × 15 days out)</t>
         </is>
       </c>
-      <c r="I96" s="2" t="inlineStr">
+      <c r="J96" s="2" t="inlineStr">
         <is>
           <t>Brewers rotation loses a top starter for at least two full turns</t>
         </is>
       </c>
-      <c r="J96" s="2" t="inlineStr">
+      <c r="K96" s="2" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="K96" s="2" t="inlineStr">
+      <c r="L96" s="2" t="inlineStr">
         <is>
           <t>Covers - MLB Injuries 2026</t>
         </is>
       </c>
-      <c r="L96" s="2" t="inlineStr">
+      <c r="M96" s="2" t="inlineStr">
         <is>
           <t>https://www.covers.com/sport/baseball/mlb/injuries</t>
         </is>
@@ -6459,27 +6688,30 @@
           <t>Likely season-ending; setback in rehab timeline</t>
         </is>
       </c>
-      <c r="H97" s="2" t="inlineStr">
+      <c r="H97" s="3" t="n">
+        <v>374932</v>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
         <is>
           <t>$374,932 prorated sunk cost (annual salary ~$1.61M per Spotrac ÷ 365 × 85 days out)</t>
         </is>
       </c>
-      <c r="I97" s="2" t="inlineStr">
+      <c r="J97" s="2" t="inlineStr">
         <is>
           <t>Red Sox lose starting first baseman for the remainder of the 2026 season</t>
         </is>
       </c>
-      <c r="J97" s="2" t="inlineStr">
+      <c r="K97" s="2" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="K97" s="2" t="inlineStr">
+      <c r="L97" s="2" t="inlineStr">
         <is>
           <t>Yardbarker - 2026 Injury Report: Updates on Buxton, Suarez, Chisholm Jr.</t>
         </is>
       </c>
-      <c r="L97" s="2" t="inlineStr">
+      <c r="M97" s="2" t="inlineStr">
         <is>
           <t>https://www.yardbarker.com/mlb/articles/2026_injury_report_updates_on_buxton_suarez_chisholm_jr/s1_17653_44031703</t>
         </is>
@@ -6521,27 +6753,30 @@
           <t>Ruled out of the Lynx's game vs. Connecticut on July 6, the first game of her WNBA career she has missed; no firm timetable given, though signs point to a quick recovery</t>
         </is>
       </c>
-      <c r="H98" s="2" t="inlineStr">
+      <c r="H98" s="3" t="n">
+        <v>3838</v>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
         <is>
           <t>$3,838 prorated sunk cost (annual salary ~$466,913 per Spotrac/On3 ÷ 365 × 3 days out) [assumption: day-to-day, signs point to quick recovery]</t>
         </is>
       </c>
-      <c r="I98" s="2" t="inlineStr">
+      <c r="J98" s="2" t="inlineStr">
         <is>
           <t>Costly absence for a Lynx team leaning on its rookie floor general; came a day after Miles was named a starter for the 2026 WNBA All-Star Game and while she remains a near-lock for Rookie of the Year (18.5 ppg, 4.8 rpg, 5.7 apg)</t>
         </is>
       </c>
-      <c r="J98" s="2" t="inlineStr">
+      <c r="K98" s="2" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="K98" s="2" t="inlineStr">
+      <c r="L98" s="2" t="inlineStr">
         <is>
           <t>ESPN - Olivia Miles sidelined Monday against Sun with calf injury</t>
         </is>
       </c>
-      <c r="L98" s="2" t="inlineStr">
+      <c r="M98" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/wnba/story/_/id/49287945/olivia-miles-sidelined-monday-sun-calf-injury</t>
         </is>
@@ -6583,27 +6818,28 @@
           <t>Withdrew from the Wimbledon doubles draw alongside sister Venus Williams; no return timeline given</t>
         </is>
       </c>
-      <c r="H99" s="2" t="inlineStr">
+      <c r="H99" s="2" t="n"/>
+      <c r="I99" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): £64.2M (~$86.1M) total 2026 Wimbledon Championships prize money (per CBS Sports/ATP Tour) — she withdrew from the doubles draw specifically, not the whole event's purse.</t>
         </is>
       </c>
-      <c r="I99" s="2" t="inlineStr">
+      <c r="J99" s="2" t="inlineStr">
         <is>
           <t>Ends a highly anticipated comeback pairing with Venus Williams in doubles, coming during Serena's first singles match in nearly four years</t>
         </is>
       </c>
-      <c r="J99" s="2" t="inlineStr">
+      <c r="K99" s="2" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="K99" s="2" t="inlineStr">
+      <c r="L99" s="2" t="inlineStr">
         <is>
           <t>NBC News - Serena Williams withdraws from Wimbledon doubles competition after knee injury</t>
         </is>
       </c>
-      <c r="L99" s="2" t="inlineStr">
+      <c r="M99" s="2" t="inlineStr">
         <is>
           <t>https://www.nbcnews.com/sports/tennis/serena-williams-withdraws-wimbledon-rcna352965</t>
         </is>
@@ -6645,27 +6881,30 @@
           <t>Ongoing; currently restricted to 20-25 minutes per match</t>
         </is>
       </c>
-      <c r="H100" s="2" t="inlineStr">
+      <c r="H100" s="3" t="n">
+        <v>162268</v>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
         <is>
           <t>$162,268 prorated sunk cost (annual salary ~$11.85M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
         </is>
       </c>
-      <c r="I100" s="2" t="inlineStr">
+      <c r="J100" s="2" t="inlineStr">
         <is>
           <t>Spurs managing his minutes carefully, limiting his impact as a starter</t>
         </is>
       </c>
-      <c r="J100" s="2" t="inlineStr">
+      <c r="K100" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="K100" s="2" t="inlineStr">
+      <c r="L100" s="2" t="inlineStr">
         <is>
           <t>Premier League club injury coverage</t>
         </is>
       </c>
-      <c r="L100" s="2" t="inlineStr">
+      <c r="M100" s="2" t="inlineStr">
         <is>
           <t>https://www.premierleague.com/en/latest-player-injuries</t>
         </is>
@@ -6707,27 +6946,28 @@
           <t>Withdrew after an opening-round 6-over 77 at the John Deere Classic on July 2; no return timeline given</t>
         </is>
       </c>
-      <c r="H101" s="2" t="inlineStr">
+      <c r="H101" s="2" t="n"/>
+      <c r="I101" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $8.8M total tournament prize purse for the 2026 John Deere Classic (per Golf Channel/PGA Tour).</t>
         </is>
       </c>
-      <c r="I101" s="2" t="inlineStr">
+      <c r="J101" s="2" t="inlineStr">
         <is>
           <t>Removes a two-time PGA Tour winner from the field partway through the event</t>
         </is>
       </c>
-      <c r="J101" s="2" t="inlineStr">
+      <c r="K101" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="K101" s="2" t="inlineStr">
+      <c r="L101" s="2" t="inlineStr">
         <is>
           <t>Golfmagic - Two-time PGA Tour winner forced out of John Deere Classic as injury problems strike again</t>
         </is>
       </c>
-      <c r="L101" s="2" t="inlineStr">
+      <c r="M101" s="2" t="inlineStr">
         <is>
           <t>https://www.golfmagic.com/tour/pga-tour/two-time-pga-tour-winner-forced-out-john-deere-classic-injury-problems-strike-again</t>
         </is>
@@ -6769,27 +7009,28 @@
           <t>Out for the remainder of the 2026 NWSL season</t>
         </is>
       </c>
-      <c r="H102" s="2" t="inlineStr">
+      <c r="H102" s="2" t="n"/>
+      <c r="I102" s="2" t="inlineStr">
         <is>
           <t>Not disclosed — NWSL player salaries are confidential under the league/NWSLPA collective bargaining agreement and not publicly released</t>
         </is>
       </c>
-      <c r="I102" s="2" t="inlineStr">
+      <c r="J102" s="2" t="inlineStr">
         <is>
           <t>Denver Summit FC lose a starter for the rest of the season</t>
         </is>
       </c>
-      <c r="J102" s="2" t="inlineStr">
+      <c r="K102" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="K102" s="2" t="inlineStr">
+      <c r="L102" s="2" t="inlineStr">
         <is>
           <t>Spotrac - 2026 NWSL Injured Tracker</t>
         </is>
       </c>
-      <c r="L102" s="2" t="inlineStr">
+      <c r="M102" s="2" t="inlineStr">
         <is>
           <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
         </is>
@@ -6831,27 +7072,28 @@
           <t>Withdrew from the John Deere Classic prior to the first round on July 2; no recovery timeline disclosed</t>
         </is>
       </c>
-      <c r="H103" s="2" t="inlineStr">
+      <c r="H103" s="2" t="n"/>
+      <c r="I103" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $8.8M total tournament prize purse for the 2026 John Deere Classic (per Golf Channel).</t>
         </is>
       </c>
-      <c r="I103" s="2" t="inlineStr">
+      <c r="J103" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting</t>
         </is>
       </c>
-      <c r="J103" s="2" t="inlineStr">
+      <c r="K103" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="K103" s="2" t="inlineStr">
+      <c r="L103" s="2" t="inlineStr">
         <is>
           <t>Golf Monthly - Pro Withdraws From John Deere Classic Hours Before First Round</t>
         </is>
       </c>
-      <c r="L103" s="2" t="inlineStr">
+      <c r="M103" s="2" t="inlineStr">
         <is>
           <t>https://www.golfmonthly.com/news/patrick-rodgers-withdraws-john-deere-classic-2026</t>
         </is>
@@ -6893,27 +7135,30 @@
           <t>Expected back for training camp, fall 2026</t>
         </is>
       </c>
-      <c r="H104" s="2" t="inlineStr">
+      <c r="H104" s="3" t="n">
+        <v>9424658</v>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
         <is>
           <t>$9,424,658 prorated sunk cost (annual salary ~$40.00M per Spotrac ÷ 365 × 86 days out)</t>
         </is>
       </c>
-      <c r="I104" s="2" t="inlineStr">
+      <c r="J104" s="2" t="inlineStr">
         <is>
           <t>Raptors plan around his absence through the offseason program</t>
         </is>
       </c>
-      <c r="J104" s="2" t="inlineStr">
+      <c r="K104" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="K104" s="2" t="inlineStr">
+      <c r="L104" s="2" t="inlineStr">
         <is>
           <t>Bleacher Report - Brandon Ingram Injury Update Provided by Raptors After Surgery</t>
         </is>
       </c>
-      <c r="L104" s="2" t="inlineStr">
+      <c r="M104" s="2" t="inlineStr">
         <is>
           <t>https://bleacherreport.com/articles/25426220-brandon-ingram-injury-update-provided-raptors-after-surgery-latest-timeline-2026-nba-season</t>
         </is>
@@ -6955,27 +7200,30 @@
           <t>~3 months to resume basketball activities; targeting training camp</t>
         </is>
       </c>
-      <c r="H105" s="2" t="inlineStr">
+      <c r="H105" s="3" t="n">
+        <v>6164384</v>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
         <is>
           <t>$6,164,384 prorated sunk cost (annual salary ~$25.00M per Spotrac ÷ 365 × 90 days out)</t>
         </is>
       </c>
-      <c r="I105" s="2" t="inlineStr">
+      <c r="J105" s="2" t="inlineStr">
         <is>
           <t>Bulls lose a starting guard for the entire offseason program</t>
         </is>
       </c>
-      <c r="J105" s="2" t="inlineStr">
+      <c r="K105" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="K105" s="2" t="inlineStr">
+      <c r="L105" s="2" t="inlineStr">
         <is>
           <t>Bleacher Report - Josh Giddey Injury Update Provided by Bulls After Ankle Surgery</t>
         </is>
       </c>
-      <c r="L105" s="2" t="inlineStr">
+      <c r="M105" s="2" t="inlineStr">
         <is>
           <t>https://bleacherreport.com/articles/25427505-josh-giddey-injury-update-provided-bulls-after-ankle-surgery-latest-timeline-2026-nba-season</t>
         </is>
@@ -7017,27 +7265,30 @@
           <t>Placed on the 10-day injured list</t>
         </is>
       </c>
-      <c r="H106" s="2" t="inlineStr">
+      <c r="H106" s="3" t="n">
+        <v>849315</v>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
         <is>
           <t>$849,315 prorated sunk cost (annual salary ~$31.00M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
-      <c r="I106" s="2" t="inlineStr">
+      <c r="J106" s="2" t="inlineStr">
         <is>
           <t>Rangers lose their star shortstop again, continuing a season of infield instability; Josh Smith recalled from Triple-A as replacement</t>
         </is>
       </c>
-      <c r="J106" s="2" t="inlineStr">
+      <c r="K106" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="K106" s="2" t="inlineStr">
+      <c r="L106" s="2" t="inlineStr">
         <is>
           <t>ESPN - Rangers' Corey Seager back on IL with lower back inflammation</t>
         </is>
       </c>
-      <c r="L106" s="2" t="inlineStr">
+      <c r="M106" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/mlb/story/_/id/49238350/rangers-corey-seager-back-il-lower-back-inflammation</t>
         </is>
@@ -7079,27 +7330,30 @@
           <t>Season-ending; hadn't played since June 8 and had been on the injured list since June 9</t>
         </is>
       </c>
-      <c r="H107" s="2" t="inlineStr">
+      <c r="H107" s="3" t="n">
+        <v>1463014</v>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
         <is>
           <t>$1,463,014 prorated sunk cost (annual salary ~$6.00M per Spotrac ÷ 365 × 89 days out)</t>
         </is>
       </c>
-      <c r="I107" s="2" t="inlineStr">
+      <c r="J107" s="2" t="inlineStr">
         <is>
           <t>Athletics lose their two-time All-Star middle-of-the-order bat for the remainder of the 2026 season</t>
         </is>
       </c>
-      <c r="J107" s="2" t="inlineStr">
+      <c r="K107" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="K107" s="2" t="inlineStr">
+      <c r="L107" s="2" t="inlineStr">
         <is>
           <t>ESPN - A's slugger Brent Rooker to have season-ending left knee surgery</t>
         </is>
       </c>
-      <c r="L107" s="2" t="inlineStr">
+      <c r="M107" s="2" t="inlineStr">
         <is>
           <t>https://www.espn.com/mlb/story/_/id/49244022/a-slugger-brent-rooker-season-ending-left-knee-surgery</t>
         </is>
@@ -7141,27 +7395,28 @@
           <t>Returned to the court roughly 14 months after the injury</t>
         </is>
       </c>
-      <c r="H108" s="2" t="inlineStr">
+      <c r="H108" s="2" t="n"/>
+      <c r="I108" s="2" t="inlineStr">
         <is>
           <t>Not applicable — NCAA athlete, no fixed salary</t>
         </is>
       </c>
-      <c r="I108" s="2" t="inlineStr">
+      <c r="J108" s="2" t="inlineStr">
         <is>
           <t>USC gets back its star guard after a full season lost to the injury</t>
         </is>
       </c>
-      <c r="J108" s="2" t="inlineStr">
+      <c r="K108" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="K108" s="2" t="inlineStr">
+      <c r="L108" s="2" t="inlineStr">
         <is>
           <t>Fox Sports - 2026-2027 College Basketball Offseason Buzz</t>
         </is>
       </c>
-      <c r="L108" s="2" t="inlineStr">
+      <c r="M108" s="2" t="inlineStr">
         <is>
           <t>https://www.foxsports.com/stories/college-basketball/college-basketball-2026-2027-buzz-news-injuries-transfers</t>
         </is>
@@ -7203,27 +7458,28 @@
           <t>Will miss the entire 2026-27 season</t>
         </is>
       </c>
-      <c r="H109" s="2" t="inlineStr">
+      <c r="H109" s="2" t="n"/>
+      <c r="I109" s="2" t="inlineStr">
         <is>
           <t>Not applicable — NCAA athlete, no fixed salary</t>
         </is>
       </c>
-      <c r="I109" s="2" t="inlineStr">
+      <c r="J109" s="2" t="inlineStr">
         <is>
           <t>Major setback for coach Rick Pitino and St. John's, who added the rising junior forward as a transfer-portal pickup this offseason; Freeman averaged 16.5 points and 7.2 rebounds last season at Syracuse</t>
         </is>
       </c>
-      <c r="J109" s="2" t="inlineStr">
+      <c r="K109" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="K109" s="2" t="inlineStr">
+      <c r="L109" s="2" t="inlineStr">
         <is>
           <t>The Washington Post - St. John's Donnie Freeman to miss next season following surgery on Achilles tendon</t>
         </is>
       </c>
-      <c r="L109" s="2" t="inlineStr">
+      <c r="M109" s="2" t="inlineStr">
         <is>
           <t>https://www.washingtonpost.com/sports/colleges/2026/07/01/st-johns-donnie-freeman-achilles-injury-pitino/81e54c60-75c4-11f1-b665-5f8be87f3787_story.html</t>
         </is>
@@ -7265,27 +7521,30 @@
           <t>Underwent UCL repair surgery July 1; 10-12 month recovery timeline</t>
         </is>
       </c>
-      <c r="H110" s="2" t="inlineStr">
+      <c r="H110" s="3" t="n">
+        <v>4068493</v>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
         <is>
           <t>$4,068,493 prorated sunk cost (annual salary ~$4.5M per Spotrac ÷ 365 × 330 days out; 10-12 month recovery timeline, midpoint of 11 months used)</t>
         </is>
       </c>
-      <c r="I110" s="2" t="inlineStr">
+      <c r="J110" s="2" t="inlineStr">
         <is>
           <t>Royals lose their staff ace for the remainder of 2026 and into 2027</t>
         </is>
       </c>
-      <c r="J110" s="2" t="inlineStr">
+      <c r="K110" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="K110" s="2" t="inlineStr">
+      <c r="L110" s="2" t="inlineStr">
         <is>
           <t>CBS Sports - Kansas City Royals Injury Report and Status 2026</t>
         </is>
       </c>
-      <c r="L110" s="2" t="inlineStr">
+      <c r="M110" s="2" t="inlineStr">
         <is>
           <t>https://www.cbssports.com/mlb/teams/KC/kansas-city-royals/injuries/</t>
         </is>
@@ -7327,27 +7586,30 @@
           <t>Re-evaluation in approximately 12 weeks</t>
         </is>
       </c>
-      <c r="H111" s="2" t="inlineStr">
+      <c r="H111" s="3" t="n">
+        <v>10632329</v>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
         <is>
           <t>$10,632,329 prorated sunk cost (annual salary ~$46.20M per Spotrac ÷ 365 × 84 days out)</t>
         </is>
       </c>
-      <c r="I111" s="2" t="inlineStr">
+      <c r="J111" s="2" t="inlineStr">
         <is>
           <t>Grizzlies lose their All-Star big man through the offseason and possibly into training camp</t>
         </is>
       </c>
-      <c r="J111" s="2" t="inlineStr">
+      <c r="K111" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="K111" s="2" t="inlineStr">
+      <c r="L111" s="2" t="inlineStr">
         <is>
           <t>NBA.com - Grizzlies' Jaren Jackson Jr. has surgery to repair turf toe injury</t>
         </is>
       </c>
-      <c r="L111" s="2" t="inlineStr">
+      <c r="M111" s="2" t="inlineStr">
         <is>
           <t>https://www.nba.com/news/memphis-grizzlies-jaren-jackson-jr-turf-toe-surgery</t>
         </is>
@@ -7389,27 +7651,30 @@
           <t>Potentially several months if ACL is confirmed</t>
         </is>
       </c>
-      <c r="H112" s="2" t="inlineStr">
+      <c r="H112" s="3" t="n">
+        <v>2749019</v>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
         <is>
           <t>$2,749,019 prorated sunk cost (annual salary ~$8.36M per Capology (GBP→USD @1.34) ÷ 365 × 120 days out)</t>
         </is>
       </c>
-      <c r="I112" s="2" t="inlineStr">
+      <c r="J112" s="2" t="inlineStr">
         <is>
           <t>Would be a significant blow to Manchester United's midfield depth heading into 2026-27</t>
         </is>
       </c>
-      <c r="J112" s="2" t="inlineStr">
+      <c r="K112" s="2" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="K112" s="2" t="inlineStr">
+      <c r="L112" s="2" t="inlineStr">
         <is>
           <t>Premier League club injury coverage</t>
         </is>
       </c>
-      <c r="L112" s="2" t="inlineStr">
+      <c r="M112" s="2" t="inlineStr">
         <is>
           <t>https://www.premierleague.com/en/latest-player-injuries</t>
         </is>
@@ -7451,27 +7716,30 @@
           <t>Out for the opening weeks of the 2026-27 season</t>
         </is>
       </c>
-      <c r="H113" s="2" t="inlineStr">
+      <c r="H113" s="3" t="n">
+        <v>881977</v>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
         <is>
           <t>$881,977 prorated sunk cost (annual salary ~$15.33M per Capology (GBP→USD @1.34) ÷ 365 × 21 days out)</t>
         </is>
       </c>
-      <c r="I113" s="2" t="inlineStr">
+      <c r="J113" s="2" t="inlineStr">
         <is>
           <t>Manchester City to start the new season without their midfield anchor</t>
         </is>
       </c>
-      <c r="J113" s="2" t="inlineStr">
+      <c r="K113" s="2" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="K113" s="2" t="inlineStr">
+      <c r="L113" s="2" t="inlineStr">
         <is>
           <t>Premier League club injury coverage</t>
         </is>
       </c>
-      <c r="L113" s="2" t="inlineStr">
+      <c r="M113" s="2" t="inlineStr">
         <is>
           <t>https://www.premierleague.com/en/latest-player-injuries</t>
         </is>
@@ -7513,27 +7781,30 @@
           <t>Ruled out for at least 4 weeks as of late June; All-Star Game (July 25) status still to be decided</t>
         </is>
       </c>
-      <c r="H114" s="2" t="inlineStr">
+      <c r="H114" s="3" t="n">
+        <v>76712</v>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
         <is>
           <t>$76,712 prorated sunk cost (annual salary ~$999,999 per Spotrac ÷ 365 × 28 days out)</t>
         </is>
       </c>
-      <c r="I114" s="2" t="inlineStr">
+      <c r="J114" s="2" t="inlineStr">
         <is>
           <t>Sparks lose a starting guard through their All-Star break stretch</t>
         </is>
       </c>
-      <c r="J114" s="2" t="inlineStr">
+      <c r="K114" s="2" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="K114" s="2" t="inlineStr">
+      <c r="L114" s="2" t="inlineStr">
         <is>
           <t>Bleacher Report - Angel Reese, Kelsey Plum Headline 2026 WNBA All-Star Game Reserves</t>
         </is>
       </c>
-      <c r="L114" s="2" t="inlineStr">
+      <c r="M114" s="2" t="inlineStr">
         <is>
           <t>https://bleacherreport.com/articles/25452286-angel-reese-kelsey-plum-headline-2026-wnba-all-star-game-reserves-full-roster-announced</t>
         </is>
@@ -7575,27 +7846,30 @@
           <t>Expected recovery of approximately 4-6 months, meaning the earliest return would be late October</t>
         </is>
       </c>
-      <c r="H115" s="2" t="inlineStr">
+      <c r="H115" s="3" t="n">
+        <v>3246575</v>
+      </c>
+      <c r="I115" s="2" t="inlineStr">
         <is>
           <t>$3,246,575 prorated sunk cost (annual salary ~$7.9M AAV per Spotrac ÷ 365 × 150 days out)</t>
         </is>
       </c>
-      <c r="I115" s="2" t="inlineStr">
+      <c r="J115" s="2" t="inlineStr">
         <is>
           <t>Hurricanes will be without a top-six forward for the start of the 2026-27 season</t>
         </is>
       </c>
-      <c r="J115" s="2" t="inlineStr">
+      <c r="K115" s="2" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="K115" s="2" t="inlineStr">
+      <c r="L115" s="2" t="inlineStr">
         <is>
           <t>NHL.com - Jarvis expected to miss start of next season for Hurricanes after shoulder surgery</t>
         </is>
       </c>
-      <c r="L115" s="2" t="inlineStr">
+      <c r="M115" s="2" t="inlineStr">
         <is>
           <t>https://www.nhl.com/news/seth-jarvis-to-miss-beginning-of-2026-2027-season-for-hurricanes-after-shoulder-surgery</t>
         </is>
@@ -7637,27 +7911,30 @@
           <t>Season-ending; recovery expected to extend into 2026-27 preseason</t>
         </is>
       </c>
-      <c r="H116" s="2" t="inlineStr">
+      <c r="H116" s="3" t="n">
+        <v>1416976</v>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
         <is>
           <t>$1,416,976 prorated sunk cost (annual salary ~$5.62M per Spotrac ÷ 365 × 92 days out)</t>
         </is>
       </c>
-      <c r="I116" s="2" t="inlineStr">
+      <c r="J116" s="2" t="inlineStr">
         <is>
           <t>Clippers lose a veteran guard for the balance of the season and into next year's planning</t>
         </is>
       </c>
-      <c r="J116" s="2" t="inlineStr">
+      <c r="K116" s="2" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="K116" s="2" t="inlineStr">
+      <c r="L116" s="2" t="inlineStr">
         <is>
           <t>NBA.com - Clippers' Bradley Beal (hip) to undergo season-ending surgery</t>
         </is>
       </c>
-      <c r="L116" s="2" t="inlineStr">
+      <c r="M116" s="2" t="inlineStr">
         <is>
           <t>https://www.nba.com/news/clippers-bradley-beal-out-season-hip-fracture</t>
         </is>
@@ -7699,27 +7976,28 @@
           <t>Withdrew mid-tournament from Eastbourne</t>
         </is>
       </c>
-      <c r="H117" s="2" t="inlineStr">
+      <c r="H117" s="2" t="n"/>
+      <c r="I117" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $499,000 total tournament prize purse for the 2026 Lexus Eastbourne Open (WTA 250) (per LTA/WTA reporting).</t>
         </is>
       </c>
-      <c r="I117" s="2" t="inlineStr">
+      <c r="J117" s="2" t="inlineStr">
         <is>
           <t>Opponent Zeynep Sonmez advances by walkover</t>
         </is>
       </c>
-      <c r="J117" s="2" t="inlineStr">
+      <c r="K117" s="2" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="K117" s="2" t="inlineStr">
+      <c r="L117" s="2" t="inlineStr">
         <is>
           <t>RotoWire - Fantasy Tennis Injury News</t>
         </is>
       </c>
-      <c r="L117" s="2" t="inlineStr">
+      <c r="M117" s="2" t="inlineStr">
         <is>
           <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
         </is>
@@ -7761,27 +8039,30 @@
           <t>Will miss the 2026 World Cup; club return timeline unconfirmed</t>
         </is>
       </c>
-      <c r="H118" s="2" t="inlineStr">
+      <c r="H118" s="3" t="n">
+        <v>185397</v>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
         <is>
           <t>$185,397 prorated sunk cost (annual salary ~$13.53M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
         </is>
       </c>
-      <c r="I118" s="2" t="inlineStr">
+      <c r="J118" s="2" t="inlineStr">
         <is>
           <t>United lose a starting center-back for an extended stretch</t>
         </is>
       </c>
-      <c r="J118" s="2" t="inlineStr">
+      <c r="K118" s="2" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="K118" s="2" t="inlineStr">
+      <c r="L118" s="2" t="inlineStr">
         <is>
           <t>Premier League club injury coverage</t>
         </is>
       </c>
-      <c r="L118" s="2" t="inlineStr">
+      <c r="M118" s="2" t="inlineStr">
         <is>
           <t>https://www.premierleague.com/en/latest-player-injuries</t>
         </is>
@@ -7823,27 +8104,28 @@
           <t>Withdrew before her Bad Homburg quarterfinal</t>
         </is>
       </c>
-      <c r="H119" s="2" t="inlineStr">
+      <c r="H119" s="2" t="n"/>
+      <c r="I119" s="2" t="inlineStr">
         <is>
           <t>Not disclosed in available reporting — no specific prize money forfeiture figure found Potential prize money at stake (ceiling, not a claim of what the athlete would have won): $1.2M total tournament prize purse ($1,206,446 / €1,049,083) for the 2026 Bad Homburg Open (per Perfect Tennis/WTA).</t>
         </is>
       </c>
-      <c r="I119" s="2" t="inlineStr">
+      <c r="J119" s="2" t="inlineStr">
         <is>
           <t>Opponent Xinyu Wang advances by walkover</t>
         </is>
       </c>
-      <c r="J119" s="2" t="inlineStr">
+      <c r="K119" s="2" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="K119" s="2" t="inlineStr">
+      <c r="L119" s="2" t="inlineStr">
         <is>
           <t>RotoWire - Fantasy Tennis Injury News</t>
         </is>
       </c>
-      <c r="L119" s="2" t="inlineStr">
+      <c r="M119" s="2" t="inlineStr">
         <is>
           <t>https://www.rotowire.com/tennis/news.php?view=injuries</t>
         </is>
@@ -7885,27 +8167,30 @@
           <t>Expected to recover in time for the 2026 World Cup</t>
         </is>
       </c>
-      <c r="H120" s="2" t="inlineStr">
+      <c r="H120" s="3" t="n">
+        <v>52499</v>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
         <is>
           <t>$52,499 prorated sunk cost (annual salary ~$3.83M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
         </is>
       </c>
-      <c r="I120" s="2" t="inlineStr">
+      <c r="J120" s="2" t="inlineStr">
         <is>
           <t>Crystal Palace lose a starting center-back for a multi-week stretch</t>
         </is>
       </c>
-      <c r="J120" s="2" t="inlineStr">
+      <c r="K120" s="2" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="K120" s="2" t="inlineStr">
+      <c r="L120" s="2" t="inlineStr">
         <is>
           <t>Premier League club injury coverage</t>
         </is>
       </c>
-      <c r="L120" s="2" t="inlineStr">
+      <c r="M120" s="2" t="inlineStr">
         <is>
           <t>https://www.premierleague.com/en/latest-player-injuries</t>
         </is>
@@ -7947,27 +8232,28 @@
           <t>Placed on the 45-day short-term injury list</t>
         </is>
       </c>
-      <c r="H121" s="2" t="inlineStr">
+      <c r="H121" s="2" t="n"/>
+      <c r="I121" s="2" t="inlineStr">
         <is>
           <t>Not disclosed — NWSL player salaries are confidential under the league/NWSLPA collective bargaining agreement and not publicly released</t>
         </is>
       </c>
-      <c r="I121" s="2" t="inlineStr">
+      <c r="J121" s="2" t="inlineStr">
         <is>
           <t>Boston Legacy FC without a rostered defender for at least 45 days</t>
         </is>
       </c>
-      <c r="J121" s="2" t="inlineStr">
+      <c r="K121" s="2" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="K121" s="2" t="inlineStr">
+      <c r="L121" s="2" t="inlineStr">
         <is>
           <t>Washington Spirit / NWSL transactions coverage</t>
         </is>
       </c>
-      <c r="L121" s="2" t="inlineStr">
+      <c r="M121" s="2" t="inlineStr">
         <is>
           <t>https://www.spotrac.com/nwsl/injured/_/year/2026</t>
         </is>
@@ -7975,126 +8261,126 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L77" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L78" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L80" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L81" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L82" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L83" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L84" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L85" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L86" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L87" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L88" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L89" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L90" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L91" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L92" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L93" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L94" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L95" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L96" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L97" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L98" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L99" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L100" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L101" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L102" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L103" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L104" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L105" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L106" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L107" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L108" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L109" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L110" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L111" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L112" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L113" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L114" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L115" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L116" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L117" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L118" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L119" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L120" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId120"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Strip redundant leading dollar amount from financial_impact_calculation text
</commit_message>
<xml_diff>
--- a/injury_report.xlsx
+++ b/injury_report.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>$706 prorated sunk cost (annual salary ~$85,873 per Spotrac ÷ 365 × 3 days out) [questionable status, day-to-day default]</t>
+          <t>prorated sunk cost (annual salary ~$85,873 per Spotrac ÷ 365 × 3 days out) [questionable status, day-to-day default]</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>$6,532 prorated sunk cost (annual salary ~$794,800 per Spotrac ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual salary ~$794,800 per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>$5,579 prorated sunk cost (annual salary ~$678,882 (two-way) per Hoops Rumors ÷ 365 × 3 days out) [assumption: no timeline given, day-to-day default]</t>
+          <t>prorated sunk cost (annual salary ~$678,882 (two-way) per Hoops Rumors ÷ 365 × 3 days out) [assumption: no timeline given, day-to-day default]</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>$2,281 prorated sunk cost (annual salary ~$277,500 per Spotrac ÷ 365 × 3 days out) [assumption: single-game absence, no timeline, day-to-day default]</t>
+          <t>prorated sunk cost (annual salary ~$277,500 per Spotrac ÷ 365 × 3 days out) [assumption: single-game absence, no timeline, day-to-day default]</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>$13,020 prorated sunk cost (annual salary ~$678,882 (two-way) per Hoops Rumors ÷ 365 × 7 days out) [assumption: ruled out for remainder of NBA Summer League (~July 13-20); true post-surgery recovery likely longer but not specified]</t>
+          <t>prorated sunk cost (annual salary ~$678,882 (two-way) per Hoops Rumors ÷ 365 × 7 days out) [assumption: ruled out for remainder of NBA Summer League (~July 13-20); true post-surgery recovery likely longer but not specified]</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>$78,272 prorated sunk cost (annual salary ~$9.52M per Spotrac ÷ 365 × 3 days out) [assumption: held out as precaution, no formal diagnosis/timeline, day-to-day default]</t>
+          <t>prorated sunk cost (annual salary ~$9.52M per Spotrac ÷ 365 × 3 days out) [assumption: held out as precaution, no formal diagnosis/timeline, day-to-day default]</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>$1,109,589 prorated sunk cost (annual salary ~$27M per Spotrac ÷ 365 × 15 days out) [estimate: ~15 days from July 13 to a "late July" return target]</t>
+          <t>prorated sunk cost (annual salary ~$27M per Spotrac ÷ 365 × 15 days out) [estimate: ~15 days from July 13 to a "late July" return target]</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>$41,096 prorated sunk cost (annual salary ~$3.0M per Spotrac ÷ 365 × 5 days out) [undetermined additional recovery time following the rehab setback]</t>
+          <t>prorated sunk cost (annual salary ~$3.0M per Spotrac ÷ 365 × 5 days out) [undetermined additional recovery time following the rehab setback]</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>$18,942 prorated sunk cost (annual salary ~$493,851 per Spotrac ÷ 365 × 14 days out) [expected out at least two weeks]</t>
+          <t>prorated sunk cost (annual salary ~$493,851 per Spotrac ÷ 365 × 14 days out) [expected out at least two weeks]</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>$246,575 prorated sunk cost (annual salary ~$9M per Spotrac ÷ 365 × 10 days out)</t>
+          <t>prorated sunk cost (annual salary ~$9M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>$32,305 prorated sunk cost (annual salary ~$786,100 per Spotrac ÷ 365 × 15 days out)</t>
+          <t>prorated sunk cost (annual salary ~$786,100 per Spotrac ÷ 365 × 15 days out)</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>$1,553 prorated sunk cost (annual salary ~$113,400 per Capology ÷ 365 × 5 days out; no specific recovery timeline disclosed, conservative 5-day default used)</t>
+          <t>prorated sunk cost (annual salary ~$113,400 per Capology ÷ 365 × 5 days out; no specific recovery timeline disclosed, conservative 5-day default used)</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>$30,822 prorated sunk cost (annual salary ~$2.25M per Capology ÷ 365 × 5 days out; no specific recovery timeline disclosed, conservative 5-day default used)</t>
+          <t>prorated sunk cost (annual salary ~$2.25M per Capology ÷ 365 × 5 days out; no specific recovery timeline disclosed, conservative 5-day default used)</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>$64,658 prorated sunk cost (annual salary cap hit ~$200,000 per Capology ÷ 365 × 118 days out; days out estimated from date reported to 2026 MLS regular season end ~Nov 7)</t>
+          <t>prorated sunk cost (annual salary cap hit ~$200,000 per Capology ÷ 365 × 118 days out; days out estimated from date reported to 2026 MLS regular season end ~Nov 7)</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>$6,520 prorated sunk cost (annual salary ~$793,300 per Spotrac ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual salary ~$793,300 per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>$166,685 prorated sunk cost (annual salary ~$780,000 per Spotrac ÷ 365 × 78 days out; possible season-ending surgery, days out estimated from date reported to MLB regular season end ~Sept 28)</t>
+          <t>prorated sunk cost (annual salary ~$780,000 per Spotrac ÷ 365 × 78 days out; possible season-ending surgery, days out estimated from date reported to MLB regular season end ~Sept 28)</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>$65,178 prorated sunk cost (annual salary ~$792,800 per Spotrac ÷ 365 × 30 days out) [estimate: 'at least a month' minimum]</t>
+          <t>prorated sunk cost (annual salary ~$792,800 per Spotrac ÷ 365 × 30 days out) [estimate: 'at least a month' minimum]</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>$905,205 prorated sunk cost (annual salary ~$22.025M per Spotrac ÷ 365 × 15 days out)</t>
+          <t>prorated sunk cost (annual salary ~$22.025M per Spotrac ÷ 365 × 15 days out)</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>$11,164 prorated sunk cost (annual salary ~$815K per Spotrac ÷ 365 × 5 days out) [assumption: concussion protocol with no return timeline, used 5-day undetermined default]</t>
+          <t>prorated sunk cost (annual salary ~$815K per Spotrac ÷ 365 × 5 days out) [assumption: concussion protocol with no return timeline, used 5-day undetermined default]</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>$2,882 prorated sunk cost (annual salary ~$350,692 per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day questionable status]</t>
+          <t>prorated sunk cost (annual salary ~$350,692 per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day questionable status]</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>$153,425 prorated sunk cost (annual salary ~$1M per Spotrac ÷ 365 × 56 days out) [assumption: out since ~start of 2026 WNBA season (~May 16) through date reported (July 11), ~56 days]</t>
+          <t>prorated sunk cost (annual salary ~$1M per Spotrac ÷ 365 × 56 days out) [assumption: out since ~start of 2026 WNBA season (~May 16) through date reported (July 11), ~56 days]</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>$4,021 prorated sunk cost (annual salary ~$293,510 per Spotrac ÷ 365 × 5 days out) [assumption: no return timeline, used 5-day undetermined default]</t>
+          <t>prorated sunk cost (annual salary ~$293,510 per Spotrac ÷ 365 × 5 days out) [assumption: no return timeline, used 5-day undetermined default]</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>$21,507 prorated sunk cost (annual salary ~$785K per Spotrac ÷ 365 × 10 days out) [10-day injured list stint]</t>
+          <t>prorated sunk cost (annual salary ~$785K per Spotrac ÷ 365 × 10 days out) [10-day injured list stint]</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>$194,178 prorated sunk cost (annual salary ~$4.725M per Spotrac ÷ 365 × 15 days out) [15-day injured list stint]</t>
+          <t>prorated sunk cost (annual salary ~$4.725M per Spotrac ÷ 365 × 15 days out) [15-day injured list stint]</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3217,7 +3217,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>$345,205 prorated sunk cost (annual salary ~$42M (contract AAV) per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day, not placed on IL, used 3-day estimate]</t>
+          <t>prorated sunk cost (annual salary ~$42M (contract AAV) per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day, not placed on IL, used 3-day estimate]</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>$47,945 prorated sunk cost (annual salary ~$1.25M per Spotrac ÷ 365 × 14 days out) [assumption: 'reevaluated in the next couple of weeks' = 2 weeks]</t>
+          <t>prorated sunk cost (annual salary ~$1.25M per Spotrac ÷ 365 × 14 days out) [assumption: 'reevaluated in the next couple of weeks' = 2 weeks]</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>$172,603 prorated sunk cost (annual salary ~$1M base salary per Spotrac ÷ 365 × 63 days out) [8-10 week recovery timeline, used midpoint of 9 weeks = 63 days; excludes one-time signing bonus from prorated base]</t>
+          <t>prorated sunk cost (annual salary ~$1M base salary per Spotrac ÷ 365 × 63 days out) [8-10 week recovery timeline, used midpoint of 9 weeks = 63 days; excludes one-time signing bonus from prorated base]</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>$65,205 prorated sunk cost (annual salary ~$850,000 per Spotrac ÷ 365 × 28 days out)</t>
+          <t>prorated sunk cost (annual salary ~$850,000 per Spotrac ÷ 365 × 28 days out)</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>$356,164 prorated sunk cost (annual salary ~$13M per Spotrac ÷ 365 × 10 days out)</t>
+          <t>prorated sunk cost (annual salary ~$13M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>$17,961 prorated sunk cost (annual salary ~$2.19M per Spotrac [2026-27 base salary on new 2-year deal] ÷ 365 × 3 days out) [assumption: single-game absence, no diagnosis timeline given, day-to-day default]</t>
+          <t>prorated sunk cost (annual salary ~$2.19M per Spotrac [2026-27 base salary on new 2-year deal] ÷ 365 × 3 days out) [assumption: single-game absence, no diagnosis timeline given, day-to-day default]</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>$277,397 prorated sunk cost (annual salary ~€31.25M / ~$33.75M per Capology [EUR→USD @1.08] ÷ 365 × 3 days out) [day-to-day default; reporting indicates no games were actually missed]</t>
+          <t>prorated sunk cost (annual salary ~€31.25M / ~$33.75M per Capology [EUR→USD @1.08] ÷ 365 × 3 days out) [day-to-day default; reporting indicates no games were actually missed]</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>$86,747 prorated sunk cost (annual salary ~$6.33M per Spotrac ÷ 365 × 5 days out) [assumption: no firm return timeline reported, used 5-day undetermined default]</t>
+          <t>prorated sunk cost (annual salary ~$6.33M per Spotrac ÷ 365 × 5 days out) [assumption: no firm return timeline reported, used 5-day undetermined default]</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>$575,342 prorated sunk cost (annual salary ~$70M (contract AAV) per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day knee issue, skipping one start and the All-Star Game, no IL move reported]</t>
+          <t>prorated sunk cost (annual salary ~$70M (contract AAV) per Spotrac ÷ 365 × 3 days out) [assumption: day-to-day knee issue, skipping one start and the All-Star Game, no IL move reported]</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>$106,925 prorated sunk cost (annual salary ~$3.9M per Spotrac ÷ 365 × 10 days out) [assumption: ruled out for entire 2026 NBA Summer League, ~July 10-20]</t>
+          <t>prorated sunk cost (annual salary ~$3.9M per Spotrac ÷ 365 × 10 days out) [assumption: ruled out for entire 2026 NBA Summer League, ~July 10-20]</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
@@ -3930,7 +3930,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>$684,932 prorated sunk cost (annual salary ~$25M per Spotrac ÷ 365 × 10 days out)</t>
+          <t>prorated sunk cost (annual salary ~$25M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>$10,685 prorated sunk cost (annual salary ~$780,000 per Spotrac ÷ 365 × 5 days out; recovery timeline undisclosed, conservative 5-day default used)</t>
+          <t>prorated sunk cost (annual salary ~$780,000 per Spotrac ÷ 365 × 5 days out; recovery timeline undisclosed, conservative 5-day default used)</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -4375,7 +4375,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>$547,945 prorated sunk cost (annual salary ~$40M per Spotrac ÷ 365 × 5 days out)</t>
+          <t>prorated sunk cost (annual salary ~$40M per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>$93,637 prorated sunk cost (annual salary ~$813,750 per Spotrac ÷ 365 × 42 days out)</t>
+          <t>prorated sunk cost (annual salary ~$813,750 per Spotrac ÷ 365 × 42 days out)</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>$10,479 prorated sunk cost (annual salary ~$765,000 per Spotrac ÷ 365 × 5 days out)</t>
+          <t>prorated sunk cost (annual salary ~$765,000 per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>$616,438 prorated sunk cost (annual salary ~$3.75M AAV per Spotrac ÷ 365 × 60 days out) [assumption: 60 days used as the near-term horizon to the September training-camp re-evaluation date; reporting indicates his full 2026-27 season could be at risk if complications persist, which would raise this figure substantially]</t>
+          <t>prorated sunk cost (annual salary ~$3.75M AAV per Spotrac ÷ 365 × 60 days out) [assumption: 60 days used as the near-term horizon to the September training-camp re-evaluation date; reporting indicates his full 2026-27 season could be at risk if complications persist, which would raise this figure substantially]</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -4950,7 +4950,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>$312,329 prorated sunk cost (2025-26 entry-level contract cap hit ~$950,000 per Spotrac/Puckpedia ÷ 365 × 120 days out [~4-month recovery])</t>
+          <t>prorated sunk cost (2025-26 entry-level contract cap hit ~$950,000 per Spotrac/Puckpedia ÷ 365 × 120 days out [~4-month recovery])</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -5015,7 +5015,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>$8,219 prorated sunk cost (annual salary ~$1M per Spotrac ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual salary ~$1M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>$85,479 prorated sunk cost (annual salary ~£10.4M (~$10.4M gross fixed wages) per Capology ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual salary ~£10.4M (~$10.4M gross fixed wages) per Capology ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -5145,7 +5145,7 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>$102,740 prorated sunk cost (annual salary ~€12.5M gross (~$13.5M) per Capology ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual salary ~€12.5M gross (~$13.5M) per Capology ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>$32,055 prorated sunk cost (annual salary ~$780,000 MLB minimum per Spotrac ÷ 365 × 15 days out)</t>
+          <t>prorated sunk cost (annual salary ~$780,000 MLB minimum per Spotrac ÷ 365 × 15 days out)</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -5338,7 +5338,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>$21,370 prorated sunk cost (annual salary ~$780,000 MLB minimum per Spotrac ÷ 365 × 10 days out)</t>
+          <t>prorated sunk cost (annual salary ~$780,000 MLB minimum per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>$6,203,757 prorated sunk cost (annual salary ~$37.74M per Spotrac ÷ 365 × 60 days out)</t>
+          <t>prorated sunk cost (annual salary ~$37.74M per Spotrac ÷ 365 × 60 days out)</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>$6,414,378 prorated sunk cost (annual salary ~$9.76M per Capology (GBP→USD @1.34) ÷ 365 × 240 days out)</t>
+          <t>prorated sunk cost (annual salary ~$9.76M per Capology (GBP→USD @1.34) ÷ 365 × 240 days out)</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -5659,7 +5659,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>$397,260 prorated sunk cost (annual salary ~$29.00M per Spotrac ÷ 365 × 5 days out)</t>
+          <t>prorated sunk cost (annual salary ~$29.00M per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>$7,562 prorated sunk cost (annual salary ~$920,000 per Spotrac ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual salary ~$920,000 per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -5852,7 +5852,7 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>£40,000 (~$53,600) forfeited guaranteed prize money — 50% of the £80,000 first-round Wimbledon payout, per WTA withdrawal rules (per GB News / Tennis365)</t>
+          <t>forfeited guaranteed prize money — 50% of the £80,000 first-round Wimbledon payout, per WTA withdrawal rules (per GB News / Tennis365)</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -5980,7 +5980,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>$72,304 prorated sunk cost (annual salary ~$5.28M per Capology (EUR→USD @1.14) ÷ 365 × 5 days out)</t>
+          <t>prorated sunk cost (annual salary ~$5.28M per Capology (EUR→USD @1.14) ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -6045,7 +6045,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>$48,723 prorated sunk cost (annual base salary ~€5.2M / ~$5.93M per Capology (EUR→USD @1.14) ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual base salary ~€5.2M / ~$5.93M per Capology (EUR→USD @1.14) ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>$11,507 prorated sunk cost (annual salary ~$1.40M per Spotrac ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual salary ~$1.40M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>$4,347 prorated sunk cost (annual salary ~$528,846 per Spotrac ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual salary ~$528,846 per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>$11,507 prorated sunk cost (annual salary ~$1.4M per Spotrac ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual salary ~$1.4M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -6368,7 +6368,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>$8,219 prorated sunk cost (annual salary ~$300,000 per Spotrac ÷ 365 × 10 days out)</t>
+          <t>prorated sunk cost (annual salary ~$300,000 per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>$123,288 prorated sunk cost (annual salary ~$15.00M per Spotrac ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual salary ~$15.00M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -6498,7 +6498,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>$83,836 prorated sunk cost (annual salary ~$10.20M per Spotrac ÷ 365 × 3 days out)</t>
+          <t>prorated sunk cost (annual salary ~$10.20M per Spotrac ÷ 365 × 3 days out)</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>$95,890 prorated sunk cost (annual salary ~$7.00M per Spotrac ÷ 365 × 5 days out)</t>
+          <t>prorated sunk cost (annual salary ~$7.00M per Spotrac ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -6628,7 +6628,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>$905,137 prorated sunk cost (annual salary ~$22.02M per Spotrac ÷ 365 × 15 days out)</t>
+          <t>prorated sunk cost (annual salary ~$22.02M per Spotrac ÷ 365 × 15 days out)</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>$374,932 prorated sunk cost (annual salary ~$1.61M per Spotrac ÷ 365 × 85 days out)</t>
+          <t>prorated sunk cost (annual salary ~$1.61M per Spotrac ÷ 365 × 85 days out)</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -6758,7 +6758,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>$3,838 prorated sunk cost (annual salary ~$466,913 per Spotrac/On3 ÷ 365 × 3 days out) [assumption: day-to-day, signs point to quick recovery]</t>
+          <t>prorated sunk cost (annual salary ~$466,913 per Spotrac/On3 ÷ 365 × 3 days out) [assumption: day-to-day, signs point to quick recovery]</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>$162,268 prorated sunk cost (annual salary ~$11.85M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
+          <t>prorated sunk cost (annual salary ~$11.85M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>$9,424,658 prorated sunk cost (annual salary ~$40.00M per Spotrac ÷ 365 × 86 days out)</t>
+          <t>prorated sunk cost (annual salary ~$40.00M per Spotrac ÷ 365 × 86 days out)</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -7205,7 +7205,7 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>$6,164,384 prorated sunk cost (annual salary ~$25.00M per Spotrac ÷ 365 × 90 days out)</t>
+          <t>prorated sunk cost (annual salary ~$25.00M per Spotrac ÷ 365 × 90 days out)</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>$849,315 prorated sunk cost (annual salary ~$31.00M per Spotrac ÷ 365 × 10 days out)</t>
+          <t>prorated sunk cost (annual salary ~$31.00M per Spotrac ÷ 365 × 10 days out)</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -7335,7 +7335,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>$1,463,014 prorated sunk cost (annual salary ~$6.00M per Spotrac ÷ 365 × 89 days out)</t>
+          <t>prorated sunk cost (annual salary ~$6.00M per Spotrac ÷ 365 × 89 days out)</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -7526,7 +7526,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>$4,068,493 prorated sunk cost (annual salary ~$4.5M per Spotrac ÷ 365 × 330 days out; 10-12 month recovery timeline, midpoint of 11 months used)</t>
+          <t>prorated sunk cost (annual salary ~$4.5M per Spotrac ÷ 365 × 330 days out; 10-12 month recovery timeline, midpoint of 11 months used)</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -7591,7 +7591,7 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>$10,632,329 prorated sunk cost (annual salary ~$46.20M per Spotrac ÷ 365 × 84 days out)</t>
+          <t>prorated sunk cost (annual salary ~$46.20M per Spotrac ÷ 365 × 84 days out)</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr">
@@ -7656,7 +7656,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>$2,749,019 prorated sunk cost (annual salary ~$8.36M per Capology (GBP→USD @1.34) ÷ 365 × 120 days out)</t>
+          <t>prorated sunk cost (annual salary ~$8.36M per Capology (GBP→USD @1.34) ÷ 365 × 120 days out)</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -7721,7 +7721,7 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>$881,977 prorated sunk cost (annual salary ~$15.33M per Capology (GBP→USD @1.34) ÷ 365 × 21 days out)</t>
+          <t>prorated sunk cost (annual salary ~$15.33M per Capology (GBP→USD @1.34) ÷ 365 × 21 days out)</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -7786,7 +7786,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>$76,712 prorated sunk cost (annual salary ~$999,999 per Spotrac ÷ 365 × 28 days out)</t>
+          <t>prorated sunk cost (annual salary ~$999,999 per Spotrac ÷ 365 × 28 days out)</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>$3,246,575 prorated sunk cost (annual salary ~$7.9M AAV per Spotrac ÷ 365 × 150 days out)</t>
+          <t>prorated sunk cost (annual salary ~$7.9M AAV per Spotrac ÷ 365 × 150 days out)</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -7916,7 +7916,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>$1,416,976 prorated sunk cost (annual salary ~$5.62M per Spotrac ÷ 365 × 92 days out)</t>
+          <t>prorated sunk cost (annual salary ~$5.62M per Spotrac ÷ 365 × 92 days out)</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -8044,7 +8044,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>$185,397 prorated sunk cost (annual salary ~$13.53M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
+          <t>prorated sunk cost (annual salary ~$13.53M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -8172,7 +8172,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>$52,499 prorated sunk cost (annual salary ~$3.83M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
+          <t>prorated sunk cost (annual salary ~$3.83M per Capology (GBP→USD @1.34) ÷ 365 × 5 days out)</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">

</xml_diff>